<commit_message>
Otomatik veri güncelleme (17.07.2026 09:38 UTC)
</commit_message>
<xml_diff>
--- a/butce/butce.xlsx
+++ b/butce/butce.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,69 +421,69 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tarih</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>yil</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ay</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>gelir</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>vergi</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>dolaysiz_vergi</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>dolayli_vergi</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>gider</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>faiz_haric_gider</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>faiz_gideri</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>faiz_disi_denge</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>denge</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>38718</v>
       </c>
       <c r="B2" t="n">
@@ -533,7 +521,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>38749</v>
       </c>
       <c r="B3" t="n">
@@ -571,7 +559,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>38777</v>
       </c>
       <c r="B4" t="n">
@@ -609,7 +597,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>38808</v>
       </c>
       <c r="B5" t="n">
@@ -647,7 +635,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>38838</v>
       </c>
       <c r="B6" t="n">
@@ -685,7 +673,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>38869</v>
       </c>
       <c r="B7" t="n">
@@ -723,7 +711,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>38899</v>
       </c>
       <c r="B8" t="n">
@@ -761,7 +749,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>38930</v>
       </c>
       <c r="B9" t="n">
@@ -799,7 +787,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>38961</v>
       </c>
       <c r="B10" t="n">
@@ -837,7 +825,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>38991</v>
       </c>
       <c r="B11" t="n">
@@ -875,7 +863,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>39022</v>
       </c>
       <c r="B12" t="n">
@@ -913,7 +901,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>39052</v>
       </c>
       <c r="B13" t="n">
@@ -951,7 +939,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>39083</v>
       </c>
       <c r="B14" t="n">
@@ -989,7 +977,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>39114</v>
       </c>
       <c r="B15" t="n">
@@ -1027,7 +1015,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>39142</v>
       </c>
       <c r="B16" t="n">
@@ -1065,7 +1053,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>39173</v>
       </c>
       <c r="B17" t="n">
@@ -1103,7 +1091,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>39203</v>
       </c>
       <c r="B18" t="n">
@@ -1141,7 +1129,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>39234</v>
       </c>
       <c r="B19" t="n">
@@ -1179,7 +1167,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>39264</v>
       </c>
       <c r="B20" t="n">
@@ -1217,7 +1205,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>39295</v>
       </c>
       <c r="B21" t="n">
@@ -1255,7 +1243,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>39326</v>
       </c>
       <c r="B22" t="n">
@@ -1293,7 +1281,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>39356</v>
       </c>
       <c r="B23" t="n">
@@ -1331,7 +1319,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>39387</v>
       </c>
       <c r="B24" t="n">
@@ -1369,7 +1357,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>39417</v>
       </c>
       <c r="B25" t="n">
@@ -1407,7 +1395,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>39448</v>
       </c>
       <c r="B26" t="n">
@@ -1445,7 +1433,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="1" t="n">
         <v>39479</v>
       </c>
       <c r="B27" t="n">
@@ -1483,7 +1471,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>39508</v>
       </c>
       <c r="B28" t="n">
@@ -1521,7 +1509,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>39539</v>
       </c>
       <c r="B29" t="n">
@@ -1559,7 +1547,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>39569</v>
       </c>
       <c r="B30" t="n">
@@ -1597,7 +1585,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>39600</v>
       </c>
       <c r="B31" t="n">
@@ -1635,7 +1623,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>39630</v>
       </c>
       <c r="B32" t="n">
@@ -1673,7 +1661,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>39661</v>
       </c>
       <c r="B33" t="n">
@@ -1711,7 +1699,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>39692</v>
       </c>
       <c r="B34" t="n">
@@ -1749,7 +1737,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>39722</v>
       </c>
       <c r="B35" t="n">
@@ -1787,7 +1775,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>39753</v>
       </c>
       <c r="B36" t="n">
@@ -1825,7 +1813,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>39783</v>
       </c>
       <c r="B37" t="n">
@@ -1863,7 +1851,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>39814</v>
       </c>
       <c r="B38" t="n">
@@ -1901,7 +1889,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>39845</v>
       </c>
       <c r="B39" t="n">
@@ -1939,7 +1927,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>39873</v>
       </c>
       <c r="B40" t="n">
@@ -1977,7 +1965,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>39904</v>
       </c>
       <c r="B41" t="n">
@@ -2015,7 +2003,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>39934</v>
       </c>
       <c r="B42" t="n">
@@ -2053,7 +2041,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>39965</v>
       </c>
       <c r="B43" t="n">
@@ -2091,7 +2079,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>39995</v>
       </c>
       <c r="B44" t="n">
@@ -2129,7 +2117,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>40026</v>
       </c>
       <c r="B45" t="n">
@@ -2167,7 +2155,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>40057</v>
       </c>
       <c r="B46" t="n">
@@ -2205,7 +2193,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>40087</v>
       </c>
       <c r="B47" t="n">
@@ -2243,7 +2231,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>40118</v>
       </c>
       <c r="B48" t="n">
@@ -2281,7 +2269,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>40148</v>
       </c>
       <c r="B49" t="n">
@@ -2319,7 +2307,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>40179</v>
       </c>
       <c r="B50" t="n">
@@ -2357,7 +2345,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>40210</v>
       </c>
       <c r="B51" t="n">
@@ -2395,7 +2383,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>40238</v>
       </c>
       <c r="B52" t="n">
@@ -2433,7 +2421,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>40269</v>
       </c>
       <c r="B53" t="n">
@@ -2471,7 +2459,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>40299</v>
       </c>
       <c r="B54" t="n">
@@ -2509,7 +2497,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>40330</v>
       </c>
       <c r="B55" t="n">
@@ -2547,7 +2535,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>40360</v>
       </c>
       <c r="B56" t="n">
@@ -2585,7 +2573,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>40391</v>
       </c>
       <c r="B57" t="n">
@@ -2623,7 +2611,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>40422</v>
       </c>
       <c r="B58" t="n">
@@ -2661,7 +2649,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>40452</v>
       </c>
       <c r="B59" t="n">
@@ -2699,7 +2687,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>40483</v>
       </c>
       <c r="B60" t="n">
@@ -2737,7 +2725,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>40513</v>
       </c>
       <c r="B61" t="n">
@@ -2775,7 +2763,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>40544</v>
       </c>
       <c r="B62" t="n">
@@ -2813,7 +2801,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="1" t="n">
         <v>40575</v>
       </c>
       <c r="B63" t="n">
@@ -2851,7 +2839,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="1" t="n">
         <v>40603</v>
       </c>
       <c r="B64" t="n">
@@ -2889,7 +2877,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="1" t="n">
         <v>40634</v>
       </c>
       <c r="B65" t="n">
@@ -2927,7 +2915,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="1" t="n">
         <v>40664</v>
       </c>
       <c r="B66" t="n">
@@ -2965,7 +2953,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="1" t="n">
         <v>40695</v>
       </c>
       <c r="B67" t="n">
@@ -3003,7 +2991,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="1" t="n">
         <v>40725</v>
       </c>
       <c r="B68" t="n">
@@ -3041,7 +3029,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="1" t="n">
         <v>40756</v>
       </c>
       <c r="B69" t="n">
@@ -3079,7 +3067,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="1" t="n">
         <v>40787</v>
       </c>
       <c r="B70" t="n">
@@ -3117,7 +3105,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="1" t="n">
         <v>40817</v>
       </c>
       <c r="B71" t="n">
@@ -3155,7 +3143,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="1" t="n">
         <v>40848</v>
       </c>
       <c r="B72" t="n">
@@ -3193,7 +3181,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="1" t="n">
         <v>40878</v>
       </c>
       <c r="B73" t="n">
@@ -3231,7 +3219,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="1" t="n">
         <v>40909</v>
       </c>
       <c r="B74" t="n">
@@ -3269,7 +3257,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="1" t="n">
         <v>40940</v>
       </c>
       <c r="B75" t="n">
@@ -3307,7 +3295,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="1" t="n">
         <v>40969</v>
       </c>
       <c r="B76" t="n">
@@ -3345,7 +3333,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="1" t="n">
         <v>41000</v>
       </c>
       <c r="B77" t="n">
@@ -3383,7 +3371,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="1" t="n">
         <v>41030</v>
       </c>
       <c r="B78" t="n">
@@ -3421,7 +3409,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="1" t="n">
         <v>41061</v>
       </c>
       <c r="B79" t="n">
@@ -3459,7 +3447,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="1" t="n">
         <v>41091</v>
       </c>
       <c r="B80" t="n">
@@ -3497,7 +3485,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="1" t="n">
         <v>41122</v>
       </c>
       <c r="B81" t="n">
@@ -3535,7 +3523,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="1" t="n">
         <v>41153</v>
       </c>
       <c r="B82" t="n">
@@ -3573,7 +3561,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="1" t="n">
         <v>41183</v>
       </c>
       <c r="B83" t="n">
@@ -3611,7 +3599,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="1" t="n">
         <v>41214</v>
       </c>
       <c r="B84" t="n">
@@ -3649,7 +3637,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="1" t="n">
         <v>41244</v>
       </c>
       <c r="B85" t="n">
@@ -3687,7 +3675,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="1" t="n">
         <v>41275</v>
       </c>
       <c r="B86" t="n">
@@ -3725,7 +3713,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="1" t="n">
         <v>41306</v>
       </c>
       <c r="B87" t="n">
@@ -3763,7 +3751,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="1" t="n">
         <v>41334</v>
       </c>
       <c r="B88" t="n">
@@ -3801,7 +3789,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="1" t="n">
         <v>41365</v>
       </c>
       <c r="B89" t="n">
@@ -3839,7 +3827,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="1" t="n">
         <v>41395</v>
       </c>
       <c r="B90" t="n">
@@ -3877,7 +3865,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="1" t="n">
         <v>41426</v>
       </c>
       <c r="B91" t="n">
@@ -3915,7 +3903,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="1" t="n">
         <v>41456</v>
       </c>
       <c r="B92" t="n">
@@ -3953,7 +3941,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="1" t="n">
         <v>41487</v>
       </c>
       <c r="B93" t="n">
@@ -3991,7 +3979,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="1" t="n">
         <v>41518</v>
       </c>
       <c r="B94" t="n">
@@ -4029,7 +4017,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" s="1" t="n">
         <v>41548</v>
       </c>
       <c r="B95" t="n">
@@ -4067,7 +4055,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="1" t="n">
         <v>41579</v>
       </c>
       <c r="B96" t="n">
@@ -4105,7 +4093,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="1" t="n">
         <v>41609</v>
       </c>
       <c r="B97" t="n">
@@ -4143,7 +4131,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="1" t="n">
         <v>41640</v>
       </c>
       <c r="B98" t="n">
@@ -4181,7 +4169,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="1" t="n">
         <v>41671</v>
       </c>
       <c r="B99" t="n">
@@ -4219,7 +4207,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="1" t="n">
         <v>41699</v>
       </c>
       <c r="B100" t="n">
@@ -4257,7 +4245,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="1" t="n">
         <v>41730</v>
       </c>
       <c r="B101" t="n">
@@ -4295,7 +4283,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="1" t="n">
         <v>41760</v>
       </c>
       <c r="B102" t="n">
@@ -4333,7 +4321,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="1" t="n">
         <v>41791</v>
       </c>
       <c r="B103" t="n">
@@ -4371,7 +4359,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="1" t="n">
         <v>41821</v>
       </c>
       <c r="B104" t="n">
@@ -4409,7 +4397,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="1" t="n">
         <v>41852</v>
       </c>
       <c r="B105" t="n">
@@ -4447,7 +4435,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="1" t="n">
         <v>41883</v>
       </c>
       <c r="B106" t="n">
@@ -4485,7 +4473,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="1" t="n">
         <v>41913</v>
       </c>
       <c r="B107" t="n">
@@ -4523,7 +4511,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="1" t="n">
         <v>41944</v>
       </c>
       <c r="B108" t="n">
@@ -4561,7 +4549,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
+      <c r="A109" s="1" t="n">
         <v>41974</v>
       </c>
       <c r="B109" t="n">
@@ -4599,7 +4587,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
+      <c r="A110" s="1" t="n">
         <v>42005</v>
       </c>
       <c r="B110" t="n">
@@ -4637,7 +4625,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="1" t="n">
         <v>42036</v>
       </c>
       <c r="B111" t="n">
@@ -4675,7 +4663,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="1" t="n">
         <v>42064</v>
       </c>
       <c r="B112" t="n">
@@ -4713,7 +4701,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="1" t="n">
         <v>42095</v>
       </c>
       <c r="B113" t="n">
@@ -4751,7 +4739,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="1" t="n">
         <v>42125</v>
       </c>
       <c r="B114" t="n">
@@ -4789,7 +4777,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="1" t="n">
         <v>42156</v>
       </c>
       <c r="B115" t="n">
@@ -4827,7 +4815,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
+      <c r="A116" s="1" t="n">
         <v>42186</v>
       </c>
       <c r="B116" t="n">
@@ -4865,7 +4853,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
+      <c r="A117" s="1" t="n">
         <v>42217</v>
       </c>
       <c r="B117" t="n">
@@ -4903,7 +4891,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
+      <c r="A118" s="1" t="n">
         <v>42248</v>
       </c>
       <c r="B118" t="n">
@@ -4941,7 +4929,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
+      <c r="A119" s="1" t="n">
         <v>42278</v>
       </c>
       <c r="B119" t="n">
@@ -4979,7 +4967,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
+      <c r="A120" s="1" t="n">
         <v>42309</v>
       </c>
       <c r="B120" t="n">
@@ -5017,7 +5005,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
+      <c r="A121" s="1" t="n">
         <v>42339</v>
       </c>
       <c r="B121" t="n">
@@ -5055,7 +5043,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
+      <c r="A122" s="1" t="n">
         <v>42370</v>
       </c>
       <c r="B122" t="n">
@@ -5093,7 +5081,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
+      <c r="A123" s="1" t="n">
         <v>42401</v>
       </c>
       <c r="B123" t="n">
@@ -5131,7 +5119,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
+      <c r="A124" s="1" t="n">
         <v>42430</v>
       </c>
       <c r="B124" t="n">
@@ -5169,7 +5157,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
+      <c r="A125" s="1" t="n">
         <v>42461</v>
       </c>
       <c r="B125" t="n">
@@ -5207,7 +5195,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" s="1" t="n">
         <v>42491</v>
       </c>
       <c r="B126" t="n">
@@ -5245,7 +5233,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
+      <c r="A127" s="1" t="n">
         <v>42522</v>
       </c>
       <c r="B127" t="n">
@@ -5283,7 +5271,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
+      <c r="A128" s="1" t="n">
         <v>42552</v>
       </c>
       <c r="B128" t="n">
@@ -5321,7 +5309,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
+      <c r="A129" s="1" t="n">
         <v>42583</v>
       </c>
       <c r="B129" t="n">
@@ -5359,7 +5347,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
+      <c r="A130" s="1" t="n">
         <v>42614</v>
       </c>
       <c r="B130" t="n">
@@ -5397,7 +5385,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
+      <c r="A131" s="1" t="n">
         <v>42644</v>
       </c>
       <c r="B131" t="n">
@@ -5435,7 +5423,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" s="1" t="n">
         <v>42675</v>
       </c>
       <c r="B132" t="n">
@@ -5473,7 +5461,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" s="1" t="n">
         <v>42705</v>
       </c>
       <c r="B133" t="n">
@@ -5511,7 +5499,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
+      <c r="A134" s="1" t="n">
         <v>42736</v>
       </c>
       <c r="B134" t="n">
@@ -5549,7 +5537,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
+      <c r="A135" s="1" t="n">
         <v>42767</v>
       </c>
       <c r="B135" t="n">
@@ -5587,7 +5575,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="1" t="n">
         <v>42795</v>
       </c>
       <c r="B136" t="n">
@@ -5625,7 +5613,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
+      <c r="A137" s="1" t="n">
         <v>42826</v>
       </c>
       <c r="B137" t="n">
@@ -5663,7 +5651,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
+      <c r="A138" s="1" t="n">
         <v>42856</v>
       </c>
       <c r="B138" t="n">
@@ -5701,7 +5689,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
+      <c r="A139" s="1" t="n">
         <v>42887</v>
       </c>
       <c r="B139" t="n">
@@ -5739,7 +5727,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
+      <c r="A140" s="1" t="n">
         <v>42917</v>
       </c>
       <c r="B140" t="n">
@@ -5777,7 +5765,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
+      <c r="A141" s="1" t="n">
         <v>42948</v>
       </c>
       <c r="B141" t="n">
@@ -5815,7 +5803,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
+      <c r="A142" s="1" t="n">
         <v>42979</v>
       </c>
       <c r="B142" t="n">
@@ -5853,7 +5841,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
+      <c r="A143" s="1" t="n">
         <v>43009</v>
       </c>
       <c r="B143" t="n">
@@ -5891,7 +5879,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
+      <c r="A144" s="1" t="n">
         <v>43040</v>
       </c>
       <c r="B144" t="n">
@@ -5929,7 +5917,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
+      <c r="A145" s="1" t="n">
         <v>43070</v>
       </c>
       <c r="B145" t="n">
@@ -5967,7 +5955,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n">
+      <c r="A146" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="B146" t="n">
@@ -6005,7 +5993,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
+      <c r="A147" s="1" t="n">
         <v>43132</v>
       </c>
       <c r="B147" t="n">
@@ -6043,7 +6031,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
+      <c r="A148" s="1" t="n">
         <v>43160</v>
       </c>
       <c r="B148" t="n">
@@ -6081,7 +6069,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
+      <c r="A149" s="1" t="n">
         <v>43191</v>
       </c>
       <c r="B149" t="n">
@@ -6119,7 +6107,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
+      <c r="A150" s="1" t="n">
         <v>43221</v>
       </c>
       <c r="B150" t="n">
@@ -6157,7 +6145,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n">
+      <c r="A151" s="1" t="n">
         <v>43252</v>
       </c>
       <c r="B151" t="n">
@@ -6195,7 +6183,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n">
+      <c r="A152" s="1" t="n">
         <v>43282</v>
       </c>
       <c r="B152" t="n">
@@ -6233,7 +6221,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
+      <c r="A153" s="1" t="n">
         <v>43313</v>
       </c>
       <c r="B153" t="n">
@@ -6271,7 +6259,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
+      <c r="A154" s="1" t="n">
         <v>43344</v>
       </c>
       <c r="B154" t="n">
@@ -6309,7 +6297,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n">
+      <c r="A155" s="1" t="n">
         <v>43374</v>
       </c>
       <c r="B155" t="n">
@@ -6347,7 +6335,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
+      <c r="A156" s="1" t="n">
         <v>43405</v>
       </c>
       <c r="B156" t="n">
@@ -6385,7 +6373,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n">
+      <c r="A157" s="1" t="n">
         <v>43435</v>
       </c>
       <c r="B157" t="n">
@@ -6423,7 +6411,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n">
+      <c r="A158" s="1" t="n">
         <v>43466</v>
       </c>
       <c r="B158" t="n">
@@ -6461,7 +6449,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n">
+      <c r="A159" s="1" t="n">
         <v>43497</v>
       </c>
       <c r="B159" t="n">
@@ -6499,7 +6487,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
+      <c r="A160" s="1" t="n">
         <v>43525</v>
       </c>
       <c r="B160" t="n">
@@ -6537,7 +6525,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
+      <c r="A161" s="1" t="n">
         <v>43556</v>
       </c>
       <c r="B161" t="n">
@@ -6575,7 +6563,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
+      <c r="A162" s="1" t="n">
         <v>43586</v>
       </c>
       <c r="B162" t="n">
@@ -6613,7 +6601,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
+      <c r="A163" s="1" t="n">
         <v>43617</v>
       </c>
       <c r="B163" t="n">
@@ -6651,7 +6639,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
+      <c r="A164" s="1" t="n">
         <v>43647</v>
       </c>
       <c r="B164" t="n">
@@ -6689,7 +6677,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n">
+      <c r="A165" s="1" t="n">
         <v>43678</v>
       </c>
       <c r="B165" t="n">
@@ -6727,7 +6715,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n">
+      <c r="A166" s="1" t="n">
         <v>43709</v>
       </c>
       <c r="B166" t="n">
@@ -6765,7 +6753,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
+      <c r="A167" s="1" t="n">
         <v>43739</v>
       </c>
       <c r="B167" t="n">
@@ -6803,7 +6791,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
+      <c r="A168" s="1" t="n">
         <v>43770</v>
       </c>
       <c r="B168" t="n">
@@ -6841,7 +6829,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
+      <c r="A169" s="1" t="n">
         <v>43800</v>
       </c>
       <c r="B169" t="n">
@@ -6879,7 +6867,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n">
+      <c r="A170" s="1" t="n">
         <v>43831</v>
       </c>
       <c r="B170" t="n">
@@ -6917,7 +6905,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
+      <c r="A171" s="1" t="n">
         <v>43862</v>
       </c>
       <c r="B171" t="n">
@@ -6955,7 +6943,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n">
+      <c r="A172" s="1" t="n">
         <v>43891</v>
       </c>
       <c r="B172" t="n">
@@ -6993,7 +6981,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n">
+      <c r="A173" s="1" t="n">
         <v>43922</v>
       </c>
       <c r="B173" t="n">
@@ -7031,7 +7019,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
+      <c r="A174" s="1" t="n">
         <v>43952</v>
       </c>
       <c r="B174" t="n">
@@ -7069,7 +7057,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
+      <c r="A175" s="1" t="n">
         <v>43983</v>
       </c>
       <c r="B175" t="n">
@@ -7107,7 +7095,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
+      <c r="A176" s="1" t="n">
         <v>44013</v>
       </c>
       <c r="B176" t="n">
@@ -7145,7 +7133,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
+      <c r="A177" s="1" t="n">
         <v>44044</v>
       </c>
       <c r="B177" t="n">
@@ -7183,7 +7171,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
+      <c r="A178" s="1" t="n">
         <v>44075</v>
       </c>
       <c r="B178" t="n">
@@ -7221,7 +7209,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n">
+      <c r="A179" s="1" t="n">
         <v>44105</v>
       </c>
       <c r="B179" t="n">
@@ -7259,7 +7247,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n">
+      <c r="A180" s="1" t="n">
         <v>44136</v>
       </c>
       <c r="B180" t="n">
@@ -7297,7 +7285,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
+      <c r="A181" s="1" t="n">
         <v>44166</v>
       </c>
       <c r="B181" t="n">
@@ -7335,7 +7323,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
+      <c r="A182" s="1" t="n">
         <v>44197</v>
       </c>
       <c r="B182" t="n">
@@ -7373,7 +7361,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
+      <c r="A183" s="1" t="n">
         <v>44228</v>
       </c>
       <c r="B183" t="n">
@@ -7411,7 +7399,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n">
+      <c r="A184" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="B184" t="n">
@@ -7449,7 +7437,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n">
+      <c r="A185" s="1" t="n">
         <v>44287</v>
       </c>
       <c r="B185" t="n">
@@ -7487,7 +7475,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n">
+      <c r="A186" s="1" t="n">
         <v>44317</v>
       </c>
       <c r="B186" t="n">
@@ -7525,7 +7513,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n">
+      <c r="A187" s="1" t="n">
         <v>44348</v>
       </c>
       <c r="B187" t="n">
@@ -7563,7 +7551,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n">
+      <c r="A188" s="1" t="n">
         <v>44378</v>
       </c>
       <c r="B188" t="n">
@@ -7601,7 +7589,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n">
+      <c r="A189" s="1" t="n">
         <v>44409</v>
       </c>
       <c r="B189" t="n">
@@ -7639,7 +7627,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n">
+      <c r="A190" s="1" t="n">
         <v>44440</v>
       </c>
       <c r="B190" t="n">
@@ -7677,7 +7665,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="n">
+      <c r="A191" s="1" t="n">
         <v>44470</v>
       </c>
       <c r="B191" t="n">
@@ -7715,7 +7703,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n">
+      <c r="A192" s="1" t="n">
         <v>44501</v>
       </c>
       <c r="B192" t="n">
@@ -7753,7 +7741,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="n">
+      <c r="A193" s="1" t="n">
         <v>44531</v>
       </c>
       <c r="B193" t="n">
@@ -7791,7 +7779,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="n">
+      <c r="A194" s="1" t="n">
         <v>44562</v>
       </c>
       <c r="B194" t="n">
@@ -7829,7 +7817,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="n">
+      <c r="A195" s="1" t="n">
         <v>44593</v>
       </c>
       <c r="B195" t="n">
@@ -7867,7 +7855,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="n">
+      <c r="A196" s="1" t="n">
         <v>44621</v>
       </c>
       <c r="B196" t="n">
@@ -7905,7 +7893,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="n">
+      <c r="A197" s="1" t="n">
         <v>44652</v>
       </c>
       <c r="B197" t="n">
@@ -7943,7 +7931,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n">
+      <c r="A198" s="1" t="n">
         <v>44682</v>
       </c>
       <c r="B198" t="n">
@@ -7981,7 +7969,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="n">
+      <c r="A199" s="1" t="n">
         <v>44713</v>
       </c>
       <c r="B199" t="n">
@@ -8019,7 +8007,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n">
+      <c r="A200" s="1" t="n">
         <v>44743</v>
       </c>
       <c r="B200" t="n">
@@ -8057,7 +8045,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="n">
+      <c r="A201" s="1" t="n">
         <v>44774</v>
       </c>
       <c r="B201" t="n">
@@ -8095,7 +8083,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="n">
+      <c r="A202" s="1" t="n">
         <v>44805</v>
       </c>
       <c r="B202" t="n">
@@ -8133,7 +8121,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="n">
+      <c r="A203" s="1" t="n">
         <v>44835</v>
       </c>
       <c r="B203" t="n">
@@ -8171,7 +8159,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="n">
+      <c r="A204" s="1" t="n">
         <v>44866</v>
       </c>
       <c r="B204" t="n">
@@ -8209,7 +8197,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="n">
+      <c r="A205" s="1" t="n">
         <v>44896</v>
       </c>
       <c r="B205" t="n">
@@ -8247,7 +8235,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="n">
+      <c r="A206" s="1" t="n">
         <v>44927</v>
       </c>
       <c r="B206" t="n">
@@ -8285,7 +8273,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="n">
+      <c r="A207" s="1" t="n">
         <v>44958</v>
       </c>
       <c r="B207" t="n">
@@ -8323,7 +8311,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="n">
+      <c r="A208" s="1" t="n">
         <v>44986</v>
       </c>
       <c r="B208" t="n">
@@ -8361,7 +8349,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="n">
+      <c r="A209" s="1" t="n">
         <v>45017</v>
       </c>
       <c r="B209" t="n">
@@ -8399,7 +8387,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n">
+      <c r="A210" s="1" t="n">
         <v>45047</v>
       </c>
       <c r="B210" t="n">
@@ -8437,7 +8425,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="2" t="n">
+      <c r="A211" s="1" t="n">
         <v>45078</v>
       </c>
       <c r="B211" t="n">
@@ -8475,7 +8463,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="n">
+      <c r="A212" s="1" t="n">
         <v>45108</v>
       </c>
       <c r="B212" t="n">
@@ -8513,7 +8501,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="n">
+      <c r="A213" s="1" t="n">
         <v>45139</v>
       </c>
       <c r="B213" t="n">
@@ -8551,7 +8539,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="n">
+      <c r="A214" s="1" t="n">
         <v>45170</v>
       </c>
       <c r="B214" t="n">
@@ -8589,7 +8577,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="2" t="n">
+      <c r="A215" s="1" t="n">
         <v>45200</v>
       </c>
       <c r="B215" t="n">
@@ -8627,7 +8615,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="2" t="n">
+      <c r="A216" s="1" t="n">
         <v>45231</v>
       </c>
       <c r="B216" t="n">
@@ -8665,7 +8653,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="n">
+      <c r="A217" s="1" t="n">
         <v>45261</v>
       </c>
       <c r="B217" t="n">
@@ -8703,7 +8691,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="n">
+      <c r="A218" s="1" t="n">
         <v>45292</v>
       </c>
       <c r="B218" t="n">
@@ -8741,7 +8729,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="n">
+      <c r="A219" s="1" t="n">
         <v>45323</v>
       </c>
       <c r="B219" t="n">
@@ -8779,7 +8767,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="n">
+      <c r="A220" s="1" t="n">
         <v>45352</v>
       </c>
       <c r="B220" t="n">
@@ -8817,7 +8805,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="n">
+      <c r="A221" s="1" t="n">
         <v>45383</v>
       </c>
       <c r="B221" t="n">
@@ -8855,7 +8843,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="n">
+      <c r="A222" s="1" t="n">
         <v>45413</v>
       </c>
       <c r="B222" t="n">
@@ -8893,7 +8881,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="n">
+      <c r="A223" s="1" t="n">
         <v>45444</v>
       </c>
       <c r="B223" t="n">
@@ -8931,7 +8919,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="n">
+      <c r="A224" s="1" t="n">
         <v>45474</v>
       </c>
       <c r="B224" t="n">
@@ -8969,7 +8957,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="n">
+      <c r="A225" s="1" t="n">
         <v>45505</v>
       </c>
       <c r="B225" t="n">
@@ -9007,7 +8995,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="n">
+      <c r="A226" s="1" t="n">
         <v>45536</v>
       </c>
       <c r="B226" t="n">
@@ -9045,7 +9033,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="n">
+      <c r="A227" s="1" t="n">
         <v>45566</v>
       </c>
       <c r="B227" t="n">
@@ -9083,7 +9071,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="n">
+      <c r="A228" s="1" t="n">
         <v>45597</v>
       </c>
       <c r="B228" t="n">
@@ -9121,7 +9109,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="n">
+      <c r="A229" s="1" t="n">
         <v>45627</v>
       </c>
       <c r="B229" t="n">
@@ -9159,7 +9147,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="n">
+      <c r="A230" s="1" t="n">
         <v>45658</v>
       </c>
       <c r="B230" t="n">
@@ -9197,7 +9185,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="n">
+      <c r="A231" s="1" t="n">
         <v>45689</v>
       </c>
       <c r="B231" t="n">
@@ -9235,7 +9223,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="n">
+      <c r="A232" s="1" t="n">
         <v>45717</v>
       </c>
       <c r="B232" t="n">
@@ -9273,7 +9261,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="n">
+      <c r="A233" s="1" t="n">
         <v>45748</v>
       </c>
       <c r="B233" t="n">
@@ -9311,7 +9299,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="n">
+      <c r="A234" s="1" t="n">
         <v>45778</v>
       </c>
       <c r="B234" t="n">
@@ -9349,7 +9337,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="n">
+      <c r="A235" s="1" t="n">
         <v>45809</v>
       </c>
       <c r="B235" t="n">
@@ -9387,7 +9375,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="2" t="n">
+      <c r="A236" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="B236" t="n">
@@ -9425,7 +9413,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="2" t="n">
+      <c r="A237" s="1" t="n">
         <v>45870</v>
       </c>
       <c r="B237" t="n">
@@ -9463,7 +9451,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="2" t="n">
+      <c r="A238" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="B238" t="n">
@@ -9501,7 +9489,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="2" t="n">
+      <c r="A239" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="B239" t="n">
@@ -9539,7 +9527,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="2" t="n">
+      <c r="A240" s="1" t="n">
         <v>45962</v>
       </c>
       <c r="B240" t="n">
@@ -9577,7 +9565,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="2" t="n">
+      <c r="A241" s="1" t="n">
         <v>45992</v>
       </c>
       <c r="B241" t="n">
@@ -9615,7 +9603,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="2" t="n">
+      <c r="A242" s="1" t="n">
         <v>46023</v>
       </c>
       <c r="B242" t="n">
@@ -9653,7 +9641,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="n">
+      <c r="A243" s="1" t="n">
         <v>46054</v>
       </c>
       <c r="B243" t="n">
@@ -9691,7 +9679,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="2" t="n">
+      <c r="A244" s="1" t="n">
         <v>46082</v>
       </c>
       <c r="B244" t="n">
@@ -9729,7 +9717,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="2" t="n">
+      <c r="A245" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="B245" t="n">
@@ -9767,7 +9755,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="2" t="n">
+      <c r="A246" s="1" t="n">
         <v>46143</v>
       </c>
       <c r="B246" t="n">

</xml_diff>

<commit_message>
Toplu veri güncelleme (yerel, 17.07.2026 13:30)
</commit_message>
<xml_diff>
--- a/butce/butce.xlsx
+++ b/butce/butce.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,69 +433,69 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>tarih</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>yil</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ay</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>gelir</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>vergi</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>dolaysiz_vergi</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>dolayli_vergi</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>gider</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>faiz_haric_gider</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>faiz_gideri</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>faiz_disi_denge</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>denge</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>38718</v>
       </c>
       <c r="B2" t="n">
@@ -521,7 +533,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>38749</v>
       </c>
       <c r="B3" t="n">
@@ -559,7 +571,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>38777</v>
       </c>
       <c r="B4" t="n">
@@ -597,7 +609,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>38808</v>
       </c>
       <c r="B5" t="n">
@@ -635,7 +647,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>38838</v>
       </c>
       <c r="B6" t="n">
@@ -673,7 +685,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>38869</v>
       </c>
       <c r="B7" t="n">
@@ -711,7 +723,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>38899</v>
       </c>
       <c r="B8" t="n">
@@ -749,7 +761,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>38930</v>
       </c>
       <c r="B9" t="n">
@@ -787,7 +799,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>38961</v>
       </c>
       <c r="B10" t="n">
@@ -825,7 +837,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>38991</v>
       </c>
       <c r="B11" t="n">
@@ -863,7 +875,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>39022</v>
       </c>
       <c r="B12" t="n">
@@ -901,7 +913,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>39052</v>
       </c>
       <c r="B13" t="n">
@@ -939,7 +951,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>39083</v>
       </c>
       <c r="B14" t="n">
@@ -977,7 +989,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>39114</v>
       </c>
       <c r="B15" t="n">
@@ -1015,7 +1027,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>39142</v>
       </c>
       <c r="B16" t="n">
@@ -1053,7 +1065,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>39173</v>
       </c>
       <c r="B17" t="n">
@@ -1091,7 +1103,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>39203</v>
       </c>
       <c r="B18" t="n">
@@ -1129,7 +1141,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>39234</v>
       </c>
       <c r="B19" t="n">
@@ -1167,7 +1179,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>39264</v>
       </c>
       <c r="B20" t="n">
@@ -1205,7 +1217,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>39295</v>
       </c>
       <c r="B21" t="n">
@@ -1243,7 +1255,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>39326</v>
       </c>
       <c r="B22" t="n">
@@ -1281,7 +1293,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>39356</v>
       </c>
       <c r="B23" t="n">
@@ -1319,7 +1331,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>39387</v>
       </c>
       <c r="B24" t="n">
@@ -1357,7 +1369,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>39417</v>
       </c>
       <c r="B25" t="n">
@@ -1395,7 +1407,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>39448</v>
       </c>
       <c r="B26" t="n">
@@ -1433,7 +1445,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>39479</v>
       </c>
       <c r="B27" t="n">
@@ -1471,7 +1483,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>39508</v>
       </c>
       <c r="B28" t="n">
@@ -1509,7 +1521,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>39539</v>
       </c>
       <c r="B29" t="n">
@@ -1547,7 +1559,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>39569</v>
       </c>
       <c r="B30" t="n">
@@ -1585,7 +1597,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>39600</v>
       </c>
       <c r="B31" t="n">
@@ -1623,7 +1635,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>39630</v>
       </c>
       <c r="B32" t="n">
@@ -1661,7 +1673,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>39661</v>
       </c>
       <c r="B33" t="n">
@@ -1699,7 +1711,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>39692</v>
       </c>
       <c r="B34" t="n">
@@ -1737,7 +1749,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>39722</v>
       </c>
       <c r="B35" t="n">
@@ -1775,7 +1787,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>39753</v>
       </c>
       <c r="B36" t="n">
@@ -1813,7 +1825,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>39783</v>
       </c>
       <c r="B37" t="n">
@@ -1851,7 +1863,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>39814</v>
       </c>
       <c r="B38" t="n">
@@ -1889,7 +1901,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>39845</v>
       </c>
       <c r="B39" t="n">
@@ -1927,7 +1939,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>39873</v>
       </c>
       <c r="B40" t="n">
@@ -1965,7 +1977,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>39904</v>
       </c>
       <c r="B41" t="n">
@@ -2003,7 +2015,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>39934</v>
       </c>
       <c r="B42" t="n">
@@ -2041,7 +2053,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>39965</v>
       </c>
       <c r="B43" t="n">
@@ -2079,7 +2091,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>39995</v>
       </c>
       <c r="B44" t="n">
@@ -2117,7 +2129,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>40026</v>
       </c>
       <c r="B45" t="n">
@@ -2155,7 +2167,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>40057</v>
       </c>
       <c r="B46" t="n">
@@ -2193,7 +2205,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>40087</v>
       </c>
       <c r="B47" t="n">
@@ -2231,7 +2243,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>40118</v>
       </c>
       <c r="B48" t="n">
@@ -2269,7 +2281,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>40148</v>
       </c>
       <c r="B49" t="n">
@@ -2307,7 +2319,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>40179</v>
       </c>
       <c r="B50" t="n">
@@ -2345,7 +2357,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>40210</v>
       </c>
       <c r="B51" t="n">
@@ -2383,7 +2395,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>40238</v>
       </c>
       <c r="B52" t="n">
@@ -2421,7 +2433,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>40269</v>
       </c>
       <c r="B53" t="n">
@@ -2459,7 +2471,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>40299</v>
       </c>
       <c r="B54" t="n">
@@ -2497,7 +2509,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>40330</v>
       </c>
       <c r="B55" t="n">
@@ -2535,7 +2547,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>40360</v>
       </c>
       <c r="B56" t="n">
@@ -2573,7 +2585,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>40391</v>
       </c>
       <c r="B57" t="n">
@@ -2611,7 +2623,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>40422</v>
       </c>
       <c r="B58" t="n">
@@ -2649,7 +2661,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>40452</v>
       </c>
       <c r="B59" t="n">
@@ -2687,7 +2699,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>40483</v>
       </c>
       <c r="B60" t="n">
@@ -2725,7 +2737,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>40513</v>
       </c>
       <c r="B61" t="n">
@@ -2763,7 +2775,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>40544</v>
       </c>
       <c r="B62" t="n">
@@ -2801,7 +2813,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" s="2" t="n">
         <v>40575</v>
       </c>
       <c r="B63" t="n">
@@ -2839,7 +2851,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" s="2" t="n">
         <v>40603</v>
       </c>
       <c r="B64" t="n">
@@ -2877,7 +2889,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" s="2" t="n">
         <v>40634</v>
       </c>
       <c r="B65" t="n">
@@ -2915,7 +2927,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="2" t="n">
         <v>40664</v>
       </c>
       <c r="B66" t="n">
@@ -2953,7 +2965,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="2" t="n">
         <v>40695</v>
       </c>
       <c r="B67" t="n">
@@ -2991,7 +3003,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="2" t="n">
         <v>40725</v>
       </c>
       <c r="B68" t="n">
@@ -3029,7 +3041,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="2" t="n">
         <v>40756</v>
       </c>
       <c r="B69" t="n">
@@ -3067,7 +3079,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="2" t="n">
         <v>40787</v>
       </c>
       <c r="B70" t="n">
@@ -3105,7 +3117,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="2" t="n">
         <v>40817</v>
       </c>
       <c r="B71" t="n">
@@ -3143,7 +3155,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" s="2" t="n">
         <v>40848</v>
       </c>
       <c r="B72" t="n">
@@ -3181,7 +3193,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="2" t="n">
         <v>40878</v>
       </c>
       <c r="B73" t="n">
@@ -3219,7 +3231,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="2" t="n">
         <v>40909</v>
       </c>
       <c r="B74" t="n">
@@ -3257,7 +3269,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="2" t="n">
         <v>40940</v>
       </c>
       <c r="B75" t="n">
@@ -3295,7 +3307,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="2" t="n">
         <v>40969</v>
       </c>
       <c r="B76" t="n">
@@ -3333,7 +3345,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="2" t="n">
         <v>41000</v>
       </c>
       <c r="B77" t="n">
@@ -3371,7 +3383,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="2" t="n">
         <v>41030</v>
       </c>
       <c r="B78" t="n">
@@ -3409,7 +3421,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="2" t="n">
         <v>41061</v>
       </c>
       <c r="B79" t="n">
@@ -3447,7 +3459,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="2" t="n">
         <v>41091</v>
       </c>
       <c r="B80" t="n">
@@ -3485,7 +3497,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" s="2" t="n">
         <v>41122</v>
       </c>
       <c r="B81" t="n">
@@ -3523,7 +3535,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" s="2" t="n">
         <v>41153</v>
       </c>
       <c r="B82" t="n">
@@ -3561,7 +3573,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="2" t="n">
         <v>41183</v>
       </c>
       <c r="B83" t="n">
@@ -3599,7 +3611,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="2" t="n">
         <v>41214</v>
       </c>
       <c r="B84" t="n">
@@ -3637,7 +3649,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" s="2" t="n">
         <v>41244</v>
       </c>
       <c r="B85" t="n">
@@ -3675,7 +3687,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" s="2" t="n">
         <v>41275</v>
       </c>
       <c r="B86" t="n">
@@ -3713,7 +3725,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="2" t="n">
         <v>41306</v>
       </c>
       <c r="B87" t="n">
@@ -3751,7 +3763,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="2" t="n">
         <v>41334</v>
       </c>
       <c r="B88" t="n">
@@ -3789,7 +3801,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="2" t="n">
         <v>41365</v>
       </c>
       <c r="B89" t="n">
@@ -3827,7 +3839,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="2" t="n">
         <v>41395</v>
       </c>
       <c r="B90" t="n">
@@ -3865,7 +3877,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="2" t="n">
         <v>41426</v>
       </c>
       <c r="B91" t="n">
@@ -3903,7 +3915,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="2" t="n">
         <v>41456</v>
       </c>
       <c r="B92" t="n">
@@ -3941,7 +3953,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" s="2" t="n">
         <v>41487</v>
       </c>
       <c r="B93" t="n">
@@ -3979,7 +3991,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" s="2" t="n">
         <v>41518</v>
       </c>
       <c r="B94" t="n">
@@ -4017,7 +4029,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" s="2" t="n">
         <v>41548</v>
       </c>
       <c r="B95" t="n">
@@ -4055,7 +4067,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" s="2" t="n">
         <v>41579</v>
       </c>
       <c r="B96" t="n">
@@ -4093,7 +4105,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" s="2" t="n">
         <v>41609</v>
       </c>
       <c r="B97" t="n">
@@ -4131,7 +4143,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" s="2" t="n">
         <v>41640</v>
       </c>
       <c r="B98" t="n">
@@ -4169,7 +4181,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" s="2" t="n">
         <v>41671</v>
       </c>
       <c r="B99" t="n">
@@ -4207,7 +4219,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" s="2" t="n">
         <v>41699</v>
       </c>
       <c r="B100" t="n">
@@ -4245,7 +4257,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" s="2" t="n">
         <v>41730</v>
       </c>
       <c r="B101" t="n">
@@ -4283,7 +4295,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" s="2" t="n">
         <v>41760</v>
       </c>
       <c r="B102" t="n">
@@ -4321,7 +4333,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" s="2" t="n">
         <v>41791</v>
       </c>
       <c r="B103" t="n">
@@ -4359,7 +4371,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" s="2" t="n">
         <v>41821</v>
       </c>
       <c r="B104" t="n">
@@ -4397,7 +4409,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" s="2" t="n">
         <v>41852</v>
       </c>
       <c r="B105" t="n">
@@ -4435,7 +4447,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" s="2" t="n">
         <v>41883</v>
       </c>
       <c r="B106" t="n">
@@ -4473,7 +4485,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" s="2" t="n">
         <v>41913</v>
       </c>
       <c r="B107" t="n">
@@ -4511,7 +4523,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" s="2" t="n">
         <v>41944</v>
       </c>
       <c r="B108" t="n">
@@ -4549,7 +4561,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" s="2" t="n">
         <v>41974</v>
       </c>
       <c r="B109" t="n">
@@ -4587,7 +4599,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" s="2" t="n">
         <v>42005</v>
       </c>
       <c r="B110" t="n">
@@ -4625,7 +4637,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" s="2" t="n">
         <v>42036</v>
       </c>
       <c r="B111" t="n">
@@ -4663,7 +4675,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" s="2" t="n">
         <v>42064</v>
       </c>
       <c r="B112" t="n">
@@ -4701,7 +4713,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" s="2" t="n">
         <v>42095</v>
       </c>
       <c r="B113" t="n">
@@ -4739,7 +4751,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" s="2" t="n">
         <v>42125</v>
       </c>
       <c r="B114" t="n">
@@ -4777,7 +4789,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" s="2" t="n">
         <v>42156</v>
       </c>
       <c r="B115" t="n">
@@ -4815,7 +4827,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" s="2" t="n">
         <v>42186</v>
       </c>
       <c r="B116" t="n">
@@ -4853,7 +4865,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" s="2" t="n">
         <v>42217</v>
       </c>
       <c r="B117" t="n">
@@ -4891,7 +4903,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" s="2" t="n">
         <v>42248</v>
       </c>
       <c r="B118" t="n">
@@ -4929,7 +4941,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" s="2" t="n">
         <v>42278</v>
       </c>
       <c r="B119" t="n">
@@ -4967,7 +4979,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" s="2" t="n">
         <v>42309</v>
       </c>
       <c r="B120" t="n">
@@ -5005,7 +5017,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" s="2" t="n">
         <v>42339</v>
       </c>
       <c r="B121" t="n">
@@ -5043,7 +5055,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" s="2" t="n">
         <v>42370</v>
       </c>
       <c r="B122" t="n">
@@ -5081,7 +5093,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" s="2" t="n">
         <v>42401</v>
       </c>
       <c r="B123" t="n">
@@ -5119,7 +5131,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" s="2" t="n">
         <v>42430</v>
       </c>
       <c r="B124" t="n">
@@ -5157,7 +5169,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" s="2" t="n">
         <v>42461</v>
       </c>
       <c r="B125" t="n">
@@ -5195,7 +5207,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" s="2" t="n">
         <v>42491</v>
       </c>
       <c r="B126" t="n">
@@ -5233,7 +5245,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" s="2" t="n">
         <v>42522</v>
       </c>
       <c r="B127" t="n">
@@ -5271,7 +5283,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" s="2" t="n">
         <v>42552</v>
       </c>
       <c r="B128" t="n">
@@ -5309,7 +5321,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" s="2" t="n">
         <v>42583</v>
       </c>
       <c r="B129" t="n">
@@ -5347,7 +5359,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
+      <c r="A130" s="2" t="n">
         <v>42614</v>
       </c>
       <c r="B130" t="n">
@@ -5385,7 +5397,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
+      <c r="A131" s="2" t="n">
         <v>42644</v>
       </c>
       <c r="B131" t="n">
@@ -5423,7 +5435,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
+      <c r="A132" s="2" t="n">
         <v>42675</v>
       </c>
       <c r="B132" t="n">
@@ -5461,7 +5473,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
+      <c r="A133" s="2" t="n">
         <v>42705</v>
       </c>
       <c r="B133" t="n">
@@ -5499,7 +5511,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
+      <c r="A134" s="2" t="n">
         <v>42736</v>
       </c>
       <c r="B134" t="n">
@@ -5537,7 +5549,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
+      <c r="A135" s="2" t="n">
         <v>42767</v>
       </c>
       <c r="B135" t="n">
@@ -5575,7 +5587,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
+      <c r="A136" s="2" t="n">
         <v>42795</v>
       </c>
       <c r="B136" t="n">
@@ -5613,7 +5625,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
+      <c r="A137" s="2" t="n">
         <v>42826</v>
       </c>
       <c r="B137" t="n">
@@ -5651,7 +5663,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
+      <c r="A138" s="2" t="n">
         <v>42856</v>
       </c>
       <c r="B138" t="n">
@@ -5689,7 +5701,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="n">
+      <c r="A139" s="2" t="n">
         <v>42887</v>
       </c>
       <c r="B139" t="n">
@@ -5727,7 +5739,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="n">
+      <c r="A140" s="2" t="n">
         <v>42917</v>
       </c>
       <c r="B140" t="n">
@@ -5765,7 +5777,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="n">
+      <c r="A141" s="2" t="n">
         <v>42948</v>
       </c>
       <c r="B141" t="n">
@@ -5803,7 +5815,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="n">
+      <c r="A142" s="2" t="n">
         <v>42979</v>
       </c>
       <c r="B142" t="n">
@@ -5841,7 +5853,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="n">
+      <c r="A143" s="2" t="n">
         <v>43009</v>
       </c>
       <c r="B143" t="n">
@@ -5879,7 +5891,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="n">
+      <c r="A144" s="2" t="n">
         <v>43040</v>
       </c>
       <c r="B144" t="n">
@@ -5917,7 +5929,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="n">
+      <c r="A145" s="2" t="n">
         <v>43070</v>
       </c>
       <c r="B145" t="n">
@@ -5955,7 +5967,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="1" t="n">
+      <c r="A146" s="2" t="n">
         <v>43101</v>
       </c>
       <c r="B146" t="n">
@@ -5993,7 +6005,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="1" t="n">
+      <c r="A147" s="2" t="n">
         <v>43132</v>
       </c>
       <c r="B147" t="n">
@@ -6031,7 +6043,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="1" t="n">
+      <c r="A148" s="2" t="n">
         <v>43160</v>
       </c>
       <c r="B148" t="n">
@@ -6069,7 +6081,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="1" t="n">
+      <c r="A149" s="2" t="n">
         <v>43191</v>
       </c>
       <c r="B149" t="n">
@@ -6107,7 +6119,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="1" t="n">
+      <c r="A150" s="2" t="n">
         <v>43221</v>
       </c>
       <c r="B150" t="n">
@@ -6145,7 +6157,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="1" t="n">
+      <c r="A151" s="2" t="n">
         <v>43252</v>
       </c>
       <c r="B151" t="n">
@@ -6183,7 +6195,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="1" t="n">
+      <c r="A152" s="2" t="n">
         <v>43282</v>
       </c>
       <c r="B152" t="n">
@@ -6221,7 +6233,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="1" t="n">
+      <c r="A153" s="2" t="n">
         <v>43313</v>
       </c>
       <c r="B153" t="n">
@@ -6259,7 +6271,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="1" t="n">
+      <c r="A154" s="2" t="n">
         <v>43344</v>
       </c>
       <c r="B154" t="n">
@@ -6297,7 +6309,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="1" t="n">
+      <c r="A155" s="2" t="n">
         <v>43374</v>
       </c>
       <c r="B155" t="n">
@@ -6335,7 +6347,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="1" t="n">
+      <c r="A156" s="2" t="n">
         <v>43405</v>
       </c>
       <c r="B156" t="n">
@@ -6373,7 +6385,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="1" t="n">
+      <c r="A157" s="2" t="n">
         <v>43435</v>
       </c>
       <c r="B157" t="n">
@@ -6411,7 +6423,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="1" t="n">
+      <c r="A158" s="2" t="n">
         <v>43466</v>
       </c>
       <c r="B158" t="n">
@@ -6449,7 +6461,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="1" t="n">
+      <c r="A159" s="2" t="n">
         <v>43497</v>
       </c>
       <c r="B159" t="n">
@@ -6487,7 +6499,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="1" t="n">
+      <c r="A160" s="2" t="n">
         <v>43525</v>
       </c>
       <c r="B160" t="n">
@@ -6525,7 +6537,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="1" t="n">
+      <c r="A161" s="2" t="n">
         <v>43556</v>
       </c>
       <c r="B161" t="n">
@@ -6563,7 +6575,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="1" t="n">
+      <c r="A162" s="2" t="n">
         <v>43586</v>
       </c>
       <c r="B162" t="n">
@@ -6601,7 +6613,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="1" t="n">
+      <c r="A163" s="2" t="n">
         <v>43617</v>
       </c>
       <c r="B163" t="n">
@@ -6639,7 +6651,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="1" t="n">
+      <c r="A164" s="2" t="n">
         <v>43647</v>
       </c>
       <c r="B164" t="n">
@@ -6677,7 +6689,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="1" t="n">
+      <c r="A165" s="2" t="n">
         <v>43678</v>
       </c>
       <c r="B165" t="n">
@@ -6715,7 +6727,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="1" t="n">
+      <c r="A166" s="2" t="n">
         <v>43709</v>
       </c>
       <c r="B166" t="n">
@@ -6753,7 +6765,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="1" t="n">
+      <c r="A167" s="2" t="n">
         <v>43739</v>
       </c>
       <c r="B167" t="n">
@@ -6791,7 +6803,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="1" t="n">
+      <c r="A168" s="2" t="n">
         <v>43770</v>
       </c>
       <c r="B168" t="n">
@@ -6829,7 +6841,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="1" t="n">
+      <c r="A169" s="2" t="n">
         <v>43800</v>
       </c>
       <c r="B169" t="n">
@@ -6867,7 +6879,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="1" t="n">
+      <c r="A170" s="2" t="n">
         <v>43831</v>
       </c>
       <c r="B170" t="n">
@@ -6905,7 +6917,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="1" t="n">
+      <c r="A171" s="2" t="n">
         <v>43862</v>
       </c>
       <c r="B171" t="n">
@@ -6943,7 +6955,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="1" t="n">
+      <c r="A172" s="2" t="n">
         <v>43891</v>
       </c>
       <c r="B172" t="n">
@@ -6981,7 +6993,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="1" t="n">
+      <c r="A173" s="2" t="n">
         <v>43922</v>
       </c>
       <c r="B173" t="n">
@@ -7019,7 +7031,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="1" t="n">
+      <c r="A174" s="2" t="n">
         <v>43952</v>
       </c>
       <c r="B174" t="n">
@@ -7057,7 +7069,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="1" t="n">
+      <c r="A175" s="2" t="n">
         <v>43983</v>
       </c>
       <c r="B175" t="n">
@@ -7095,7 +7107,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="1" t="n">
+      <c r="A176" s="2" t="n">
         <v>44013</v>
       </c>
       <c r="B176" t="n">
@@ -7133,7 +7145,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="1" t="n">
+      <c r="A177" s="2" t="n">
         <v>44044</v>
       </c>
       <c r="B177" t="n">
@@ -7171,7 +7183,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="1" t="n">
+      <c r="A178" s="2" t="n">
         <v>44075</v>
       </c>
       <c r="B178" t="n">
@@ -7209,7 +7221,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="1" t="n">
+      <c r="A179" s="2" t="n">
         <v>44105</v>
       </c>
       <c r="B179" t="n">
@@ -7247,7 +7259,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="1" t="n">
+      <c r="A180" s="2" t="n">
         <v>44136</v>
       </c>
       <c r="B180" t="n">
@@ -7285,7 +7297,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="1" t="n">
+      <c r="A181" s="2" t="n">
         <v>44166</v>
       </c>
       <c r="B181" t="n">
@@ -7323,7 +7335,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="1" t="n">
+      <c r="A182" s="2" t="n">
         <v>44197</v>
       </c>
       <c r="B182" t="n">
@@ -7361,7 +7373,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="1" t="n">
+      <c r="A183" s="2" t="n">
         <v>44228</v>
       </c>
       <c r="B183" t="n">
@@ -7399,7 +7411,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="1" t="n">
+      <c r="A184" s="2" t="n">
         <v>44256</v>
       </c>
       <c r="B184" t="n">
@@ -7437,7 +7449,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="1" t="n">
+      <c r="A185" s="2" t="n">
         <v>44287</v>
       </c>
       <c r="B185" t="n">
@@ -7475,7 +7487,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="1" t="n">
+      <c r="A186" s="2" t="n">
         <v>44317</v>
       </c>
       <c r="B186" t="n">
@@ -7513,7 +7525,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="1" t="n">
+      <c r="A187" s="2" t="n">
         <v>44348</v>
       </c>
       <c r="B187" t="n">
@@ -7551,7 +7563,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="1" t="n">
+      <c r="A188" s="2" t="n">
         <v>44378</v>
       </c>
       <c r="B188" t="n">
@@ -7589,7 +7601,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="1" t="n">
+      <c r="A189" s="2" t="n">
         <v>44409</v>
       </c>
       <c r="B189" t="n">
@@ -7627,7 +7639,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="1" t="n">
+      <c r="A190" s="2" t="n">
         <v>44440</v>
       </c>
       <c r="B190" t="n">
@@ -7665,7 +7677,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="1" t="n">
+      <c r="A191" s="2" t="n">
         <v>44470</v>
       </c>
       <c r="B191" t="n">
@@ -7703,7 +7715,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="1" t="n">
+      <c r="A192" s="2" t="n">
         <v>44501</v>
       </c>
       <c r="B192" t="n">
@@ -7741,7 +7753,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="1" t="n">
+      <c r="A193" s="2" t="n">
         <v>44531</v>
       </c>
       <c r="B193" t="n">
@@ -7779,7 +7791,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="1" t="n">
+      <c r="A194" s="2" t="n">
         <v>44562</v>
       </c>
       <c r="B194" t="n">
@@ -7817,7 +7829,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="1" t="n">
+      <c r="A195" s="2" t="n">
         <v>44593</v>
       </c>
       <c r="B195" t="n">
@@ -7855,7 +7867,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="1" t="n">
+      <c r="A196" s="2" t="n">
         <v>44621</v>
       </c>
       <c r="B196" t="n">
@@ -7893,7 +7905,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="1" t="n">
+      <c r="A197" s="2" t="n">
         <v>44652</v>
       </c>
       <c r="B197" t="n">
@@ -7931,7 +7943,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="1" t="n">
+      <c r="A198" s="2" t="n">
         <v>44682</v>
       </c>
       <c r="B198" t="n">
@@ -7969,7 +7981,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="1" t="n">
+      <c r="A199" s="2" t="n">
         <v>44713</v>
       </c>
       <c r="B199" t="n">
@@ -8007,7 +8019,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="1" t="n">
+      <c r="A200" s="2" t="n">
         <v>44743</v>
       </c>
       <c r="B200" t="n">
@@ -8045,7 +8057,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="1" t="n">
+      <c r="A201" s="2" t="n">
         <v>44774</v>
       </c>
       <c r="B201" t="n">
@@ -8083,7 +8095,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="1" t="n">
+      <c r="A202" s="2" t="n">
         <v>44805</v>
       </c>
       <c r="B202" t="n">
@@ -8121,7 +8133,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="1" t="n">
+      <c r="A203" s="2" t="n">
         <v>44835</v>
       </c>
       <c r="B203" t="n">
@@ -8159,7 +8171,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="1" t="n">
+      <c r="A204" s="2" t="n">
         <v>44866</v>
       </c>
       <c r="B204" t="n">
@@ -8197,7 +8209,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="1" t="n">
+      <c r="A205" s="2" t="n">
         <v>44896</v>
       </c>
       <c r="B205" t="n">
@@ -8235,7 +8247,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="1" t="n">
+      <c r="A206" s="2" t="n">
         <v>44927</v>
       </c>
       <c r="B206" t="n">
@@ -8273,7 +8285,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="1" t="n">
+      <c r="A207" s="2" t="n">
         <v>44958</v>
       </c>
       <c r="B207" t="n">
@@ -8311,7 +8323,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="1" t="n">
+      <c r="A208" s="2" t="n">
         <v>44986</v>
       </c>
       <c r="B208" t="n">
@@ -8349,7 +8361,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="1" t="n">
+      <c r="A209" s="2" t="n">
         <v>45017</v>
       </c>
       <c r="B209" t="n">
@@ -8387,7 +8399,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="1" t="n">
+      <c r="A210" s="2" t="n">
         <v>45047</v>
       </c>
       <c r="B210" t="n">
@@ -8425,7 +8437,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="1" t="n">
+      <c r="A211" s="2" t="n">
         <v>45078</v>
       </c>
       <c r="B211" t="n">
@@ -8463,7 +8475,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="1" t="n">
+      <c r="A212" s="2" t="n">
         <v>45108</v>
       </c>
       <c r="B212" t="n">
@@ -8501,7 +8513,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="1" t="n">
+      <c r="A213" s="2" t="n">
         <v>45139</v>
       </c>
       <c r="B213" t="n">
@@ -8539,7 +8551,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="1" t="n">
+      <c r="A214" s="2" t="n">
         <v>45170</v>
       </c>
       <c r="B214" t="n">
@@ -8577,7 +8589,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="1" t="n">
+      <c r="A215" s="2" t="n">
         <v>45200</v>
       </c>
       <c r="B215" t="n">
@@ -8615,7 +8627,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="1" t="n">
+      <c r="A216" s="2" t="n">
         <v>45231</v>
       </c>
       <c r="B216" t="n">
@@ -8653,7 +8665,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="1" t="n">
+      <c r="A217" s="2" t="n">
         <v>45261</v>
       </c>
       <c r="B217" t="n">
@@ -8691,7 +8703,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="1" t="n">
+      <c r="A218" s="2" t="n">
         <v>45292</v>
       </c>
       <c r="B218" t="n">
@@ -8729,7 +8741,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="1" t="n">
+      <c r="A219" s="2" t="n">
         <v>45323</v>
       </c>
       <c r="B219" t="n">
@@ -8767,7 +8779,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="1" t="n">
+      <c r="A220" s="2" t="n">
         <v>45352</v>
       </c>
       <c r="B220" t="n">
@@ -8805,7 +8817,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="1" t="n">
+      <c r="A221" s="2" t="n">
         <v>45383</v>
       </c>
       <c r="B221" t="n">
@@ -8843,7 +8855,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="1" t="n">
+      <c r="A222" s="2" t="n">
         <v>45413</v>
       </c>
       <c r="B222" t="n">
@@ -8881,7 +8893,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="1" t="n">
+      <c r="A223" s="2" t="n">
         <v>45444</v>
       </c>
       <c r="B223" t="n">
@@ -8919,7 +8931,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="1" t="n">
+      <c r="A224" s="2" t="n">
         <v>45474</v>
       </c>
       <c r="B224" t="n">
@@ -8957,7 +8969,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="1" t="n">
+      <c r="A225" s="2" t="n">
         <v>45505</v>
       </c>
       <c r="B225" t="n">
@@ -8995,7 +9007,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="1" t="n">
+      <c r="A226" s="2" t="n">
         <v>45536</v>
       </c>
       <c r="B226" t="n">
@@ -9033,7 +9045,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="1" t="n">
+      <c r="A227" s="2" t="n">
         <v>45566</v>
       </c>
       <c r="B227" t="n">
@@ -9071,7 +9083,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="1" t="n">
+      <c r="A228" s="2" t="n">
         <v>45597</v>
       </c>
       <c r="B228" t="n">
@@ -9109,7 +9121,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="1" t="n">
+      <c r="A229" s="2" t="n">
         <v>45627</v>
       </c>
       <c r="B229" t="n">
@@ -9147,7 +9159,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="1" t="n">
+      <c r="A230" s="2" t="n">
         <v>45658</v>
       </c>
       <c r="B230" t="n">
@@ -9185,7 +9197,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="1" t="n">
+      <c r="A231" s="2" t="n">
         <v>45689</v>
       </c>
       <c r="B231" t="n">
@@ -9223,7 +9235,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="1" t="n">
+      <c r="A232" s="2" t="n">
         <v>45717</v>
       </c>
       <c r="B232" t="n">
@@ -9261,7 +9273,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="1" t="n">
+      <c r="A233" s="2" t="n">
         <v>45748</v>
       </c>
       <c r="B233" t="n">
@@ -9299,7 +9311,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="1" t="n">
+      <c r="A234" s="2" t="n">
         <v>45778</v>
       </c>
       <c r="B234" t="n">
@@ -9337,7 +9349,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="1" t="n">
+      <c r="A235" s="2" t="n">
         <v>45809</v>
       </c>
       <c r="B235" t="n">
@@ -9375,7 +9387,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="1" t="n">
+      <c r="A236" s="2" t="n">
         <v>45839</v>
       </c>
       <c r="B236" t="n">
@@ -9413,7 +9425,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="1" t="n">
+      <c r="A237" s="2" t="n">
         <v>45870</v>
       </c>
       <c r="B237" t="n">
@@ -9451,7 +9463,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="1" t="n">
+      <c r="A238" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="B238" t="n">
@@ -9489,7 +9501,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="1" t="n">
+      <c r="A239" s="2" t="n">
         <v>45931</v>
       </c>
       <c r="B239" t="n">
@@ -9527,7 +9539,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="1" t="n">
+      <c r="A240" s="2" t="n">
         <v>45962</v>
       </c>
       <c r="B240" t="n">
@@ -9565,7 +9577,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="1" t="n">
+      <c r="A241" s="2" t="n">
         <v>45992</v>
       </c>
       <c r="B241" t="n">
@@ -9603,7 +9615,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="1" t="n">
+      <c r="A242" s="2" t="n">
         <v>46023</v>
       </c>
       <c r="B242" t="n">
@@ -9641,7 +9653,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="1" t="n">
+      <c r="A243" s="2" t="n">
         <v>46054</v>
       </c>
       <c r="B243" t="n">
@@ -9679,7 +9691,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="1" t="n">
+      <c r="A244" s="2" t="n">
         <v>46082</v>
       </c>
       <c r="B244" t="n">
@@ -9717,7 +9729,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="1" t="n">
+      <c r="A245" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="B245" t="n">
@@ -9755,7 +9767,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="1" t="n">
+      <c r="A246" s="2" t="n">
         <v>46143</v>
       </c>
       <c r="B246" t="n">

</xml_diff>

<commit_message>
Otomatik veri güncelleme (17.07.2026 12:49 UTC)
</commit_message>
<xml_diff>
--- a/butce/butce.xlsx
+++ b/butce/butce.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,69 +421,69 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tarih</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>yil</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ay</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>gelir</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>vergi</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>dolaysiz_vergi</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>dolayli_vergi</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>gider</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>faiz_haric_gider</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>faiz_gideri</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>faiz_disi_denge</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>denge</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>38718</v>
       </c>
       <c r="B2" t="n">
@@ -533,7 +521,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>38749</v>
       </c>
       <c r="B3" t="n">
@@ -571,7 +559,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>38777</v>
       </c>
       <c r="B4" t="n">
@@ -609,7 +597,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>38808</v>
       </c>
       <c r="B5" t="n">
@@ -647,7 +635,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>38838</v>
       </c>
       <c r="B6" t="n">
@@ -685,7 +673,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>38869</v>
       </c>
       <c r="B7" t="n">
@@ -723,7 +711,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>38899</v>
       </c>
       <c r="B8" t="n">
@@ -761,7 +749,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>38930</v>
       </c>
       <c r="B9" t="n">
@@ -799,7 +787,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>38961</v>
       </c>
       <c r="B10" t="n">
@@ -837,7 +825,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>38991</v>
       </c>
       <c r="B11" t="n">
@@ -875,7 +863,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>39022</v>
       </c>
       <c r="B12" t="n">
@@ -913,7 +901,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>39052</v>
       </c>
       <c r="B13" t="n">
@@ -951,7 +939,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>39083</v>
       </c>
       <c r="B14" t="n">
@@ -989,7 +977,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>39114</v>
       </c>
       <c r="B15" t="n">
@@ -1027,7 +1015,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>39142</v>
       </c>
       <c r="B16" t="n">
@@ -1065,7 +1053,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>39173</v>
       </c>
       <c r="B17" t="n">
@@ -1103,7 +1091,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>39203</v>
       </c>
       <c r="B18" t="n">
@@ -1141,7 +1129,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>39234</v>
       </c>
       <c r="B19" t="n">
@@ -1179,7 +1167,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>39264</v>
       </c>
       <c r="B20" t="n">
@@ -1217,7 +1205,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>39295</v>
       </c>
       <c r="B21" t="n">
@@ -1255,7 +1243,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>39326</v>
       </c>
       <c r="B22" t="n">
@@ -1293,7 +1281,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>39356</v>
       </c>
       <c r="B23" t="n">
@@ -1331,7 +1319,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>39387</v>
       </c>
       <c r="B24" t="n">
@@ -1369,7 +1357,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>39417</v>
       </c>
       <c r="B25" t="n">
@@ -1407,7 +1395,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>39448</v>
       </c>
       <c r="B26" t="n">
@@ -1445,7 +1433,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="1" t="n">
         <v>39479</v>
       </c>
       <c r="B27" t="n">
@@ -1483,7 +1471,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>39508</v>
       </c>
       <c r="B28" t="n">
@@ -1521,7 +1509,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>39539</v>
       </c>
       <c r="B29" t="n">
@@ -1559,7 +1547,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>39569</v>
       </c>
       <c r="B30" t="n">
@@ -1597,7 +1585,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>39600</v>
       </c>
       <c r="B31" t="n">
@@ -1635,7 +1623,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>39630</v>
       </c>
       <c r="B32" t="n">
@@ -1673,7 +1661,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>39661</v>
       </c>
       <c r="B33" t="n">
@@ -1711,7 +1699,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>39692</v>
       </c>
       <c r="B34" t="n">
@@ -1749,7 +1737,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>39722</v>
       </c>
       <c r="B35" t="n">
@@ -1787,7 +1775,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>39753</v>
       </c>
       <c r="B36" t="n">
@@ -1825,7 +1813,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>39783</v>
       </c>
       <c r="B37" t="n">
@@ -1863,7 +1851,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>39814</v>
       </c>
       <c r="B38" t="n">
@@ -1901,7 +1889,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>39845</v>
       </c>
       <c r="B39" t="n">
@@ -1939,7 +1927,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>39873</v>
       </c>
       <c r="B40" t="n">
@@ -1977,7 +1965,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>39904</v>
       </c>
       <c r="B41" t="n">
@@ -2015,7 +2003,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>39934</v>
       </c>
       <c r="B42" t="n">
@@ -2053,7 +2041,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>39965</v>
       </c>
       <c r="B43" t="n">
@@ -2091,7 +2079,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>39995</v>
       </c>
       <c r="B44" t="n">
@@ -2129,7 +2117,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>40026</v>
       </c>
       <c r="B45" t="n">
@@ -2167,7 +2155,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>40057</v>
       </c>
       <c r="B46" t="n">
@@ -2205,7 +2193,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>40087</v>
       </c>
       <c r="B47" t="n">
@@ -2243,7 +2231,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>40118</v>
       </c>
       <c r="B48" t="n">
@@ -2281,7 +2269,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>40148</v>
       </c>
       <c r="B49" t="n">
@@ -2319,7 +2307,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>40179</v>
       </c>
       <c r="B50" t="n">
@@ -2357,7 +2345,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>40210</v>
       </c>
       <c r="B51" t="n">
@@ -2395,7 +2383,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>40238</v>
       </c>
       <c r="B52" t="n">
@@ -2433,7 +2421,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>40269</v>
       </c>
       <c r="B53" t="n">
@@ -2471,7 +2459,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>40299</v>
       </c>
       <c r="B54" t="n">
@@ -2509,7 +2497,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>40330</v>
       </c>
       <c r="B55" t="n">
@@ -2547,7 +2535,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>40360</v>
       </c>
       <c r="B56" t="n">
@@ -2585,7 +2573,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>40391</v>
       </c>
       <c r="B57" t="n">
@@ -2623,7 +2611,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>40422</v>
       </c>
       <c r="B58" t="n">
@@ -2661,7 +2649,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>40452</v>
       </c>
       <c r="B59" t="n">
@@ -2699,7 +2687,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>40483</v>
       </c>
       <c r="B60" t="n">
@@ -2737,7 +2725,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>40513</v>
       </c>
       <c r="B61" t="n">
@@ -2775,7 +2763,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>40544</v>
       </c>
       <c r="B62" t="n">
@@ -2813,7 +2801,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="1" t="n">
         <v>40575</v>
       </c>
       <c r="B63" t="n">
@@ -2851,7 +2839,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="1" t="n">
         <v>40603</v>
       </c>
       <c r="B64" t="n">
@@ -2889,7 +2877,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="1" t="n">
         <v>40634</v>
       </c>
       <c r="B65" t="n">
@@ -2927,7 +2915,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="1" t="n">
         <v>40664</v>
       </c>
       <c r="B66" t="n">
@@ -2965,7 +2953,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="1" t="n">
         <v>40695</v>
       </c>
       <c r="B67" t="n">
@@ -3003,7 +2991,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="1" t="n">
         <v>40725</v>
       </c>
       <c r="B68" t="n">
@@ -3041,7 +3029,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="1" t="n">
         <v>40756</v>
       </c>
       <c r="B69" t="n">
@@ -3079,7 +3067,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="1" t="n">
         <v>40787</v>
       </c>
       <c r="B70" t="n">
@@ -3117,7 +3105,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="1" t="n">
         <v>40817</v>
       </c>
       <c r="B71" t="n">
@@ -3155,7 +3143,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="1" t="n">
         <v>40848</v>
       </c>
       <c r="B72" t="n">
@@ -3193,7 +3181,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="1" t="n">
         <v>40878</v>
       </c>
       <c r="B73" t="n">
@@ -3231,7 +3219,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="1" t="n">
         <v>40909</v>
       </c>
       <c r="B74" t="n">
@@ -3269,7 +3257,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="1" t="n">
         <v>40940</v>
       </c>
       <c r="B75" t="n">
@@ -3307,7 +3295,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="1" t="n">
         <v>40969</v>
       </c>
       <c r="B76" t="n">
@@ -3345,7 +3333,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="1" t="n">
         <v>41000</v>
       </c>
       <c r="B77" t="n">
@@ -3383,7 +3371,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="1" t="n">
         <v>41030</v>
       </c>
       <c r="B78" t="n">
@@ -3421,7 +3409,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="1" t="n">
         <v>41061</v>
       </c>
       <c r="B79" t="n">
@@ -3459,7 +3447,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="1" t="n">
         <v>41091</v>
       </c>
       <c r="B80" t="n">
@@ -3497,7 +3485,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="1" t="n">
         <v>41122</v>
       </c>
       <c r="B81" t="n">
@@ -3535,7 +3523,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="1" t="n">
         <v>41153</v>
       </c>
       <c r="B82" t="n">
@@ -3573,7 +3561,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="1" t="n">
         <v>41183</v>
       </c>
       <c r="B83" t="n">
@@ -3611,7 +3599,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="1" t="n">
         <v>41214</v>
       </c>
       <c r="B84" t="n">
@@ -3649,7 +3637,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="1" t="n">
         <v>41244</v>
       </c>
       <c r="B85" t="n">
@@ -3687,7 +3675,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="1" t="n">
         <v>41275</v>
       </c>
       <c r="B86" t="n">
@@ -3725,7 +3713,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="1" t="n">
         <v>41306</v>
       </c>
       <c r="B87" t="n">
@@ -3763,7 +3751,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="1" t="n">
         <v>41334</v>
       </c>
       <c r="B88" t="n">
@@ -3801,7 +3789,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="1" t="n">
         <v>41365</v>
       </c>
       <c r="B89" t="n">
@@ -3839,7 +3827,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="1" t="n">
         <v>41395</v>
       </c>
       <c r="B90" t="n">
@@ -3877,7 +3865,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="1" t="n">
         <v>41426</v>
       </c>
       <c r="B91" t="n">
@@ -3915,7 +3903,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="1" t="n">
         <v>41456</v>
       </c>
       <c r="B92" t="n">
@@ -3953,7 +3941,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="1" t="n">
         <v>41487</v>
       </c>
       <c r="B93" t="n">
@@ -3991,7 +3979,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="1" t="n">
         <v>41518</v>
       </c>
       <c r="B94" t="n">
@@ -4029,7 +4017,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" s="1" t="n">
         <v>41548</v>
       </c>
       <c r="B95" t="n">
@@ -4067,7 +4055,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="1" t="n">
         <v>41579</v>
       </c>
       <c r="B96" t="n">
@@ -4105,7 +4093,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="1" t="n">
         <v>41609</v>
       </c>
       <c r="B97" t="n">
@@ -4143,7 +4131,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="1" t="n">
         <v>41640</v>
       </c>
       <c r="B98" t="n">
@@ -4181,7 +4169,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="1" t="n">
         <v>41671</v>
       </c>
       <c r="B99" t="n">
@@ -4219,7 +4207,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="1" t="n">
         <v>41699</v>
       </c>
       <c r="B100" t="n">
@@ -4257,7 +4245,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="1" t="n">
         <v>41730</v>
       </c>
       <c r="B101" t="n">
@@ -4295,7 +4283,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="1" t="n">
         <v>41760</v>
       </c>
       <c r="B102" t="n">
@@ -4333,7 +4321,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="1" t="n">
         <v>41791</v>
       </c>
       <c r="B103" t="n">
@@ -4371,7 +4359,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="1" t="n">
         <v>41821</v>
       </c>
       <c r="B104" t="n">
@@ -4409,7 +4397,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="1" t="n">
         <v>41852</v>
       </c>
       <c r="B105" t="n">
@@ -4447,7 +4435,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="1" t="n">
         <v>41883</v>
       </c>
       <c r="B106" t="n">
@@ -4485,7 +4473,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="1" t="n">
         <v>41913</v>
       </c>
       <c r="B107" t="n">
@@ -4523,7 +4511,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="1" t="n">
         <v>41944</v>
       </c>
       <c r="B108" t="n">
@@ -4561,7 +4549,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
+      <c r="A109" s="1" t="n">
         <v>41974</v>
       </c>
       <c r="B109" t="n">
@@ -4599,7 +4587,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
+      <c r="A110" s="1" t="n">
         <v>42005</v>
       </c>
       <c r="B110" t="n">
@@ -4637,7 +4625,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="1" t="n">
         <v>42036</v>
       </c>
       <c r="B111" t="n">
@@ -4675,7 +4663,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="1" t="n">
         <v>42064</v>
       </c>
       <c r="B112" t="n">
@@ -4713,7 +4701,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="1" t="n">
         <v>42095</v>
       </c>
       <c r="B113" t="n">
@@ -4751,7 +4739,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="1" t="n">
         <v>42125</v>
       </c>
       <c r="B114" t="n">
@@ -4789,7 +4777,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="1" t="n">
         <v>42156</v>
       </c>
       <c r="B115" t="n">
@@ -4827,7 +4815,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
+      <c r="A116" s="1" t="n">
         <v>42186</v>
       </c>
       <c r="B116" t="n">
@@ -4865,7 +4853,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
+      <c r="A117" s="1" t="n">
         <v>42217</v>
       </c>
       <c r="B117" t="n">
@@ -4903,7 +4891,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
+      <c r="A118" s="1" t="n">
         <v>42248</v>
       </c>
       <c r="B118" t="n">
@@ -4941,7 +4929,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
+      <c r="A119" s="1" t="n">
         <v>42278</v>
       </c>
       <c r="B119" t="n">
@@ -4979,7 +4967,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
+      <c r="A120" s="1" t="n">
         <v>42309</v>
       </c>
       <c r="B120" t="n">
@@ -5017,7 +5005,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
+      <c r="A121" s="1" t="n">
         <v>42339</v>
       </c>
       <c r="B121" t="n">
@@ -5055,7 +5043,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
+      <c r="A122" s="1" t="n">
         <v>42370</v>
       </c>
       <c r="B122" t="n">
@@ -5093,7 +5081,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
+      <c r="A123" s="1" t="n">
         <v>42401</v>
       </c>
       <c r="B123" t="n">
@@ -5131,7 +5119,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
+      <c r="A124" s="1" t="n">
         <v>42430</v>
       </c>
       <c r="B124" t="n">
@@ -5169,7 +5157,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
+      <c r="A125" s="1" t="n">
         <v>42461</v>
       </c>
       <c r="B125" t="n">
@@ -5207,7 +5195,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" s="1" t="n">
         <v>42491</v>
       </c>
       <c r="B126" t="n">
@@ -5245,7 +5233,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
+      <c r="A127" s="1" t="n">
         <v>42522</v>
       </c>
       <c r="B127" t="n">
@@ -5283,7 +5271,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
+      <c r="A128" s="1" t="n">
         <v>42552</v>
       </c>
       <c r="B128" t="n">
@@ -5321,7 +5309,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
+      <c r="A129" s="1" t="n">
         <v>42583</v>
       </c>
       <c r="B129" t="n">
@@ -5359,7 +5347,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
+      <c r="A130" s="1" t="n">
         <v>42614</v>
       </c>
       <c r="B130" t="n">
@@ -5397,7 +5385,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
+      <c r="A131" s="1" t="n">
         <v>42644</v>
       </c>
       <c r="B131" t="n">
@@ -5435,7 +5423,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" s="1" t="n">
         <v>42675</v>
       </c>
       <c r="B132" t="n">
@@ -5473,7 +5461,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" s="1" t="n">
         <v>42705</v>
       </c>
       <c r="B133" t="n">
@@ -5511,7 +5499,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
+      <c r="A134" s="1" t="n">
         <v>42736</v>
       </c>
       <c r="B134" t="n">
@@ -5549,7 +5537,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
+      <c r="A135" s="1" t="n">
         <v>42767</v>
       </c>
       <c r="B135" t="n">
@@ -5587,7 +5575,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="1" t="n">
         <v>42795</v>
       </c>
       <c r="B136" t="n">
@@ -5625,7 +5613,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
+      <c r="A137" s="1" t="n">
         <v>42826</v>
       </c>
       <c r="B137" t="n">
@@ -5663,7 +5651,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
+      <c r="A138" s="1" t="n">
         <v>42856</v>
       </c>
       <c r="B138" t="n">
@@ -5701,7 +5689,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
+      <c r="A139" s="1" t="n">
         <v>42887</v>
       </c>
       <c r="B139" t="n">
@@ -5739,7 +5727,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
+      <c r="A140" s="1" t="n">
         <v>42917</v>
       </c>
       <c r="B140" t="n">
@@ -5777,7 +5765,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
+      <c r="A141" s="1" t="n">
         <v>42948</v>
       </c>
       <c r="B141" t="n">
@@ -5815,7 +5803,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
+      <c r="A142" s="1" t="n">
         <v>42979</v>
       </c>
       <c r="B142" t="n">
@@ -5853,7 +5841,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
+      <c r="A143" s="1" t="n">
         <v>43009</v>
       </c>
       <c r="B143" t="n">
@@ -5891,7 +5879,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
+      <c r="A144" s="1" t="n">
         <v>43040</v>
       </c>
       <c r="B144" t="n">
@@ -5929,7 +5917,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
+      <c r="A145" s="1" t="n">
         <v>43070</v>
       </c>
       <c r="B145" t="n">
@@ -5967,7 +5955,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n">
+      <c r="A146" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="B146" t="n">
@@ -6005,7 +5993,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
+      <c r="A147" s="1" t="n">
         <v>43132</v>
       </c>
       <c r="B147" t="n">
@@ -6043,7 +6031,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
+      <c r="A148" s="1" t="n">
         <v>43160</v>
       </c>
       <c r="B148" t="n">
@@ -6081,7 +6069,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
+      <c r="A149" s="1" t="n">
         <v>43191</v>
       </c>
       <c r="B149" t="n">
@@ -6119,7 +6107,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
+      <c r="A150" s="1" t="n">
         <v>43221</v>
       </c>
       <c r="B150" t="n">
@@ -6157,7 +6145,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n">
+      <c r="A151" s="1" t="n">
         <v>43252</v>
       </c>
       <c r="B151" t="n">
@@ -6195,7 +6183,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n">
+      <c r="A152" s="1" t="n">
         <v>43282</v>
       </c>
       <c r="B152" t="n">
@@ -6233,7 +6221,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
+      <c r="A153" s="1" t="n">
         <v>43313</v>
       </c>
       <c r="B153" t="n">
@@ -6271,7 +6259,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
+      <c r="A154" s="1" t="n">
         <v>43344</v>
       </c>
       <c r="B154" t="n">
@@ -6309,7 +6297,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n">
+      <c r="A155" s="1" t="n">
         <v>43374</v>
       </c>
       <c r="B155" t="n">
@@ -6347,7 +6335,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
+      <c r="A156" s="1" t="n">
         <v>43405</v>
       </c>
       <c r="B156" t="n">
@@ -6385,7 +6373,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n">
+      <c r="A157" s="1" t="n">
         <v>43435</v>
       </c>
       <c r="B157" t="n">
@@ -6423,7 +6411,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n">
+      <c r="A158" s="1" t="n">
         <v>43466</v>
       </c>
       <c r="B158" t="n">
@@ -6461,7 +6449,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n">
+      <c r="A159" s="1" t="n">
         <v>43497</v>
       </c>
       <c r="B159" t="n">
@@ -6499,7 +6487,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
+      <c r="A160" s="1" t="n">
         <v>43525</v>
       </c>
       <c r="B160" t="n">
@@ -6537,7 +6525,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
+      <c r="A161" s="1" t="n">
         <v>43556</v>
       </c>
       <c r="B161" t="n">
@@ -6575,7 +6563,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
+      <c r="A162" s="1" t="n">
         <v>43586</v>
       </c>
       <c r="B162" t="n">
@@ -6613,7 +6601,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
+      <c r="A163" s="1" t="n">
         <v>43617</v>
       </c>
       <c r="B163" t="n">
@@ -6651,7 +6639,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
+      <c r="A164" s="1" t="n">
         <v>43647</v>
       </c>
       <c r="B164" t="n">
@@ -6689,7 +6677,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n">
+      <c r="A165" s="1" t="n">
         <v>43678</v>
       </c>
       <c r="B165" t="n">
@@ -6727,7 +6715,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n">
+      <c r="A166" s="1" t="n">
         <v>43709</v>
       </c>
       <c r="B166" t="n">
@@ -6765,7 +6753,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
+      <c r="A167" s="1" t="n">
         <v>43739</v>
       </c>
       <c r="B167" t="n">
@@ -6803,7 +6791,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
+      <c r="A168" s="1" t="n">
         <v>43770</v>
       </c>
       <c r="B168" t="n">
@@ -6841,7 +6829,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
+      <c r="A169" s="1" t="n">
         <v>43800</v>
       </c>
       <c r="B169" t="n">
@@ -6879,7 +6867,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n">
+      <c r="A170" s="1" t="n">
         <v>43831</v>
       </c>
       <c r="B170" t="n">
@@ -6917,7 +6905,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
+      <c r="A171" s="1" t="n">
         <v>43862</v>
       </c>
       <c r="B171" t="n">
@@ -6955,7 +6943,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n">
+      <c r="A172" s="1" t="n">
         <v>43891</v>
       </c>
       <c r="B172" t="n">
@@ -6993,7 +6981,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n">
+      <c r="A173" s="1" t="n">
         <v>43922</v>
       </c>
       <c r="B173" t="n">
@@ -7031,7 +7019,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
+      <c r="A174" s="1" t="n">
         <v>43952</v>
       </c>
       <c r="B174" t="n">
@@ -7069,7 +7057,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
+      <c r="A175" s="1" t="n">
         <v>43983</v>
       </c>
       <c r="B175" t="n">
@@ -7107,7 +7095,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
+      <c r="A176" s="1" t="n">
         <v>44013</v>
       </c>
       <c r="B176" t="n">
@@ -7145,7 +7133,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
+      <c r="A177" s="1" t="n">
         <v>44044</v>
       </c>
       <c r="B177" t="n">
@@ -7183,7 +7171,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
+      <c r="A178" s="1" t="n">
         <v>44075</v>
       </c>
       <c r="B178" t="n">
@@ -7221,7 +7209,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n">
+      <c r="A179" s="1" t="n">
         <v>44105</v>
       </c>
       <c r="B179" t="n">
@@ -7259,7 +7247,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n">
+      <c r="A180" s="1" t="n">
         <v>44136</v>
       </c>
       <c r="B180" t="n">
@@ -7297,7 +7285,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
+      <c r="A181" s="1" t="n">
         <v>44166</v>
       </c>
       <c r="B181" t="n">
@@ -7335,7 +7323,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
+      <c r="A182" s="1" t="n">
         <v>44197</v>
       </c>
       <c r="B182" t="n">
@@ -7373,7 +7361,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
+      <c r="A183" s="1" t="n">
         <v>44228</v>
       </c>
       <c r="B183" t="n">
@@ -7411,7 +7399,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n">
+      <c r="A184" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="B184" t="n">
@@ -7449,7 +7437,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n">
+      <c r="A185" s="1" t="n">
         <v>44287</v>
       </c>
       <c r="B185" t="n">
@@ -7487,7 +7475,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n">
+      <c r="A186" s="1" t="n">
         <v>44317</v>
       </c>
       <c r="B186" t="n">
@@ -7525,7 +7513,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n">
+      <c r="A187" s="1" t="n">
         <v>44348</v>
       </c>
       <c r="B187" t="n">
@@ -7563,7 +7551,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n">
+      <c r="A188" s="1" t="n">
         <v>44378</v>
       </c>
       <c r="B188" t="n">
@@ -7601,7 +7589,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n">
+      <c r="A189" s="1" t="n">
         <v>44409</v>
       </c>
       <c r="B189" t="n">
@@ -7639,7 +7627,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n">
+      <c r="A190" s="1" t="n">
         <v>44440</v>
       </c>
       <c r="B190" t="n">
@@ -7677,7 +7665,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="n">
+      <c r="A191" s="1" t="n">
         <v>44470</v>
       </c>
       <c r="B191" t="n">
@@ -7715,7 +7703,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n">
+      <c r="A192" s="1" t="n">
         <v>44501</v>
       </c>
       <c r="B192" t="n">
@@ -7753,7 +7741,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="n">
+      <c r="A193" s="1" t="n">
         <v>44531</v>
       </c>
       <c r="B193" t="n">
@@ -7791,7 +7779,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="n">
+      <c r="A194" s="1" t="n">
         <v>44562</v>
       </c>
       <c r="B194" t="n">
@@ -7829,7 +7817,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="n">
+      <c r="A195" s="1" t="n">
         <v>44593</v>
       </c>
       <c r="B195" t="n">
@@ -7867,7 +7855,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="n">
+      <c r="A196" s="1" t="n">
         <v>44621</v>
       </c>
       <c r="B196" t="n">
@@ -7905,7 +7893,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="n">
+      <c r="A197" s="1" t="n">
         <v>44652</v>
       </c>
       <c r="B197" t="n">
@@ -7943,7 +7931,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n">
+      <c r="A198" s="1" t="n">
         <v>44682</v>
       </c>
       <c r="B198" t="n">
@@ -7981,7 +7969,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="n">
+      <c r="A199" s="1" t="n">
         <v>44713</v>
       </c>
       <c r="B199" t="n">
@@ -8019,7 +8007,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n">
+      <c r="A200" s="1" t="n">
         <v>44743</v>
       </c>
       <c r="B200" t="n">
@@ -8057,7 +8045,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="n">
+      <c r="A201" s="1" t="n">
         <v>44774</v>
       </c>
       <c r="B201" t="n">
@@ -8095,7 +8083,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="n">
+      <c r="A202" s="1" t="n">
         <v>44805</v>
       </c>
       <c r="B202" t="n">
@@ -8133,7 +8121,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="n">
+      <c r="A203" s="1" t="n">
         <v>44835</v>
       </c>
       <c r="B203" t="n">
@@ -8171,7 +8159,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="n">
+      <c r="A204" s="1" t="n">
         <v>44866</v>
       </c>
       <c r="B204" t="n">
@@ -8209,7 +8197,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="n">
+      <c r="A205" s="1" t="n">
         <v>44896</v>
       </c>
       <c r="B205" t="n">
@@ -8247,7 +8235,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="n">
+      <c r="A206" s="1" t="n">
         <v>44927</v>
       </c>
       <c r="B206" t="n">
@@ -8285,7 +8273,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="n">
+      <c r="A207" s="1" t="n">
         <v>44958</v>
       </c>
       <c r="B207" t="n">
@@ -8323,7 +8311,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="n">
+      <c r="A208" s="1" t="n">
         <v>44986</v>
       </c>
       <c r="B208" t="n">
@@ -8361,7 +8349,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="n">
+      <c r="A209" s="1" t="n">
         <v>45017</v>
       </c>
       <c r="B209" t="n">
@@ -8399,7 +8387,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n">
+      <c r="A210" s="1" t="n">
         <v>45047</v>
       </c>
       <c r="B210" t="n">
@@ -8437,7 +8425,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="2" t="n">
+      <c r="A211" s="1" t="n">
         <v>45078</v>
       </c>
       <c r="B211" t="n">
@@ -8475,7 +8463,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="n">
+      <c r="A212" s="1" t="n">
         <v>45108</v>
       </c>
       <c r="B212" t="n">
@@ -8513,7 +8501,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="n">
+      <c r="A213" s="1" t="n">
         <v>45139</v>
       </c>
       <c r="B213" t="n">
@@ -8551,7 +8539,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="n">
+      <c r="A214" s="1" t="n">
         <v>45170</v>
       </c>
       <c r="B214" t="n">
@@ -8589,7 +8577,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="2" t="n">
+      <c r="A215" s="1" t="n">
         <v>45200</v>
       </c>
       <c r="B215" t="n">
@@ -8627,7 +8615,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="2" t="n">
+      <c r="A216" s="1" t="n">
         <v>45231</v>
       </c>
       <c r="B216" t="n">
@@ -8665,7 +8653,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="n">
+      <c r="A217" s="1" t="n">
         <v>45261</v>
       </c>
       <c r="B217" t="n">
@@ -8703,7 +8691,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="n">
+      <c r="A218" s="1" t="n">
         <v>45292</v>
       </c>
       <c r="B218" t="n">
@@ -8741,7 +8729,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="n">
+      <c r="A219" s="1" t="n">
         <v>45323</v>
       </c>
       <c r="B219" t="n">
@@ -8779,7 +8767,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="n">
+      <c r="A220" s="1" t="n">
         <v>45352</v>
       </c>
       <c r="B220" t="n">
@@ -8817,7 +8805,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="n">
+      <c r="A221" s="1" t="n">
         <v>45383</v>
       </c>
       <c r="B221" t="n">
@@ -8855,7 +8843,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="n">
+      <c r="A222" s="1" t="n">
         <v>45413</v>
       </c>
       <c r="B222" t="n">
@@ -8893,7 +8881,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="n">
+      <c r="A223" s="1" t="n">
         <v>45444</v>
       </c>
       <c r="B223" t="n">
@@ -8931,7 +8919,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="n">
+      <c r="A224" s="1" t="n">
         <v>45474</v>
       </c>
       <c r="B224" t="n">
@@ -8969,7 +8957,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="n">
+      <c r="A225" s="1" t="n">
         <v>45505</v>
       </c>
       <c r="B225" t="n">
@@ -9007,7 +8995,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="n">
+      <c r="A226" s="1" t="n">
         <v>45536</v>
       </c>
       <c r="B226" t="n">
@@ -9045,7 +9033,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="n">
+      <c r="A227" s="1" t="n">
         <v>45566</v>
       </c>
       <c r="B227" t="n">
@@ -9083,7 +9071,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="n">
+      <c r="A228" s="1" t="n">
         <v>45597</v>
       </c>
       <c r="B228" t="n">
@@ -9121,7 +9109,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="n">
+      <c r="A229" s="1" t="n">
         <v>45627</v>
       </c>
       <c r="B229" t="n">
@@ -9159,7 +9147,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="n">
+      <c r="A230" s="1" t="n">
         <v>45658</v>
       </c>
       <c r="B230" t="n">
@@ -9197,7 +9185,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="n">
+      <c r="A231" s="1" t="n">
         <v>45689</v>
       </c>
       <c r="B231" t="n">
@@ -9235,7 +9223,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="n">
+      <c r="A232" s="1" t="n">
         <v>45717</v>
       </c>
       <c r="B232" t="n">
@@ -9273,7 +9261,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="n">
+      <c r="A233" s="1" t="n">
         <v>45748</v>
       </c>
       <c r="B233" t="n">
@@ -9311,7 +9299,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="n">
+      <c r="A234" s="1" t="n">
         <v>45778</v>
       </c>
       <c r="B234" t="n">
@@ -9349,7 +9337,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="n">
+      <c r="A235" s="1" t="n">
         <v>45809</v>
       </c>
       <c r="B235" t="n">
@@ -9387,7 +9375,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="2" t="n">
+      <c r="A236" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="B236" t="n">
@@ -9425,7 +9413,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="2" t="n">
+      <c r="A237" s="1" t="n">
         <v>45870</v>
       </c>
       <c r="B237" t="n">
@@ -9463,7 +9451,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="2" t="n">
+      <c r="A238" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="B238" t="n">
@@ -9501,7 +9489,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="2" t="n">
+      <c r="A239" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="B239" t="n">
@@ -9539,7 +9527,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="2" t="n">
+      <c r="A240" s="1" t="n">
         <v>45962</v>
       </c>
       <c r="B240" t="n">
@@ -9577,7 +9565,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="2" t="n">
+      <c r="A241" s="1" t="n">
         <v>45992</v>
       </c>
       <c r="B241" t="n">
@@ -9615,7 +9603,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="2" t="n">
+      <c r="A242" s="1" t="n">
         <v>46023</v>
       </c>
       <c r="B242" t="n">
@@ -9653,7 +9641,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="n">
+      <c r="A243" s="1" t="n">
         <v>46054</v>
       </c>
       <c r="B243" t="n">
@@ -9691,7 +9679,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="2" t="n">
+      <c r="A244" s="1" t="n">
         <v>46082</v>
       </c>
       <c r="B244" t="n">
@@ -9729,7 +9717,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="2" t="n">
+      <c r="A245" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="B245" t="n">
@@ -9767,7 +9755,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="2" t="n">
+      <c r="A246" s="1" t="n">
         <v>46143</v>
       </c>
       <c r="B246" t="n">

</xml_diff>

<commit_message>
Otomatik veri güncelleme (23.07.2026 13:14 UTC)
</commit_message>
<xml_diff>
--- a/butce/butce.xlsx
+++ b/butce/butce.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L246"/>
+  <dimension ref="A1:L247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9792,6 +9792,44 @@
         <v>-298222.8126177003</v>
       </c>
     </row>
+    <row r="247">
+      <c r="A247" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B247" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C247" t="n">
+        <v>6</v>
+      </c>
+      <c r="D247" t="n">
+        <v>1509630.375028101</v>
+      </c>
+      <c r="E247" t="n">
+        <v>1315662.34503416</v>
+      </c>
+      <c r="F247" t="n">
+        <v>527477.4564320402</v>
+      </c>
+      <c r="G247" t="n">
+        <v>788184.8886021201</v>
+      </c>
+      <c r="H247" t="n">
+        <v>1395466.82655272</v>
+      </c>
+      <c r="I247" t="n">
+        <v>1193859.94901229</v>
+      </c>
+      <c r="J247" t="n">
+        <v>201606.8775404299</v>
+      </c>
+      <c r="K247" t="n">
+        <v>315770.4260158106</v>
+      </c>
+      <c r="L247" t="n">
+        <v>114163.5484753808</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Toplu veri güncelleme + BDDK (yerel, 14.08.2026)
14 modül EVDS/HMB'den yenilendi; BDDK 07.08 kesim haftası (sabah
koşusunun senkron çakışması bulut tabanına yeniden oturtularak çözüldü).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/butce/butce.xlsx
+++ b/butce/butce.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,69 +433,69 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>tarih</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>yil</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ay</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>gelir</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>vergi</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>dolaysiz_vergi</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>dolayli_vergi</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>gider</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>faiz_haric_gider</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>faiz_gideri</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>faiz_disi_denge</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>denge</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>38718</v>
       </c>
       <c r="B2" t="n">
@@ -521,7 +533,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>38749</v>
       </c>
       <c r="B3" t="n">
@@ -559,7 +571,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>38777</v>
       </c>
       <c r="B4" t="n">
@@ -597,7 +609,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>38808</v>
       </c>
       <c r="B5" t="n">
@@ -635,7 +647,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>38838</v>
       </c>
       <c r="B6" t="n">
@@ -673,7 +685,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>38869</v>
       </c>
       <c r="B7" t="n">
@@ -711,7 +723,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>38899</v>
       </c>
       <c r="B8" t="n">
@@ -749,7 +761,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>38930</v>
       </c>
       <c r="B9" t="n">
@@ -787,7 +799,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>38961</v>
       </c>
       <c r="B10" t="n">
@@ -825,7 +837,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>38991</v>
       </c>
       <c r="B11" t="n">
@@ -863,7 +875,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>39022</v>
       </c>
       <c r="B12" t="n">
@@ -901,7 +913,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>39052</v>
       </c>
       <c r="B13" t="n">
@@ -939,7 +951,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>39083</v>
       </c>
       <c r="B14" t="n">
@@ -977,7 +989,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>39114</v>
       </c>
       <c r="B15" t="n">
@@ -1015,7 +1027,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>39142</v>
       </c>
       <c r="B16" t="n">
@@ -1053,7 +1065,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>39173</v>
       </c>
       <c r="B17" t="n">
@@ -1091,7 +1103,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>39203</v>
       </c>
       <c r="B18" t="n">
@@ -1129,7 +1141,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>39234</v>
       </c>
       <c r="B19" t="n">
@@ -1167,7 +1179,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>39264</v>
       </c>
       <c r="B20" t="n">
@@ -1205,7 +1217,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>39295</v>
       </c>
       <c r="B21" t="n">
@@ -1243,7 +1255,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>39326</v>
       </c>
       <c r="B22" t="n">
@@ -1281,7 +1293,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>39356</v>
       </c>
       <c r="B23" t="n">
@@ -1319,7 +1331,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>39387</v>
       </c>
       <c r="B24" t="n">
@@ -1357,7 +1369,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>39417</v>
       </c>
       <c r="B25" t="n">
@@ -1395,7 +1407,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>39448</v>
       </c>
       <c r="B26" t="n">
@@ -1433,7 +1445,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>39479</v>
       </c>
       <c r="B27" t="n">
@@ -1471,7 +1483,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>39508</v>
       </c>
       <c r="B28" t="n">
@@ -1509,7 +1521,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>39539</v>
       </c>
       <c r="B29" t="n">
@@ -1547,7 +1559,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>39569</v>
       </c>
       <c r="B30" t="n">
@@ -1585,7 +1597,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>39600</v>
       </c>
       <c r="B31" t="n">
@@ -1623,7 +1635,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>39630</v>
       </c>
       <c r="B32" t="n">
@@ -1661,7 +1673,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>39661</v>
       </c>
       <c r="B33" t="n">
@@ -1699,7 +1711,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>39692</v>
       </c>
       <c r="B34" t="n">
@@ -1737,7 +1749,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>39722</v>
       </c>
       <c r="B35" t="n">
@@ -1775,7 +1787,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>39753</v>
       </c>
       <c r="B36" t="n">
@@ -1813,7 +1825,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>39783</v>
       </c>
       <c r="B37" t="n">
@@ -1851,7 +1863,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>39814</v>
       </c>
       <c r="B38" t="n">
@@ -1889,7 +1901,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>39845</v>
       </c>
       <c r="B39" t="n">
@@ -1927,7 +1939,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>39873</v>
       </c>
       <c r="B40" t="n">
@@ -1965,7 +1977,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>39904</v>
       </c>
       <c r="B41" t="n">
@@ -2003,7 +2015,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>39934</v>
       </c>
       <c r="B42" t="n">
@@ -2041,7 +2053,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>39965</v>
       </c>
       <c r="B43" t="n">
@@ -2079,7 +2091,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>39995</v>
       </c>
       <c r="B44" t="n">
@@ -2117,7 +2129,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>40026</v>
       </c>
       <c r="B45" t="n">
@@ -2155,7 +2167,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>40057</v>
       </c>
       <c r="B46" t="n">
@@ -2193,7 +2205,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>40087</v>
       </c>
       <c r="B47" t="n">
@@ -2231,7 +2243,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>40118</v>
       </c>
       <c r="B48" t="n">
@@ -2269,7 +2281,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>40148</v>
       </c>
       <c r="B49" t="n">
@@ -2307,7 +2319,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>40179</v>
       </c>
       <c r="B50" t="n">
@@ -2345,7 +2357,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>40210</v>
       </c>
       <c r="B51" t="n">
@@ -2383,7 +2395,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>40238</v>
       </c>
       <c r="B52" t="n">
@@ -2421,7 +2433,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>40269</v>
       </c>
       <c r="B53" t="n">
@@ -2459,7 +2471,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>40299</v>
       </c>
       <c r="B54" t="n">
@@ -2497,7 +2509,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>40330</v>
       </c>
       <c r="B55" t="n">
@@ -2535,7 +2547,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>40360</v>
       </c>
       <c r="B56" t="n">
@@ -2573,7 +2585,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>40391</v>
       </c>
       <c r="B57" t="n">
@@ -2611,7 +2623,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>40422</v>
       </c>
       <c r="B58" t="n">
@@ -2649,7 +2661,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>40452</v>
       </c>
       <c r="B59" t="n">
@@ -2687,7 +2699,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>40483</v>
       </c>
       <c r="B60" t="n">
@@ -2725,7 +2737,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>40513</v>
       </c>
       <c r="B61" t="n">
@@ -2763,7 +2775,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>40544</v>
       </c>
       <c r="B62" t="n">
@@ -2801,7 +2813,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" s="2" t="n">
         <v>40575</v>
       </c>
       <c r="B63" t="n">
@@ -2839,7 +2851,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" s="2" t="n">
         <v>40603</v>
       </c>
       <c r="B64" t="n">
@@ -2877,7 +2889,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" s="2" t="n">
         <v>40634</v>
       </c>
       <c r="B65" t="n">
@@ -2915,7 +2927,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="2" t="n">
         <v>40664</v>
       </c>
       <c r="B66" t="n">
@@ -2953,7 +2965,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="2" t="n">
         <v>40695</v>
       </c>
       <c r="B67" t="n">
@@ -2991,7 +3003,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="2" t="n">
         <v>40725</v>
       </c>
       <c r="B68" t="n">
@@ -3029,7 +3041,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="2" t="n">
         <v>40756</v>
       </c>
       <c r="B69" t="n">
@@ -3067,7 +3079,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="2" t="n">
         <v>40787</v>
       </c>
       <c r="B70" t="n">
@@ -3105,7 +3117,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="2" t="n">
         <v>40817</v>
       </c>
       <c r="B71" t="n">
@@ -3143,7 +3155,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" s="2" t="n">
         <v>40848</v>
       </c>
       <c r="B72" t="n">
@@ -3181,7 +3193,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="2" t="n">
         <v>40878</v>
       </c>
       <c r="B73" t="n">
@@ -3219,7 +3231,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="2" t="n">
         <v>40909</v>
       </c>
       <c r="B74" t="n">
@@ -3257,7 +3269,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="2" t="n">
         <v>40940</v>
       </c>
       <c r="B75" t="n">
@@ -3295,7 +3307,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="2" t="n">
         <v>40969</v>
       </c>
       <c r="B76" t="n">
@@ -3333,7 +3345,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="2" t="n">
         <v>41000</v>
       </c>
       <c r="B77" t="n">
@@ -3371,7 +3383,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="2" t="n">
         <v>41030</v>
       </c>
       <c r="B78" t="n">
@@ -3409,7 +3421,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="2" t="n">
         <v>41061</v>
       </c>
       <c r="B79" t="n">
@@ -3447,7 +3459,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="2" t="n">
         <v>41091</v>
       </c>
       <c r="B80" t="n">
@@ -3485,7 +3497,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" s="2" t="n">
         <v>41122</v>
       </c>
       <c r="B81" t="n">
@@ -3523,7 +3535,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" s="2" t="n">
         <v>41153</v>
       </c>
       <c r="B82" t="n">
@@ -3561,7 +3573,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="2" t="n">
         <v>41183</v>
       </c>
       <c r="B83" t="n">
@@ -3599,7 +3611,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="2" t="n">
         <v>41214</v>
       </c>
       <c r="B84" t="n">
@@ -3637,7 +3649,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" s="2" t="n">
         <v>41244</v>
       </c>
       <c r="B85" t="n">
@@ -3675,7 +3687,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" s="2" t="n">
         <v>41275</v>
       </c>
       <c r="B86" t="n">
@@ -3713,7 +3725,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="2" t="n">
         <v>41306</v>
       </c>
       <c r="B87" t="n">
@@ -3751,7 +3763,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="2" t="n">
         <v>41334</v>
       </c>
       <c r="B88" t="n">
@@ -3789,7 +3801,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="2" t="n">
         <v>41365</v>
       </c>
       <c r="B89" t="n">
@@ -3827,7 +3839,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="2" t="n">
         <v>41395</v>
       </c>
       <c r="B90" t="n">
@@ -3865,7 +3877,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="2" t="n">
         <v>41426</v>
       </c>
       <c r="B91" t="n">
@@ -3903,7 +3915,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="2" t="n">
         <v>41456</v>
       </c>
       <c r="B92" t="n">
@@ -3941,7 +3953,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" s="2" t="n">
         <v>41487</v>
       </c>
       <c r="B93" t="n">
@@ -3979,7 +3991,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" s="2" t="n">
         <v>41518</v>
       </c>
       <c r="B94" t="n">
@@ -4017,7 +4029,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" s="2" t="n">
         <v>41548</v>
       </c>
       <c r="B95" t="n">
@@ -4055,7 +4067,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" s="2" t="n">
         <v>41579</v>
       </c>
       <c r="B96" t="n">
@@ -4093,7 +4105,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" s="2" t="n">
         <v>41609</v>
       </c>
       <c r="B97" t="n">
@@ -4131,7 +4143,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" s="2" t="n">
         <v>41640</v>
       </c>
       <c r="B98" t="n">
@@ -4169,7 +4181,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" s="2" t="n">
         <v>41671</v>
       </c>
       <c r="B99" t="n">
@@ -4207,7 +4219,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" s="2" t="n">
         <v>41699</v>
       </c>
       <c r="B100" t="n">
@@ -4245,7 +4257,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" s="2" t="n">
         <v>41730</v>
       </c>
       <c r="B101" t="n">
@@ -4283,7 +4295,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" s="2" t="n">
         <v>41760</v>
       </c>
       <c r="B102" t="n">
@@ -4321,7 +4333,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" s="2" t="n">
         <v>41791</v>
       </c>
       <c r="B103" t="n">
@@ -4359,7 +4371,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" s="2" t="n">
         <v>41821</v>
       </c>
       <c r="B104" t="n">
@@ -4397,7 +4409,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" s="2" t="n">
         <v>41852</v>
       </c>
       <c r="B105" t="n">
@@ -4435,7 +4447,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" s="2" t="n">
         <v>41883</v>
       </c>
       <c r="B106" t="n">
@@ -4473,7 +4485,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" s="2" t="n">
         <v>41913</v>
       </c>
       <c r="B107" t="n">
@@ -4511,7 +4523,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" s="2" t="n">
         <v>41944</v>
       </c>
       <c r="B108" t="n">
@@ -4549,7 +4561,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" s="2" t="n">
         <v>41974</v>
       </c>
       <c r="B109" t="n">
@@ -4587,7 +4599,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" s="2" t="n">
         <v>42005</v>
       </c>
       <c r="B110" t="n">
@@ -4625,7 +4637,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" s="2" t="n">
         <v>42036</v>
       </c>
       <c r="B111" t="n">
@@ -4663,7 +4675,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" s="2" t="n">
         <v>42064</v>
       </c>
       <c r="B112" t="n">
@@ -4701,7 +4713,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" s="2" t="n">
         <v>42095</v>
       </c>
       <c r="B113" t="n">
@@ -4739,7 +4751,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" s="2" t="n">
         <v>42125</v>
       </c>
       <c r="B114" t="n">
@@ -4777,7 +4789,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" s="2" t="n">
         <v>42156</v>
       </c>
       <c r="B115" t="n">
@@ -4815,7 +4827,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" s="2" t="n">
         <v>42186</v>
       </c>
       <c r="B116" t="n">
@@ -4853,7 +4865,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" s="2" t="n">
         <v>42217</v>
       </c>
       <c r="B117" t="n">
@@ -4891,7 +4903,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" s="2" t="n">
         <v>42248</v>
       </c>
       <c r="B118" t="n">
@@ -4929,7 +4941,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" s="2" t="n">
         <v>42278</v>
       </c>
       <c r="B119" t="n">
@@ -4967,7 +4979,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" s="2" t="n">
         <v>42309</v>
       </c>
       <c r="B120" t="n">
@@ -5005,7 +5017,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" s="2" t="n">
         <v>42339</v>
       </c>
       <c r="B121" t="n">
@@ -5043,7 +5055,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" s="2" t="n">
         <v>42370</v>
       </c>
       <c r="B122" t="n">
@@ -5081,7 +5093,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" s="2" t="n">
         <v>42401</v>
       </c>
       <c r="B123" t="n">
@@ -5119,7 +5131,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" s="2" t="n">
         <v>42430</v>
       </c>
       <c r="B124" t="n">
@@ -5157,7 +5169,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" s="2" t="n">
         <v>42461</v>
       </c>
       <c r="B125" t="n">
@@ -5195,7 +5207,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" s="2" t="n">
         <v>42491</v>
       </c>
       <c r="B126" t="n">
@@ -5233,7 +5245,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" s="2" t="n">
         <v>42522</v>
       </c>
       <c r="B127" t="n">
@@ -5271,7 +5283,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" s="2" t="n">
         <v>42552</v>
       </c>
       <c r="B128" t="n">
@@ -5309,7 +5321,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" s="2" t="n">
         <v>42583</v>
       </c>
       <c r="B129" t="n">
@@ -5347,7 +5359,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
+      <c r="A130" s="2" t="n">
         <v>42614</v>
       </c>
       <c r="B130" t="n">
@@ -5385,7 +5397,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
+      <c r="A131" s="2" t="n">
         <v>42644</v>
       </c>
       <c r="B131" t="n">
@@ -5423,7 +5435,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
+      <c r="A132" s="2" t="n">
         <v>42675</v>
       </c>
       <c r="B132" t="n">
@@ -5461,7 +5473,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
+      <c r="A133" s="2" t="n">
         <v>42705</v>
       </c>
       <c r="B133" t="n">
@@ -5499,7 +5511,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
+      <c r="A134" s="2" t="n">
         <v>42736</v>
       </c>
       <c r="B134" t="n">
@@ -5537,7 +5549,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
+      <c r="A135" s="2" t="n">
         <v>42767</v>
       </c>
       <c r="B135" t="n">
@@ -5575,7 +5587,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
+      <c r="A136" s="2" t="n">
         <v>42795</v>
       </c>
       <c r="B136" t="n">
@@ -5613,7 +5625,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
+      <c r="A137" s="2" t="n">
         <v>42826</v>
       </c>
       <c r="B137" t="n">
@@ -5651,7 +5663,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
+      <c r="A138" s="2" t="n">
         <v>42856</v>
       </c>
       <c r="B138" t="n">
@@ -5689,7 +5701,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="n">
+      <c r="A139" s="2" t="n">
         <v>42887</v>
       </c>
       <c r="B139" t="n">
@@ -5727,7 +5739,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="n">
+      <c r="A140" s="2" t="n">
         <v>42917</v>
       </c>
       <c r="B140" t="n">
@@ -5765,7 +5777,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="n">
+      <c r="A141" s="2" t="n">
         <v>42948</v>
       </c>
       <c r="B141" t="n">
@@ -5803,7 +5815,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="n">
+      <c r="A142" s="2" t="n">
         <v>42979</v>
       </c>
       <c r="B142" t="n">
@@ -5841,7 +5853,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="n">
+      <c r="A143" s="2" t="n">
         <v>43009</v>
       </c>
       <c r="B143" t="n">
@@ -5879,7 +5891,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="n">
+      <c r="A144" s="2" t="n">
         <v>43040</v>
       </c>
       <c r="B144" t="n">
@@ -5917,7 +5929,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="n">
+      <c r="A145" s="2" t="n">
         <v>43070</v>
       </c>
       <c r="B145" t="n">
@@ -5955,7 +5967,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="1" t="n">
+      <c r="A146" s="2" t="n">
         <v>43101</v>
       </c>
       <c r="B146" t="n">
@@ -5993,7 +6005,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="1" t="n">
+      <c r="A147" s="2" t="n">
         <v>43132</v>
       </c>
       <c r="B147" t="n">
@@ -6031,7 +6043,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="1" t="n">
+      <c r="A148" s="2" t="n">
         <v>43160</v>
       </c>
       <c r="B148" t="n">
@@ -6069,7 +6081,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="1" t="n">
+      <c r="A149" s="2" t="n">
         <v>43191</v>
       </c>
       <c r="B149" t="n">
@@ -6107,7 +6119,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="1" t="n">
+      <c r="A150" s="2" t="n">
         <v>43221</v>
       </c>
       <c r="B150" t="n">
@@ -6145,7 +6157,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="1" t="n">
+      <c r="A151" s="2" t="n">
         <v>43252</v>
       </c>
       <c r="B151" t="n">
@@ -6183,7 +6195,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="1" t="n">
+      <c r="A152" s="2" t="n">
         <v>43282</v>
       </c>
       <c r="B152" t="n">
@@ -6221,7 +6233,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="1" t="n">
+      <c r="A153" s="2" t="n">
         <v>43313</v>
       </c>
       <c r="B153" t="n">
@@ -6259,7 +6271,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="1" t="n">
+      <c r="A154" s="2" t="n">
         <v>43344</v>
       </c>
       <c r="B154" t="n">
@@ -6297,7 +6309,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="1" t="n">
+      <c r="A155" s="2" t="n">
         <v>43374</v>
       </c>
       <c r="B155" t="n">
@@ -6335,7 +6347,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="1" t="n">
+      <c r="A156" s="2" t="n">
         <v>43405</v>
       </c>
       <c r="B156" t="n">
@@ -6373,7 +6385,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="1" t="n">
+      <c r="A157" s="2" t="n">
         <v>43435</v>
       </c>
       <c r="B157" t="n">
@@ -6411,7 +6423,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="1" t="n">
+      <c r="A158" s="2" t="n">
         <v>43466</v>
       </c>
       <c r="B158" t="n">
@@ -6449,7 +6461,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="1" t="n">
+      <c r="A159" s="2" t="n">
         <v>43497</v>
       </c>
       <c r="B159" t="n">
@@ -6487,7 +6499,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="1" t="n">
+      <c r="A160" s="2" t="n">
         <v>43525</v>
       </c>
       <c r="B160" t="n">
@@ -6525,7 +6537,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="1" t="n">
+      <c r="A161" s="2" t="n">
         <v>43556</v>
       </c>
       <c r="B161" t="n">
@@ -6563,7 +6575,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="1" t="n">
+      <c r="A162" s="2" t="n">
         <v>43586</v>
       </c>
       <c r="B162" t="n">
@@ -6601,7 +6613,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="1" t="n">
+      <c r="A163" s="2" t="n">
         <v>43617</v>
       </c>
       <c r="B163" t="n">
@@ -6639,7 +6651,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="1" t="n">
+      <c r="A164" s="2" t="n">
         <v>43647</v>
       </c>
       <c r="B164" t="n">
@@ -6677,7 +6689,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="1" t="n">
+      <c r="A165" s="2" t="n">
         <v>43678</v>
       </c>
       <c r="B165" t="n">
@@ -6715,7 +6727,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="1" t="n">
+      <c r="A166" s="2" t="n">
         <v>43709</v>
       </c>
       <c r="B166" t="n">
@@ -6753,7 +6765,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="1" t="n">
+      <c r="A167" s="2" t="n">
         <v>43739</v>
       </c>
       <c r="B167" t="n">
@@ -6791,7 +6803,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="1" t="n">
+      <c r="A168" s="2" t="n">
         <v>43770</v>
       </c>
       <c r="B168" t="n">
@@ -6829,7 +6841,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="1" t="n">
+      <c r="A169" s="2" t="n">
         <v>43800</v>
       </c>
       <c r="B169" t="n">
@@ -6867,7 +6879,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="1" t="n">
+      <c r="A170" s="2" t="n">
         <v>43831</v>
       </c>
       <c r="B170" t="n">
@@ -6905,7 +6917,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="1" t="n">
+      <c r="A171" s="2" t="n">
         <v>43862</v>
       </c>
       <c r="B171" t="n">
@@ -6943,7 +6955,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="1" t="n">
+      <c r="A172" s="2" t="n">
         <v>43891</v>
       </c>
       <c r="B172" t="n">
@@ -6981,7 +6993,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="1" t="n">
+      <c r="A173" s="2" t="n">
         <v>43922</v>
       </c>
       <c r="B173" t="n">
@@ -7019,7 +7031,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="1" t="n">
+      <c r="A174" s="2" t="n">
         <v>43952</v>
       </c>
       <c r="B174" t="n">
@@ -7057,7 +7069,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="1" t="n">
+      <c r="A175" s="2" t="n">
         <v>43983</v>
       </c>
       <c r="B175" t="n">
@@ -7095,7 +7107,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="1" t="n">
+      <c r="A176" s="2" t="n">
         <v>44013</v>
       </c>
       <c r="B176" t="n">
@@ -7133,7 +7145,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="1" t="n">
+      <c r="A177" s="2" t="n">
         <v>44044</v>
       </c>
       <c r="B177" t="n">
@@ -7171,7 +7183,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="1" t="n">
+      <c r="A178" s="2" t="n">
         <v>44075</v>
       </c>
       <c r="B178" t="n">
@@ -7209,7 +7221,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="1" t="n">
+      <c r="A179" s="2" t="n">
         <v>44105</v>
       </c>
       <c r="B179" t="n">
@@ -7247,7 +7259,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="1" t="n">
+      <c r="A180" s="2" t="n">
         <v>44136</v>
       </c>
       <c r="B180" t="n">
@@ -7285,7 +7297,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="1" t="n">
+      <c r="A181" s="2" t="n">
         <v>44166</v>
       </c>
       <c r="B181" t="n">
@@ -7323,7 +7335,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="1" t="n">
+      <c r="A182" s="2" t="n">
         <v>44197</v>
       </c>
       <c r="B182" t="n">
@@ -7361,7 +7373,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="1" t="n">
+      <c r="A183" s="2" t="n">
         <v>44228</v>
       </c>
       <c r="B183" t="n">
@@ -7399,7 +7411,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="1" t="n">
+      <c r="A184" s="2" t="n">
         <v>44256</v>
       </c>
       <c r="B184" t="n">
@@ -7437,7 +7449,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="1" t="n">
+      <c r="A185" s="2" t="n">
         <v>44287</v>
       </c>
       <c r="B185" t="n">
@@ -7475,7 +7487,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="1" t="n">
+      <c r="A186" s="2" t="n">
         <v>44317</v>
       </c>
       <c r="B186" t="n">
@@ -7513,7 +7525,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="1" t="n">
+      <c r="A187" s="2" t="n">
         <v>44348</v>
       </c>
       <c r="B187" t="n">
@@ -7551,7 +7563,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="1" t="n">
+      <c r="A188" s="2" t="n">
         <v>44378</v>
       </c>
       <c r="B188" t="n">
@@ -7589,7 +7601,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="1" t="n">
+      <c r="A189" s="2" t="n">
         <v>44409</v>
       </c>
       <c r="B189" t="n">
@@ -7627,7 +7639,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="1" t="n">
+      <c r="A190" s="2" t="n">
         <v>44440</v>
       </c>
       <c r="B190" t="n">
@@ -7665,7 +7677,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="1" t="n">
+      <c r="A191" s="2" t="n">
         <v>44470</v>
       </c>
       <c r="B191" t="n">
@@ -7703,7 +7715,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="1" t="n">
+      <c r="A192" s="2" t="n">
         <v>44501</v>
       </c>
       <c r="B192" t="n">
@@ -7741,7 +7753,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="1" t="n">
+      <c r="A193" s="2" t="n">
         <v>44531</v>
       </c>
       <c r="B193" t="n">
@@ -7779,7 +7791,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="1" t="n">
+      <c r="A194" s="2" t="n">
         <v>44562</v>
       </c>
       <c r="B194" t="n">
@@ -7817,7 +7829,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="1" t="n">
+      <c r="A195" s="2" t="n">
         <v>44593</v>
       </c>
       <c r="B195" t="n">
@@ -7855,7 +7867,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="1" t="n">
+      <c r="A196" s="2" t="n">
         <v>44621</v>
       </c>
       <c r="B196" t="n">
@@ -7893,7 +7905,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="1" t="n">
+      <c r="A197" s="2" t="n">
         <v>44652</v>
       </c>
       <c r="B197" t="n">
@@ -7931,7 +7943,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="1" t="n">
+      <c r="A198" s="2" t="n">
         <v>44682</v>
       </c>
       <c r="B198" t="n">
@@ -7969,7 +7981,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="1" t="n">
+      <c r="A199" s="2" t="n">
         <v>44713</v>
       </c>
       <c r="B199" t="n">
@@ -8007,7 +8019,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="1" t="n">
+      <c r="A200" s="2" t="n">
         <v>44743</v>
       </c>
       <c r="B200" t="n">
@@ -8045,7 +8057,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="1" t="n">
+      <c r="A201" s="2" t="n">
         <v>44774</v>
       </c>
       <c r="B201" t="n">
@@ -8083,7 +8095,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="1" t="n">
+      <c r="A202" s="2" t="n">
         <v>44805</v>
       </c>
       <c r="B202" t="n">
@@ -8121,7 +8133,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="1" t="n">
+      <c r="A203" s="2" t="n">
         <v>44835</v>
       </c>
       <c r="B203" t="n">
@@ -8159,7 +8171,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="1" t="n">
+      <c r="A204" s="2" t="n">
         <v>44866</v>
       </c>
       <c r="B204" t="n">
@@ -8197,7 +8209,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="1" t="n">
+      <c r="A205" s="2" t="n">
         <v>44896</v>
       </c>
       <c r="B205" t="n">
@@ -8235,7 +8247,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="1" t="n">
+      <c r="A206" s="2" t="n">
         <v>44927</v>
       </c>
       <c r="B206" t="n">
@@ -8273,7 +8285,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="1" t="n">
+      <c r="A207" s="2" t="n">
         <v>44958</v>
       </c>
       <c r="B207" t="n">
@@ -8311,7 +8323,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="1" t="n">
+      <c r="A208" s="2" t="n">
         <v>44986</v>
       </c>
       <c r="B208" t="n">
@@ -8349,7 +8361,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="1" t="n">
+      <c r="A209" s="2" t="n">
         <v>45017</v>
       </c>
       <c r="B209" t="n">
@@ -8387,7 +8399,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="1" t="n">
+      <c r="A210" s="2" t="n">
         <v>45047</v>
       </c>
       <c r="B210" t="n">
@@ -8425,7 +8437,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="1" t="n">
+      <c r="A211" s="2" t="n">
         <v>45078</v>
       </c>
       <c r="B211" t="n">
@@ -8463,7 +8475,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="1" t="n">
+      <c r="A212" s="2" t="n">
         <v>45108</v>
       </c>
       <c r="B212" t="n">
@@ -8501,7 +8513,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="1" t="n">
+      <c r="A213" s="2" t="n">
         <v>45139</v>
       </c>
       <c r="B213" t="n">
@@ -8539,7 +8551,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="1" t="n">
+      <c r="A214" s="2" t="n">
         <v>45170</v>
       </c>
       <c r="B214" t="n">
@@ -8577,7 +8589,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="1" t="n">
+      <c r="A215" s="2" t="n">
         <v>45200</v>
       </c>
       <c r="B215" t="n">
@@ -8615,7 +8627,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="1" t="n">
+      <c r="A216" s="2" t="n">
         <v>45231</v>
       </c>
       <c r="B216" t="n">
@@ -8653,7 +8665,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="1" t="n">
+      <c r="A217" s="2" t="n">
         <v>45261</v>
       </c>
       <c r="B217" t="n">
@@ -8691,7 +8703,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="1" t="n">
+      <c r="A218" s="2" t="n">
         <v>45292</v>
       </c>
       <c r="B218" t="n">
@@ -8729,7 +8741,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="1" t="n">
+      <c r="A219" s="2" t="n">
         <v>45323</v>
       </c>
       <c r="B219" t="n">
@@ -8767,7 +8779,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="1" t="n">
+      <c r="A220" s="2" t="n">
         <v>45352</v>
       </c>
       <c r="B220" t="n">
@@ -8805,7 +8817,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="1" t="n">
+      <c r="A221" s="2" t="n">
         <v>45383</v>
       </c>
       <c r="B221" t="n">
@@ -8843,7 +8855,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="1" t="n">
+      <c r="A222" s="2" t="n">
         <v>45413</v>
       </c>
       <c r="B222" t="n">
@@ -8881,7 +8893,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="1" t="n">
+      <c r="A223" s="2" t="n">
         <v>45444</v>
       </c>
       <c r="B223" t="n">
@@ -8919,7 +8931,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="1" t="n">
+      <c r="A224" s="2" t="n">
         <v>45474</v>
       </c>
       <c r="B224" t="n">
@@ -8957,7 +8969,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="1" t="n">
+      <c r="A225" s="2" t="n">
         <v>45505</v>
       </c>
       <c r="B225" t="n">
@@ -8995,7 +9007,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="1" t="n">
+      <c r="A226" s="2" t="n">
         <v>45536</v>
       </c>
       <c r="B226" t="n">
@@ -9033,7 +9045,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="1" t="n">
+      <c r="A227" s="2" t="n">
         <v>45566</v>
       </c>
       <c r="B227" t="n">
@@ -9071,7 +9083,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="1" t="n">
+      <c r="A228" s="2" t="n">
         <v>45597</v>
       </c>
       <c r="B228" t="n">
@@ -9109,7 +9121,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="1" t="n">
+      <c r="A229" s="2" t="n">
         <v>45627</v>
       </c>
       <c r="B229" t="n">
@@ -9147,7 +9159,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="1" t="n">
+      <c r="A230" s="2" t="n">
         <v>45658</v>
       </c>
       <c r="B230" t="n">
@@ -9185,7 +9197,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="1" t="n">
+      <c r="A231" s="2" t="n">
         <v>45689</v>
       </c>
       <c r="B231" t="n">
@@ -9223,7 +9235,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="1" t="n">
+      <c r="A232" s="2" t="n">
         <v>45717</v>
       </c>
       <c r="B232" t="n">
@@ -9261,7 +9273,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="1" t="n">
+      <c r="A233" s="2" t="n">
         <v>45748</v>
       </c>
       <c r="B233" t="n">
@@ -9299,7 +9311,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="1" t="n">
+      <c r="A234" s="2" t="n">
         <v>45778</v>
       </c>
       <c r="B234" t="n">
@@ -9337,7 +9349,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="1" t="n">
+      <c r="A235" s="2" t="n">
         <v>45809</v>
       </c>
       <c r="B235" t="n">
@@ -9375,7 +9387,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="1" t="n">
+      <c r="A236" s="2" t="n">
         <v>45839</v>
       </c>
       <c r="B236" t="n">
@@ -9413,7 +9425,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="1" t="n">
+      <c r="A237" s="2" t="n">
         <v>45870</v>
       </c>
       <c r="B237" t="n">
@@ -9451,7 +9463,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="1" t="n">
+      <c r="A238" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="B238" t="n">
@@ -9489,7 +9501,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="1" t="n">
+      <c r="A239" s="2" t="n">
         <v>45931</v>
       </c>
       <c r="B239" t="n">
@@ -9527,7 +9539,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="1" t="n">
+      <c r="A240" s="2" t="n">
         <v>45962</v>
       </c>
       <c r="B240" t="n">
@@ -9565,7 +9577,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="1" t="n">
+      <c r="A241" s="2" t="n">
         <v>45992</v>
       </c>
       <c r="B241" t="n">
@@ -9603,7 +9615,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="1" t="n">
+      <c r="A242" s="2" t="n">
         <v>46023</v>
       </c>
       <c r="B242" t="n">
@@ -9641,7 +9653,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="1" t="n">
+      <c r="A243" s="2" t="n">
         <v>46054</v>
       </c>
       <c r="B243" t="n">
@@ -9679,7 +9691,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="1" t="n">
+      <c r="A244" s="2" t="n">
         <v>46082</v>
       </c>
       <c r="B244" t="n">
@@ -9717,7 +9729,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="1" t="n">
+      <c r="A245" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="B245" t="n">
@@ -9755,7 +9767,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="1" t="n">
+      <c r="A246" s="2" t="n">
         <v>46143</v>
       </c>
       <c r="B246" t="n">
@@ -9793,7 +9805,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="1" t="n">
+      <c r="A247" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="B247" t="n">

</xml_diff>

<commit_message>
Otomatik veri güncelleme (14.08.2026 12:29 UTC)
</commit_message>
<xml_diff>
--- a/butce/butce.xlsx
+++ b/butce/butce.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,69 +421,69 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tarih</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>yil</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ay</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>gelir</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>vergi</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>dolaysiz_vergi</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>dolayli_vergi</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>gider</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>faiz_haric_gider</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>faiz_gideri</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>faiz_disi_denge</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>denge</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>38718</v>
       </c>
       <c r="B2" t="n">
@@ -533,7 +521,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>38749</v>
       </c>
       <c r="B3" t="n">
@@ -571,7 +559,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>38777</v>
       </c>
       <c r="B4" t="n">
@@ -609,7 +597,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>38808</v>
       </c>
       <c r="B5" t="n">
@@ -647,7 +635,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>38838</v>
       </c>
       <c r="B6" t="n">
@@ -685,7 +673,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>38869</v>
       </c>
       <c r="B7" t="n">
@@ -723,7 +711,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>38899</v>
       </c>
       <c r="B8" t="n">
@@ -761,7 +749,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>38930</v>
       </c>
       <c r="B9" t="n">
@@ -799,7 +787,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>38961</v>
       </c>
       <c r="B10" t="n">
@@ -837,7 +825,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>38991</v>
       </c>
       <c r="B11" t="n">
@@ -875,7 +863,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>39022</v>
       </c>
       <c r="B12" t="n">
@@ -913,7 +901,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>39052</v>
       </c>
       <c r="B13" t="n">
@@ -951,7 +939,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>39083</v>
       </c>
       <c r="B14" t="n">
@@ -989,7 +977,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>39114</v>
       </c>
       <c r="B15" t="n">
@@ -1027,7 +1015,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>39142</v>
       </c>
       <c r="B16" t="n">
@@ -1065,7 +1053,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>39173</v>
       </c>
       <c r="B17" t="n">
@@ -1103,7 +1091,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>39203</v>
       </c>
       <c r="B18" t="n">
@@ -1141,7 +1129,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>39234</v>
       </c>
       <c r="B19" t="n">
@@ -1179,7 +1167,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>39264</v>
       </c>
       <c r="B20" t="n">
@@ -1217,7 +1205,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>39295</v>
       </c>
       <c r="B21" t="n">
@@ -1255,7 +1243,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>39326</v>
       </c>
       <c r="B22" t="n">
@@ -1293,7 +1281,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>39356</v>
       </c>
       <c r="B23" t="n">
@@ -1331,7 +1319,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>39387</v>
       </c>
       <c r="B24" t="n">
@@ -1369,7 +1357,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>39417</v>
       </c>
       <c r="B25" t="n">
@@ -1407,7 +1395,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>39448</v>
       </c>
       <c r="B26" t="n">
@@ -1445,7 +1433,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="1" t="n">
         <v>39479</v>
       </c>
       <c r="B27" t="n">
@@ -1483,7 +1471,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>39508</v>
       </c>
       <c r="B28" t="n">
@@ -1521,7 +1509,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>39539</v>
       </c>
       <c r="B29" t="n">
@@ -1559,7 +1547,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>39569</v>
       </c>
       <c r="B30" t="n">
@@ -1597,7 +1585,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>39600</v>
       </c>
       <c r="B31" t="n">
@@ -1635,7 +1623,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>39630</v>
       </c>
       <c r="B32" t="n">
@@ -1673,7 +1661,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>39661</v>
       </c>
       <c r="B33" t="n">
@@ -1711,7 +1699,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>39692</v>
       </c>
       <c r="B34" t="n">
@@ -1749,7 +1737,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>39722</v>
       </c>
       <c r="B35" t="n">
@@ -1787,7 +1775,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>39753</v>
       </c>
       <c r="B36" t="n">
@@ -1825,7 +1813,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>39783</v>
       </c>
       <c r="B37" t="n">
@@ -1863,7 +1851,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>39814</v>
       </c>
       <c r="B38" t="n">
@@ -1901,7 +1889,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>39845</v>
       </c>
       <c r="B39" t="n">
@@ -1939,7 +1927,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>39873</v>
       </c>
       <c r="B40" t="n">
@@ -1977,7 +1965,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>39904</v>
       </c>
       <c r="B41" t="n">
@@ -2015,7 +2003,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>39934</v>
       </c>
       <c r="B42" t="n">
@@ -2053,7 +2041,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>39965</v>
       </c>
       <c r="B43" t="n">
@@ -2091,7 +2079,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>39995</v>
       </c>
       <c r="B44" t="n">
@@ -2129,7 +2117,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>40026</v>
       </c>
       <c r="B45" t="n">
@@ -2167,7 +2155,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>40057</v>
       </c>
       <c r="B46" t="n">
@@ -2205,7 +2193,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>40087</v>
       </c>
       <c r="B47" t="n">
@@ -2243,7 +2231,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>40118</v>
       </c>
       <c r="B48" t="n">
@@ -2281,7 +2269,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>40148</v>
       </c>
       <c r="B49" t="n">
@@ -2319,7 +2307,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>40179</v>
       </c>
       <c r="B50" t="n">
@@ -2357,7 +2345,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>40210</v>
       </c>
       <c r="B51" t="n">
@@ -2395,7 +2383,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>40238</v>
       </c>
       <c r="B52" t="n">
@@ -2433,7 +2421,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>40269</v>
       </c>
       <c r="B53" t="n">
@@ -2471,7 +2459,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>40299</v>
       </c>
       <c r="B54" t="n">
@@ -2509,7 +2497,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>40330</v>
       </c>
       <c r="B55" t="n">
@@ -2547,7 +2535,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>40360</v>
       </c>
       <c r="B56" t="n">
@@ -2585,7 +2573,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>40391</v>
       </c>
       <c r="B57" t="n">
@@ -2623,7 +2611,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>40422</v>
       </c>
       <c r="B58" t="n">
@@ -2661,7 +2649,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>40452</v>
       </c>
       <c r="B59" t="n">
@@ -2699,7 +2687,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>40483</v>
       </c>
       <c r="B60" t="n">
@@ -2737,7 +2725,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>40513</v>
       </c>
       <c r="B61" t="n">
@@ -2775,7 +2763,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>40544</v>
       </c>
       <c r="B62" t="n">
@@ -2813,7 +2801,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="1" t="n">
         <v>40575</v>
       </c>
       <c r="B63" t="n">
@@ -2851,7 +2839,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="1" t="n">
         <v>40603</v>
       </c>
       <c r="B64" t="n">
@@ -2889,7 +2877,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="1" t="n">
         <v>40634</v>
       </c>
       <c r="B65" t="n">
@@ -2927,7 +2915,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="1" t="n">
         <v>40664</v>
       </c>
       <c r="B66" t="n">
@@ -2965,7 +2953,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="1" t="n">
         <v>40695</v>
       </c>
       <c r="B67" t="n">
@@ -3003,7 +2991,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="1" t="n">
         <v>40725</v>
       </c>
       <c r="B68" t="n">
@@ -3041,7 +3029,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="1" t="n">
         <v>40756</v>
       </c>
       <c r="B69" t="n">
@@ -3079,7 +3067,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="1" t="n">
         <v>40787</v>
       </c>
       <c r="B70" t="n">
@@ -3117,7 +3105,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="1" t="n">
         <v>40817</v>
       </c>
       <c r="B71" t="n">
@@ -3155,7 +3143,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="1" t="n">
         <v>40848</v>
       </c>
       <c r="B72" t="n">
@@ -3193,7 +3181,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="1" t="n">
         <v>40878</v>
       </c>
       <c r="B73" t="n">
@@ -3231,7 +3219,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="1" t="n">
         <v>40909</v>
       </c>
       <c r="B74" t="n">
@@ -3269,7 +3257,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="1" t="n">
         <v>40940</v>
       </c>
       <c r="B75" t="n">
@@ -3307,7 +3295,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="1" t="n">
         <v>40969</v>
       </c>
       <c r="B76" t="n">
@@ -3345,7 +3333,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="1" t="n">
         <v>41000</v>
       </c>
       <c r="B77" t="n">
@@ -3383,7 +3371,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="1" t="n">
         <v>41030</v>
       </c>
       <c r="B78" t="n">
@@ -3421,7 +3409,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="1" t="n">
         <v>41061</v>
       </c>
       <c r="B79" t="n">
@@ -3459,7 +3447,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="1" t="n">
         <v>41091</v>
       </c>
       <c r="B80" t="n">
@@ -3497,7 +3485,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="1" t="n">
         <v>41122</v>
       </c>
       <c r="B81" t="n">
@@ -3535,7 +3523,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="1" t="n">
         <v>41153</v>
       </c>
       <c r="B82" t="n">
@@ -3573,7 +3561,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="1" t="n">
         <v>41183</v>
       </c>
       <c r="B83" t="n">
@@ -3611,7 +3599,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="1" t="n">
         <v>41214</v>
       </c>
       <c r="B84" t="n">
@@ -3649,7 +3637,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="1" t="n">
         <v>41244</v>
       </c>
       <c r="B85" t="n">
@@ -3687,7 +3675,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="1" t="n">
         <v>41275</v>
       </c>
       <c r="B86" t="n">
@@ -3725,7 +3713,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="1" t="n">
         <v>41306</v>
       </c>
       <c r="B87" t="n">
@@ -3763,7 +3751,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="1" t="n">
         <v>41334</v>
       </c>
       <c r="B88" t="n">
@@ -3801,7 +3789,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="1" t="n">
         <v>41365</v>
       </c>
       <c r="B89" t="n">
@@ -3839,7 +3827,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="1" t="n">
         <v>41395</v>
       </c>
       <c r="B90" t="n">
@@ -3877,7 +3865,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="1" t="n">
         <v>41426</v>
       </c>
       <c r="B91" t="n">
@@ -3915,7 +3903,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="1" t="n">
         <v>41456</v>
       </c>
       <c r="B92" t="n">
@@ -3953,7 +3941,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="1" t="n">
         <v>41487</v>
       </c>
       <c r="B93" t="n">
@@ -3991,7 +3979,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="1" t="n">
         <v>41518</v>
       </c>
       <c r="B94" t="n">
@@ -4029,7 +4017,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" s="1" t="n">
         <v>41548</v>
       </c>
       <c r="B95" t="n">
@@ -4067,7 +4055,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="1" t="n">
         <v>41579</v>
       </c>
       <c r="B96" t="n">
@@ -4105,7 +4093,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="1" t="n">
         <v>41609</v>
       </c>
       <c r="B97" t="n">
@@ -4143,7 +4131,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="1" t="n">
         <v>41640</v>
       </c>
       <c r="B98" t="n">
@@ -4181,7 +4169,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="1" t="n">
         <v>41671</v>
       </c>
       <c r="B99" t="n">
@@ -4219,7 +4207,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="1" t="n">
         <v>41699</v>
       </c>
       <c r="B100" t="n">
@@ -4257,7 +4245,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="1" t="n">
         <v>41730</v>
       </c>
       <c r="B101" t="n">
@@ -4295,7 +4283,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="1" t="n">
         <v>41760</v>
       </c>
       <c r="B102" t="n">
@@ -4333,7 +4321,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="1" t="n">
         <v>41791</v>
       </c>
       <c r="B103" t="n">
@@ -4371,7 +4359,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="1" t="n">
         <v>41821</v>
       </c>
       <c r="B104" t="n">
@@ -4409,7 +4397,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="1" t="n">
         <v>41852</v>
       </c>
       <c r="B105" t="n">
@@ -4447,7 +4435,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="1" t="n">
         <v>41883</v>
       </c>
       <c r="B106" t="n">
@@ -4485,7 +4473,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="1" t="n">
         <v>41913</v>
       </c>
       <c r="B107" t="n">
@@ -4523,7 +4511,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="1" t="n">
         <v>41944</v>
       </c>
       <c r="B108" t="n">
@@ -4561,7 +4549,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
+      <c r="A109" s="1" t="n">
         <v>41974</v>
       </c>
       <c r="B109" t="n">
@@ -4599,7 +4587,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
+      <c r="A110" s="1" t="n">
         <v>42005</v>
       </c>
       <c r="B110" t="n">
@@ -4637,7 +4625,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="1" t="n">
         <v>42036</v>
       </c>
       <c r="B111" t="n">
@@ -4675,7 +4663,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="1" t="n">
         <v>42064</v>
       </c>
       <c r="B112" t="n">
@@ -4713,7 +4701,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="1" t="n">
         <v>42095</v>
       </c>
       <c r="B113" t="n">
@@ -4751,7 +4739,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="1" t="n">
         <v>42125</v>
       </c>
       <c r="B114" t="n">
@@ -4789,7 +4777,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="1" t="n">
         <v>42156</v>
       </c>
       <c r="B115" t="n">
@@ -4827,7 +4815,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
+      <c r="A116" s="1" t="n">
         <v>42186</v>
       </c>
       <c r="B116" t="n">
@@ -4865,7 +4853,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
+      <c r="A117" s="1" t="n">
         <v>42217</v>
       </c>
       <c r="B117" t="n">
@@ -4903,7 +4891,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
+      <c r="A118" s="1" t="n">
         <v>42248</v>
       </c>
       <c r="B118" t="n">
@@ -4941,7 +4929,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
+      <c r="A119" s="1" t="n">
         <v>42278</v>
       </c>
       <c r="B119" t="n">
@@ -4979,7 +4967,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
+      <c r="A120" s="1" t="n">
         <v>42309</v>
       </c>
       <c r="B120" t="n">
@@ -5017,7 +5005,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
+      <c r="A121" s="1" t="n">
         <v>42339</v>
       </c>
       <c r="B121" t="n">
@@ -5055,7 +5043,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
+      <c r="A122" s="1" t="n">
         <v>42370</v>
       </c>
       <c r="B122" t="n">
@@ -5093,7 +5081,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
+      <c r="A123" s="1" t="n">
         <v>42401</v>
       </c>
       <c r="B123" t="n">
@@ -5131,7 +5119,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
+      <c r="A124" s="1" t="n">
         <v>42430</v>
       </c>
       <c r="B124" t="n">
@@ -5169,7 +5157,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
+      <c r="A125" s="1" t="n">
         <v>42461</v>
       </c>
       <c r="B125" t="n">
@@ -5207,7 +5195,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" s="1" t="n">
         <v>42491</v>
       </c>
       <c r="B126" t="n">
@@ -5245,7 +5233,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
+      <c r="A127" s="1" t="n">
         <v>42522</v>
       </c>
       <c r="B127" t="n">
@@ -5283,7 +5271,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
+      <c r="A128" s="1" t="n">
         <v>42552</v>
       </c>
       <c r="B128" t="n">
@@ -5321,7 +5309,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
+      <c r="A129" s="1" t="n">
         <v>42583</v>
       </c>
       <c r="B129" t="n">
@@ -5359,7 +5347,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
+      <c r="A130" s="1" t="n">
         <v>42614</v>
       </c>
       <c r="B130" t="n">
@@ -5397,7 +5385,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
+      <c r="A131" s="1" t="n">
         <v>42644</v>
       </c>
       <c r="B131" t="n">
@@ -5435,7 +5423,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" s="1" t="n">
         <v>42675</v>
       </c>
       <c r="B132" t="n">
@@ -5473,7 +5461,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" s="1" t="n">
         <v>42705</v>
       </c>
       <c r="B133" t="n">
@@ -5511,7 +5499,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
+      <c r="A134" s="1" t="n">
         <v>42736</v>
       </c>
       <c r="B134" t="n">
@@ -5549,7 +5537,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
+      <c r="A135" s="1" t="n">
         <v>42767</v>
       </c>
       <c r="B135" t="n">
@@ -5587,7 +5575,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="1" t="n">
         <v>42795</v>
       </c>
       <c r="B136" t="n">
@@ -5625,7 +5613,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
+      <c r="A137" s="1" t="n">
         <v>42826</v>
       </c>
       <c r="B137" t="n">
@@ -5663,7 +5651,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
+      <c r="A138" s="1" t="n">
         <v>42856</v>
       </c>
       <c r="B138" t="n">
@@ -5701,7 +5689,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
+      <c r="A139" s="1" t="n">
         <v>42887</v>
       </c>
       <c r="B139" t="n">
@@ -5739,7 +5727,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
+      <c r="A140" s="1" t="n">
         <v>42917</v>
       </c>
       <c r="B140" t="n">
@@ -5777,7 +5765,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
+      <c r="A141" s="1" t="n">
         <v>42948</v>
       </c>
       <c r="B141" t="n">
@@ -5815,7 +5803,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
+      <c r="A142" s="1" t="n">
         <v>42979</v>
       </c>
       <c r="B142" t="n">
@@ -5853,7 +5841,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
+      <c r="A143" s="1" t="n">
         <v>43009</v>
       </c>
       <c r="B143" t="n">
@@ -5891,7 +5879,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
+      <c r="A144" s="1" t="n">
         <v>43040</v>
       </c>
       <c r="B144" t="n">
@@ -5929,7 +5917,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
+      <c r="A145" s="1" t="n">
         <v>43070</v>
       </c>
       <c r="B145" t="n">
@@ -5967,7 +5955,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n">
+      <c r="A146" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="B146" t="n">
@@ -6005,7 +5993,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
+      <c r="A147" s="1" t="n">
         <v>43132</v>
       </c>
       <c r="B147" t="n">
@@ -6043,7 +6031,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
+      <c r="A148" s="1" t="n">
         <v>43160</v>
       </c>
       <c r="B148" t="n">
@@ -6081,7 +6069,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
+      <c r="A149" s="1" t="n">
         <v>43191</v>
       </c>
       <c r="B149" t="n">
@@ -6119,7 +6107,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
+      <c r="A150" s="1" t="n">
         <v>43221</v>
       </c>
       <c r="B150" t="n">
@@ -6157,7 +6145,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n">
+      <c r="A151" s="1" t="n">
         <v>43252</v>
       </c>
       <c r="B151" t="n">
@@ -6195,7 +6183,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n">
+      <c r="A152" s="1" t="n">
         <v>43282</v>
       </c>
       <c r="B152" t="n">
@@ -6233,7 +6221,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
+      <c r="A153" s="1" t="n">
         <v>43313</v>
       </c>
       <c r="B153" t="n">
@@ -6271,7 +6259,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
+      <c r="A154" s="1" t="n">
         <v>43344</v>
       </c>
       <c r="B154" t="n">
@@ -6309,7 +6297,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n">
+      <c r="A155" s="1" t="n">
         <v>43374</v>
       </c>
       <c r="B155" t="n">
@@ -6347,7 +6335,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
+      <c r="A156" s="1" t="n">
         <v>43405</v>
       </c>
       <c r="B156" t="n">
@@ -6385,7 +6373,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n">
+      <c r="A157" s="1" t="n">
         <v>43435</v>
       </c>
       <c r="B157" t="n">
@@ -6423,7 +6411,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n">
+      <c r="A158" s="1" t="n">
         <v>43466</v>
       </c>
       <c r="B158" t="n">
@@ -6461,7 +6449,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n">
+      <c r="A159" s="1" t="n">
         <v>43497</v>
       </c>
       <c r="B159" t="n">
@@ -6499,7 +6487,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
+      <c r="A160" s="1" t="n">
         <v>43525</v>
       </c>
       <c r="B160" t="n">
@@ -6537,7 +6525,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
+      <c r="A161" s="1" t="n">
         <v>43556</v>
       </c>
       <c r="B161" t="n">
@@ -6575,7 +6563,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
+      <c r="A162" s="1" t="n">
         <v>43586</v>
       </c>
       <c r="B162" t="n">
@@ -6613,7 +6601,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
+      <c r="A163" s="1" t="n">
         <v>43617</v>
       </c>
       <c r="B163" t="n">
@@ -6651,7 +6639,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
+      <c r="A164" s="1" t="n">
         <v>43647</v>
       </c>
       <c r="B164" t="n">
@@ -6689,7 +6677,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n">
+      <c r="A165" s="1" t="n">
         <v>43678</v>
       </c>
       <c r="B165" t="n">
@@ -6727,7 +6715,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n">
+      <c r="A166" s="1" t="n">
         <v>43709</v>
       </c>
       <c r="B166" t="n">
@@ -6765,7 +6753,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
+      <c r="A167" s="1" t="n">
         <v>43739</v>
       </c>
       <c r="B167" t="n">
@@ -6803,7 +6791,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
+      <c r="A168" s="1" t="n">
         <v>43770</v>
       </c>
       <c r="B168" t="n">
@@ -6841,7 +6829,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
+      <c r="A169" s="1" t="n">
         <v>43800</v>
       </c>
       <c r="B169" t="n">
@@ -6879,7 +6867,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n">
+      <c r="A170" s="1" t="n">
         <v>43831</v>
       </c>
       <c r="B170" t="n">
@@ -6917,7 +6905,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
+      <c r="A171" s="1" t="n">
         <v>43862</v>
       </c>
       <c r="B171" t="n">
@@ -6955,7 +6943,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n">
+      <c r="A172" s="1" t="n">
         <v>43891</v>
       </c>
       <c r="B172" t="n">
@@ -6993,7 +6981,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n">
+      <c r="A173" s="1" t="n">
         <v>43922</v>
       </c>
       <c r="B173" t="n">
@@ -7031,7 +7019,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
+      <c r="A174" s="1" t="n">
         <v>43952</v>
       </c>
       <c r="B174" t="n">
@@ -7069,7 +7057,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
+      <c r="A175" s="1" t="n">
         <v>43983</v>
       </c>
       <c r="B175" t="n">
@@ -7107,7 +7095,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
+      <c r="A176" s="1" t="n">
         <v>44013</v>
       </c>
       <c r="B176" t="n">
@@ -7145,7 +7133,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
+      <c r="A177" s="1" t="n">
         <v>44044</v>
       </c>
       <c r="B177" t="n">
@@ -7183,7 +7171,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
+      <c r="A178" s="1" t="n">
         <v>44075</v>
       </c>
       <c r="B178" t="n">
@@ -7221,7 +7209,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n">
+      <c r="A179" s="1" t="n">
         <v>44105</v>
       </c>
       <c r="B179" t="n">
@@ -7259,7 +7247,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n">
+      <c r="A180" s="1" t="n">
         <v>44136</v>
       </c>
       <c r="B180" t="n">
@@ -7297,7 +7285,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
+      <c r="A181" s="1" t="n">
         <v>44166</v>
       </c>
       <c r="B181" t="n">
@@ -7335,7 +7323,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
+      <c r="A182" s="1" t="n">
         <v>44197</v>
       </c>
       <c r="B182" t="n">
@@ -7373,7 +7361,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
+      <c r="A183" s="1" t="n">
         <v>44228</v>
       </c>
       <c r="B183" t="n">
@@ -7411,7 +7399,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n">
+      <c r="A184" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="B184" t="n">
@@ -7449,7 +7437,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n">
+      <c r="A185" s="1" t="n">
         <v>44287</v>
       </c>
       <c r="B185" t="n">
@@ -7487,7 +7475,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n">
+      <c r="A186" s="1" t="n">
         <v>44317</v>
       </c>
       <c r="B186" t="n">
@@ -7525,7 +7513,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n">
+      <c r="A187" s="1" t="n">
         <v>44348</v>
       </c>
       <c r="B187" t="n">
@@ -7563,7 +7551,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n">
+      <c r="A188" s="1" t="n">
         <v>44378</v>
       </c>
       <c r="B188" t="n">
@@ -7601,7 +7589,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n">
+      <c r="A189" s="1" t="n">
         <v>44409</v>
       </c>
       <c r="B189" t="n">
@@ -7639,7 +7627,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n">
+      <c r="A190" s="1" t="n">
         <v>44440</v>
       </c>
       <c r="B190" t="n">
@@ -7677,7 +7665,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="n">
+      <c r="A191" s="1" t="n">
         <v>44470</v>
       </c>
       <c r="B191" t="n">
@@ -7715,7 +7703,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n">
+      <c r="A192" s="1" t="n">
         <v>44501</v>
       </c>
       <c r="B192" t="n">
@@ -7753,7 +7741,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="n">
+      <c r="A193" s="1" t="n">
         <v>44531</v>
       </c>
       <c r="B193" t="n">
@@ -7791,7 +7779,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="n">
+      <c r="A194" s="1" t="n">
         <v>44562</v>
       </c>
       <c r="B194" t="n">
@@ -7829,7 +7817,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="n">
+      <c r="A195" s="1" t="n">
         <v>44593</v>
       </c>
       <c r="B195" t="n">
@@ -7867,7 +7855,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="n">
+      <c r="A196" s="1" t="n">
         <v>44621</v>
       </c>
       <c r="B196" t="n">
@@ -7905,7 +7893,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="n">
+      <c r="A197" s="1" t="n">
         <v>44652</v>
       </c>
       <c r="B197" t="n">
@@ -7943,7 +7931,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n">
+      <c r="A198" s="1" t="n">
         <v>44682</v>
       </c>
       <c r="B198" t="n">
@@ -7981,7 +7969,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="n">
+      <c r="A199" s="1" t="n">
         <v>44713</v>
       </c>
       <c r="B199" t="n">
@@ -8019,7 +8007,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n">
+      <c r="A200" s="1" t="n">
         <v>44743</v>
       </c>
       <c r="B200" t="n">
@@ -8057,7 +8045,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="n">
+      <c r="A201" s="1" t="n">
         <v>44774</v>
       </c>
       <c r="B201" t="n">
@@ -8095,7 +8083,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="n">
+      <c r="A202" s="1" t="n">
         <v>44805</v>
       </c>
       <c r="B202" t="n">
@@ -8133,7 +8121,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="n">
+      <c r="A203" s="1" t="n">
         <v>44835</v>
       </c>
       <c r="B203" t="n">
@@ -8171,7 +8159,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="n">
+      <c r="A204" s="1" t="n">
         <v>44866</v>
       </c>
       <c r="B204" t="n">
@@ -8209,7 +8197,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="n">
+      <c r="A205" s="1" t="n">
         <v>44896</v>
       </c>
       <c r="B205" t="n">
@@ -8247,7 +8235,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="n">
+      <c r="A206" s="1" t="n">
         <v>44927</v>
       </c>
       <c r="B206" t="n">
@@ -8285,7 +8273,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="n">
+      <c r="A207" s="1" t="n">
         <v>44958</v>
       </c>
       <c r="B207" t="n">
@@ -8323,7 +8311,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="n">
+      <c r="A208" s="1" t="n">
         <v>44986</v>
       </c>
       <c r="B208" t="n">
@@ -8361,7 +8349,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="n">
+      <c r="A209" s="1" t="n">
         <v>45017</v>
       </c>
       <c r="B209" t="n">
@@ -8399,7 +8387,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n">
+      <c r="A210" s="1" t="n">
         <v>45047</v>
       </c>
       <c r="B210" t="n">
@@ -8437,7 +8425,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="2" t="n">
+      <c r="A211" s="1" t="n">
         <v>45078</v>
       </c>
       <c r="B211" t="n">
@@ -8475,7 +8463,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="n">
+      <c r="A212" s="1" t="n">
         <v>45108</v>
       </c>
       <c r="B212" t="n">
@@ -8513,7 +8501,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="n">
+      <c r="A213" s="1" t="n">
         <v>45139</v>
       </c>
       <c r="B213" t="n">
@@ -8551,7 +8539,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="n">
+      <c r="A214" s="1" t="n">
         <v>45170</v>
       </c>
       <c r="B214" t="n">
@@ -8589,7 +8577,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="2" t="n">
+      <c r="A215" s="1" t="n">
         <v>45200</v>
       </c>
       <c r="B215" t="n">
@@ -8627,7 +8615,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="2" t="n">
+      <c r="A216" s="1" t="n">
         <v>45231</v>
       </c>
       <c r="B216" t="n">
@@ -8665,7 +8653,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="n">
+      <c r="A217" s="1" t="n">
         <v>45261</v>
       </c>
       <c r="B217" t="n">
@@ -8703,7 +8691,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="n">
+      <c r="A218" s="1" t="n">
         <v>45292</v>
       </c>
       <c r="B218" t="n">
@@ -8741,7 +8729,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="n">
+      <c r="A219" s="1" t="n">
         <v>45323</v>
       </c>
       <c r="B219" t="n">
@@ -8779,7 +8767,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="n">
+      <c r="A220" s="1" t="n">
         <v>45352</v>
       </c>
       <c r="B220" t="n">
@@ -8817,7 +8805,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="n">
+      <c r="A221" s="1" t="n">
         <v>45383</v>
       </c>
       <c r="B221" t="n">
@@ -8855,7 +8843,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="n">
+      <c r="A222" s="1" t="n">
         <v>45413</v>
       </c>
       <c r="B222" t="n">
@@ -8893,7 +8881,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="n">
+      <c r="A223" s="1" t="n">
         <v>45444</v>
       </c>
       <c r="B223" t="n">
@@ -8931,7 +8919,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="n">
+      <c r="A224" s="1" t="n">
         <v>45474</v>
       </c>
       <c r="B224" t="n">
@@ -8969,7 +8957,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="n">
+      <c r="A225" s="1" t="n">
         <v>45505</v>
       </c>
       <c r="B225" t="n">
@@ -9007,7 +8995,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="n">
+      <c r="A226" s="1" t="n">
         <v>45536</v>
       </c>
       <c r="B226" t="n">
@@ -9045,7 +9033,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="n">
+      <c r="A227" s="1" t="n">
         <v>45566</v>
       </c>
       <c r="B227" t="n">
@@ -9083,7 +9071,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="n">
+      <c r="A228" s="1" t="n">
         <v>45597</v>
       </c>
       <c r="B228" t="n">
@@ -9121,7 +9109,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="n">
+      <c r="A229" s="1" t="n">
         <v>45627</v>
       </c>
       <c r="B229" t="n">
@@ -9159,7 +9147,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="n">
+      <c r="A230" s="1" t="n">
         <v>45658</v>
       </c>
       <c r="B230" t="n">
@@ -9197,7 +9185,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="n">
+      <c r="A231" s="1" t="n">
         <v>45689</v>
       </c>
       <c r="B231" t="n">
@@ -9235,7 +9223,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="n">
+      <c r="A232" s="1" t="n">
         <v>45717</v>
       </c>
       <c r="B232" t="n">
@@ -9273,7 +9261,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="n">
+      <c r="A233" s="1" t="n">
         <v>45748</v>
       </c>
       <c r="B233" t="n">
@@ -9311,7 +9299,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="n">
+      <c r="A234" s="1" t="n">
         <v>45778</v>
       </c>
       <c r="B234" t="n">
@@ -9349,7 +9337,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="n">
+      <c r="A235" s="1" t="n">
         <v>45809</v>
       </c>
       <c r="B235" t="n">
@@ -9387,7 +9375,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="2" t="n">
+      <c r="A236" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="B236" t="n">
@@ -9425,7 +9413,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="2" t="n">
+      <c r="A237" s="1" t="n">
         <v>45870</v>
       </c>
       <c r="B237" t="n">
@@ -9463,7 +9451,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="2" t="n">
+      <c r="A238" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="B238" t="n">
@@ -9501,7 +9489,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="2" t="n">
+      <c r="A239" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="B239" t="n">
@@ -9539,7 +9527,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="2" t="n">
+      <c r="A240" s="1" t="n">
         <v>45962</v>
       </c>
       <c r="B240" t="n">
@@ -9577,7 +9565,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="2" t="n">
+      <c r="A241" s="1" t="n">
         <v>45992</v>
       </c>
       <c r="B241" t="n">
@@ -9615,7 +9603,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="2" t="n">
+      <c r="A242" s="1" t="n">
         <v>46023</v>
       </c>
       <c r="B242" t="n">
@@ -9653,7 +9641,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="n">
+      <c r="A243" s="1" t="n">
         <v>46054</v>
       </c>
       <c r="B243" t="n">
@@ -9691,7 +9679,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="2" t="n">
+      <c r="A244" s="1" t="n">
         <v>46082</v>
       </c>
       <c r="B244" t="n">
@@ -9729,7 +9717,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="2" t="n">
+      <c r="A245" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="B245" t="n">
@@ -9767,7 +9755,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="2" t="n">
+      <c r="A246" s="1" t="n">
         <v>46143</v>
       </c>
       <c r="B246" t="n">
@@ -9805,7 +9793,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="2" t="n">
+      <c r="A247" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="B247" t="n">

</xml_diff>

<commit_message>
Toplu veri güncelleme (yerel, 21.08.2026 15:05)
</commit_message>
<xml_diff>
--- a/butce/butce.xlsx
+++ b/butce/butce.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -417,73 +429,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L247"/>
+  <dimension ref="A1:L248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>tarih</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>yil</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ay</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>gelir</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>vergi</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>dolaysiz_vergi</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>dolayli_vergi</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>gider</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>faiz_haric_gider</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>faiz_gideri</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>faiz_disi_denge</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>denge</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>38718</v>
       </c>
       <c r="B2" t="n">
@@ -521,7 +533,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>38749</v>
       </c>
       <c r="B3" t="n">
@@ -559,7 +571,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>38777</v>
       </c>
       <c r="B4" t="n">
@@ -597,7 +609,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>38808</v>
       </c>
       <c r="B5" t="n">
@@ -635,7 +647,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>38838</v>
       </c>
       <c r="B6" t="n">
@@ -673,7 +685,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>38869</v>
       </c>
       <c r="B7" t="n">
@@ -711,7 +723,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>38899</v>
       </c>
       <c r="B8" t="n">
@@ -749,7 +761,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>38930</v>
       </c>
       <c r="B9" t="n">
@@ -787,7 +799,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>38961</v>
       </c>
       <c r="B10" t="n">
@@ -825,7 +837,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>38991</v>
       </c>
       <c r="B11" t="n">
@@ -863,7 +875,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>39022</v>
       </c>
       <c r="B12" t="n">
@@ -901,7 +913,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>39052</v>
       </c>
       <c r="B13" t="n">
@@ -939,7 +951,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>39083</v>
       </c>
       <c r="B14" t="n">
@@ -977,7 +989,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>39114</v>
       </c>
       <c r="B15" t="n">
@@ -1015,7 +1027,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>39142</v>
       </c>
       <c r="B16" t="n">
@@ -1053,7 +1065,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>39173</v>
       </c>
       <c r="B17" t="n">
@@ -1091,7 +1103,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>39203</v>
       </c>
       <c r="B18" t="n">
@@ -1129,7 +1141,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>39234</v>
       </c>
       <c r="B19" t="n">
@@ -1167,7 +1179,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>39264</v>
       </c>
       <c r="B20" t="n">
@@ -1205,7 +1217,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>39295</v>
       </c>
       <c r="B21" t="n">
@@ -1243,7 +1255,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>39326</v>
       </c>
       <c r="B22" t="n">
@@ -1281,7 +1293,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>39356</v>
       </c>
       <c r="B23" t="n">
@@ -1319,7 +1331,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>39387</v>
       </c>
       <c r="B24" t="n">
@@ -1357,7 +1369,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>39417</v>
       </c>
       <c r="B25" t="n">
@@ -1395,7 +1407,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>39448</v>
       </c>
       <c r="B26" t="n">
@@ -1433,7 +1445,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>39479</v>
       </c>
       <c r="B27" t="n">
@@ -1471,7 +1483,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>39508</v>
       </c>
       <c r="B28" t="n">
@@ -1509,7 +1521,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>39539</v>
       </c>
       <c r="B29" t="n">
@@ -1547,7 +1559,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>39569</v>
       </c>
       <c r="B30" t="n">
@@ -1585,7 +1597,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>39600</v>
       </c>
       <c r="B31" t="n">
@@ -1623,7 +1635,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>39630</v>
       </c>
       <c r="B32" t="n">
@@ -1661,7 +1673,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>39661</v>
       </c>
       <c r="B33" t="n">
@@ -1699,7 +1711,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>39692</v>
       </c>
       <c r="B34" t="n">
@@ -1737,7 +1749,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>39722</v>
       </c>
       <c r="B35" t="n">
@@ -1775,7 +1787,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>39753</v>
       </c>
       <c r="B36" t="n">
@@ -1813,7 +1825,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>39783</v>
       </c>
       <c r="B37" t="n">
@@ -1851,7 +1863,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>39814</v>
       </c>
       <c r="B38" t="n">
@@ -1889,7 +1901,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>39845</v>
       </c>
       <c r="B39" t="n">
@@ -1927,7 +1939,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>39873</v>
       </c>
       <c r="B40" t="n">
@@ -1965,7 +1977,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>39904</v>
       </c>
       <c r="B41" t="n">
@@ -2003,7 +2015,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>39934</v>
       </c>
       <c r="B42" t="n">
@@ -2041,7 +2053,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>39965</v>
       </c>
       <c r="B43" t="n">
@@ -2079,7 +2091,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>39995</v>
       </c>
       <c r="B44" t="n">
@@ -2117,7 +2129,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>40026</v>
       </c>
       <c r="B45" t="n">
@@ -2155,7 +2167,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>40057</v>
       </c>
       <c r="B46" t="n">
@@ -2193,7 +2205,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>40087</v>
       </c>
       <c r="B47" t="n">
@@ -2231,7 +2243,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>40118</v>
       </c>
       <c r="B48" t="n">
@@ -2269,7 +2281,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>40148</v>
       </c>
       <c r="B49" t="n">
@@ -2307,7 +2319,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>40179</v>
       </c>
       <c r="B50" t="n">
@@ -2345,7 +2357,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>40210</v>
       </c>
       <c r="B51" t="n">
@@ -2383,7 +2395,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>40238</v>
       </c>
       <c r="B52" t="n">
@@ -2421,7 +2433,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>40269</v>
       </c>
       <c r="B53" t="n">
@@ -2459,7 +2471,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>40299</v>
       </c>
       <c r="B54" t="n">
@@ -2497,7 +2509,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>40330</v>
       </c>
       <c r="B55" t="n">
@@ -2535,7 +2547,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>40360</v>
       </c>
       <c r="B56" t="n">
@@ -2573,7 +2585,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>40391</v>
       </c>
       <c r="B57" t="n">
@@ -2611,7 +2623,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>40422</v>
       </c>
       <c r="B58" t="n">
@@ -2649,7 +2661,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>40452</v>
       </c>
       <c r="B59" t="n">
@@ -2687,7 +2699,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>40483</v>
       </c>
       <c r="B60" t="n">
@@ -2725,7 +2737,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>40513</v>
       </c>
       <c r="B61" t="n">
@@ -2763,7 +2775,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>40544</v>
       </c>
       <c r="B62" t="n">
@@ -2801,7 +2813,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" s="2" t="n">
         <v>40575</v>
       </c>
       <c r="B63" t="n">
@@ -2839,7 +2851,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" s="2" t="n">
         <v>40603</v>
       </c>
       <c r="B64" t="n">
@@ -2877,7 +2889,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" s="2" t="n">
         <v>40634</v>
       </c>
       <c r="B65" t="n">
@@ -2915,7 +2927,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="2" t="n">
         <v>40664</v>
       </c>
       <c r="B66" t="n">
@@ -2953,7 +2965,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="2" t="n">
         <v>40695</v>
       </c>
       <c r="B67" t="n">
@@ -2991,7 +3003,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="2" t="n">
         <v>40725</v>
       </c>
       <c r="B68" t="n">
@@ -3029,7 +3041,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="2" t="n">
         <v>40756</v>
       </c>
       <c r="B69" t="n">
@@ -3067,7 +3079,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="2" t="n">
         <v>40787</v>
       </c>
       <c r="B70" t="n">
@@ -3105,7 +3117,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="2" t="n">
         <v>40817</v>
       </c>
       <c r="B71" t="n">
@@ -3143,7 +3155,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" s="2" t="n">
         <v>40848</v>
       </c>
       <c r="B72" t="n">
@@ -3181,7 +3193,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="2" t="n">
         <v>40878</v>
       </c>
       <c r="B73" t="n">
@@ -3219,7 +3231,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="2" t="n">
         <v>40909</v>
       </c>
       <c r="B74" t="n">
@@ -3257,7 +3269,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="2" t="n">
         <v>40940</v>
       </c>
       <c r="B75" t="n">
@@ -3295,7 +3307,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="2" t="n">
         <v>40969</v>
       </c>
       <c r="B76" t="n">
@@ -3333,7 +3345,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="2" t="n">
         <v>41000</v>
       </c>
       <c r="B77" t="n">
@@ -3371,7 +3383,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="2" t="n">
         <v>41030</v>
       </c>
       <c r="B78" t="n">
@@ -3409,7 +3421,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="2" t="n">
         <v>41061</v>
       </c>
       <c r="B79" t="n">
@@ -3447,7 +3459,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="2" t="n">
         <v>41091</v>
       </c>
       <c r="B80" t="n">
@@ -3485,7 +3497,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" s="2" t="n">
         <v>41122</v>
       </c>
       <c r="B81" t="n">
@@ -3523,7 +3535,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" s="2" t="n">
         <v>41153</v>
       </c>
       <c r="B82" t="n">
@@ -3561,7 +3573,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="2" t="n">
         <v>41183</v>
       </c>
       <c r="B83" t="n">
@@ -3599,7 +3611,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="2" t="n">
         <v>41214</v>
       </c>
       <c r="B84" t="n">
@@ -3637,7 +3649,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" s="2" t="n">
         <v>41244</v>
       </c>
       <c r="B85" t="n">
@@ -3675,7 +3687,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" s="2" t="n">
         <v>41275</v>
       </c>
       <c r="B86" t="n">
@@ -3713,7 +3725,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="2" t="n">
         <v>41306</v>
       </c>
       <c r="B87" t="n">
@@ -3751,7 +3763,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="2" t="n">
         <v>41334</v>
       </c>
       <c r="B88" t="n">
@@ -3789,7 +3801,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="2" t="n">
         <v>41365</v>
       </c>
       <c r="B89" t="n">
@@ -3827,7 +3839,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="2" t="n">
         <v>41395</v>
       </c>
       <c r="B90" t="n">
@@ -3865,7 +3877,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="2" t="n">
         <v>41426</v>
       </c>
       <c r="B91" t="n">
@@ -3903,7 +3915,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="2" t="n">
         <v>41456</v>
       </c>
       <c r="B92" t="n">
@@ -3941,7 +3953,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" s="2" t="n">
         <v>41487</v>
       </c>
       <c r="B93" t="n">
@@ -3979,7 +3991,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" s="2" t="n">
         <v>41518</v>
       </c>
       <c r="B94" t="n">
@@ -4017,7 +4029,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" s="2" t="n">
         <v>41548</v>
       </c>
       <c r="B95" t="n">
@@ -4055,7 +4067,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" s="2" t="n">
         <v>41579</v>
       </c>
       <c r="B96" t="n">
@@ -4093,7 +4105,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" s="2" t="n">
         <v>41609</v>
       </c>
       <c r="B97" t="n">
@@ -4131,7 +4143,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" s="2" t="n">
         <v>41640</v>
       </c>
       <c r="B98" t="n">
@@ -4169,7 +4181,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" s="2" t="n">
         <v>41671</v>
       </c>
       <c r="B99" t="n">
@@ -4207,7 +4219,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" s="2" t="n">
         <v>41699</v>
       </c>
       <c r="B100" t="n">
@@ -4245,7 +4257,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" s="2" t="n">
         <v>41730</v>
       </c>
       <c r="B101" t="n">
@@ -4283,7 +4295,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" s="2" t="n">
         <v>41760</v>
       </c>
       <c r="B102" t="n">
@@ -4321,7 +4333,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" s="2" t="n">
         <v>41791</v>
       </c>
       <c r="B103" t="n">
@@ -4359,7 +4371,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" s="2" t="n">
         <v>41821</v>
       </c>
       <c r="B104" t="n">
@@ -4397,7 +4409,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" s="2" t="n">
         <v>41852</v>
       </c>
       <c r="B105" t="n">
@@ -4435,7 +4447,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" s="2" t="n">
         <v>41883</v>
       </c>
       <c r="B106" t="n">
@@ -4473,7 +4485,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" s="2" t="n">
         <v>41913</v>
       </c>
       <c r="B107" t="n">
@@ -4511,7 +4523,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" s="2" t="n">
         <v>41944</v>
       </c>
       <c r="B108" t="n">
@@ -4549,7 +4561,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" s="2" t="n">
         <v>41974</v>
       </c>
       <c r="B109" t="n">
@@ -4587,7 +4599,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" s="2" t="n">
         <v>42005</v>
       </c>
       <c r="B110" t="n">
@@ -4625,7 +4637,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" s="2" t="n">
         <v>42036</v>
       </c>
       <c r="B111" t="n">
@@ -4663,7 +4675,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" s="2" t="n">
         <v>42064</v>
       </c>
       <c r="B112" t="n">
@@ -4701,7 +4713,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" s="2" t="n">
         <v>42095</v>
       </c>
       <c r="B113" t="n">
@@ -4739,7 +4751,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" s="2" t="n">
         <v>42125</v>
       </c>
       <c r="B114" t="n">
@@ -4777,7 +4789,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" s="2" t="n">
         <v>42156</v>
       </c>
       <c r="B115" t="n">
@@ -4815,7 +4827,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" s="2" t="n">
         <v>42186</v>
       </c>
       <c r="B116" t="n">
@@ -4853,7 +4865,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" s="2" t="n">
         <v>42217</v>
       </c>
       <c r="B117" t="n">
@@ -4891,7 +4903,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" s="2" t="n">
         <v>42248</v>
       </c>
       <c r="B118" t="n">
@@ -4929,7 +4941,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" s="2" t="n">
         <v>42278</v>
       </c>
       <c r="B119" t="n">
@@ -4967,7 +4979,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" s="2" t="n">
         <v>42309</v>
       </c>
       <c r="B120" t="n">
@@ -5005,7 +5017,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" s="2" t="n">
         <v>42339</v>
       </c>
       <c r="B121" t="n">
@@ -5043,7 +5055,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" s="2" t="n">
         <v>42370</v>
       </c>
       <c r="B122" t="n">
@@ -5081,7 +5093,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" s="2" t="n">
         <v>42401</v>
       </c>
       <c r="B123" t="n">
@@ -5119,7 +5131,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" s="2" t="n">
         <v>42430</v>
       </c>
       <c r="B124" t="n">
@@ -5157,7 +5169,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" s="2" t="n">
         <v>42461</v>
       </c>
       <c r="B125" t="n">
@@ -5195,7 +5207,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" s="2" t="n">
         <v>42491</v>
       </c>
       <c r="B126" t="n">
@@ -5233,7 +5245,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" s="2" t="n">
         <v>42522</v>
       </c>
       <c r="B127" t="n">
@@ -5271,7 +5283,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" s="2" t="n">
         <v>42552</v>
       </c>
       <c r="B128" t="n">
@@ -5309,7 +5321,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" s="2" t="n">
         <v>42583</v>
       </c>
       <c r="B129" t="n">
@@ -5347,7 +5359,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
+      <c r="A130" s="2" t="n">
         <v>42614</v>
       </c>
       <c r="B130" t="n">
@@ -5385,7 +5397,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
+      <c r="A131" s="2" t="n">
         <v>42644</v>
       </c>
       <c r="B131" t="n">
@@ -5423,7 +5435,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
+      <c r="A132" s="2" t="n">
         <v>42675</v>
       </c>
       <c r="B132" t="n">
@@ -5461,7 +5473,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
+      <c r="A133" s="2" t="n">
         <v>42705</v>
       </c>
       <c r="B133" t="n">
@@ -5499,7 +5511,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
+      <c r="A134" s="2" t="n">
         <v>42736</v>
       </c>
       <c r="B134" t="n">
@@ -5537,7 +5549,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
+      <c r="A135" s="2" t="n">
         <v>42767</v>
       </c>
       <c r="B135" t="n">
@@ -5575,7 +5587,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
+      <c r="A136" s="2" t="n">
         <v>42795</v>
       </c>
       <c r="B136" t="n">
@@ -5613,7 +5625,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
+      <c r="A137" s="2" t="n">
         <v>42826</v>
       </c>
       <c r="B137" t="n">
@@ -5651,7 +5663,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
+      <c r="A138" s="2" t="n">
         <v>42856</v>
       </c>
       <c r="B138" t="n">
@@ -5689,7 +5701,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="n">
+      <c r="A139" s="2" t="n">
         <v>42887</v>
       </c>
       <c r="B139" t="n">
@@ -5727,7 +5739,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="n">
+      <c r="A140" s="2" t="n">
         <v>42917</v>
       </c>
       <c r="B140" t="n">
@@ -5765,7 +5777,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="n">
+      <c r="A141" s="2" t="n">
         <v>42948</v>
       </c>
       <c r="B141" t="n">
@@ -5803,7 +5815,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="n">
+      <c r="A142" s="2" t="n">
         <v>42979</v>
       </c>
       <c r="B142" t="n">
@@ -5841,7 +5853,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="n">
+      <c r="A143" s="2" t="n">
         <v>43009</v>
       </c>
       <c r="B143" t="n">
@@ -5879,7 +5891,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="n">
+      <c r="A144" s="2" t="n">
         <v>43040</v>
       </c>
       <c r="B144" t="n">
@@ -5917,7 +5929,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="n">
+      <c r="A145" s="2" t="n">
         <v>43070</v>
       </c>
       <c r="B145" t="n">
@@ -5955,7 +5967,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="1" t="n">
+      <c r="A146" s="2" t="n">
         <v>43101</v>
       </c>
       <c r="B146" t="n">
@@ -5993,7 +6005,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="1" t="n">
+      <c r="A147" s="2" t="n">
         <v>43132</v>
       </c>
       <c r="B147" t="n">
@@ -6031,7 +6043,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="1" t="n">
+      <c r="A148" s="2" t="n">
         <v>43160</v>
       </c>
       <c r="B148" t="n">
@@ -6069,7 +6081,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="1" t="n">
+      <c r="A149" s="2" t="n">
         <v>43191</v>
       </c>
       <c r="B149" t="n">
@@ -6107,7 +6119,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="1" t="n">
+      <c r="A150" s="2" t="n">
         <v>43221</v>
       </c>
       <c r="B150" t="n">
@@ -6145,7 +6157,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="1" t="n">
+      <c r="A151" s="2" t="n">
         <v>43252</v>
       </c>
       <c r="B151" t="n">
@@ -6183,7 +6195,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="1" t="n">
+      <c r="A152" s="2" t="n">
         <v>43282</v>
       </c>
       <c r="B152" t="n">
@@ -6221,7 +6233,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="1" t="n">
+      <c r="A153" s="2" t="n">
         <v>43313</v>
       </c>
       <c r="B153" t="n">
@@ -6259,7 +6271,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="1" t="n">
+      <c r="A154" s="2" t="n">
         <v>43344</v>
       </c>
       <c r="B154" t="n">
@@ -6297,7 +6309,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="1" t="n">
+      <c r="A155" s="2" t="n">
         <v>43374</v>
       </c>
       <c r="B155" t="n">
@@ -6335,7 +6347,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="1" t="n">
+      <c r="A156" s="2" t="n">
         <v>43405</v>
       </c>
       <c r="B156" t="n">
@@ -6373,7 +6385,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="1" t="n">
+      <c r="A157" s="2" t="n">
         <v>43435</v>
       </c>
       <c r="B157" t="n">
@@ -6411,7 +6423,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="1" t="n">
+      <c r="A158" s="2" t="n">
         <v>43466</v>
       </c>
       <c r="B158" t="n">
@@ -6449,7 +6461,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="1" t="n">
+      <c r="A159" s="2" t="n">
         <v>43497</v>
       </c>
       <c r="B159" t="n">
@@ -6487,7 +6499,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="1" t="n">
+      <c r="A160" s="2" t="n">
         <v>43525</v>
       </c>
       <c r="B160" t="n">
@@ -6525,7 +6537,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="1" t="n">
+      <c r="A161" s="2" t="n">
         <v>43556</v>
       </c>
       <c r="B161" t="n">
@@ -6563,7 +6575,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="1" t="n">
+      <c r="A162" s="2" t="n">
         <v>43586</v>
       </c>
       <c r="B162" t="n">
@@ -6601,7 +6613,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="1" t="n">
+      <c r="A163" s="2" t="n">
         <v>43617</v>
       </c>
       <c r="B163" t="n">
@@ -6639,7 +6651,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="1" t="n">
+      <c r="A164" s="2" t="n">
         <v>43647</v>
       </c>
       <c r="B164" t="n">
@@ -6677,7 +6689,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="1" t="n">
+      <c r="A165" s="2" t="n">
         <v>43678</v>
       </c>
       <c r="B165" t="n">
@@ -6715,7 +6727,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="1" t="n">
+      <c r="A166" s="2" t="n">
         <v>43709</v>
       </c>
       <c r="B166" t="n">
@@ -6753,7 +6765,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="1" t="n">
+      <c r="A167" s="2" t="n">
         <v>43739</v>
       </c>
       <c r="B167" t="n">
@@ -6791,7 +6803,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="1" t="n">
+      <c r="A168" s="2" t="n">
         <v>43770</v>
       </c>
       <c r="B168" t="n">
@@ -6829,7 +6841,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="1" t="n">
+      <c r="A169" s="2" t="n">
         <v>43800</v>
       </c>
       <c r="B169" t="n">
@@ -6867,7 +6879,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="1" t="n">
+      <c r="A170" s="2" t="n">
         <v>43831</v>
       </c>
       <c r="B170" t="n">
@@ -6905,7 +6917,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="1" t="n">
+      <c r="A171" s="2" t="n">
         <v>43862</v>
       </c>
       <c r="B171" t="n">
@@ -6943,7 +6955,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="1" t="n">
+      <c r="A172" s="2" t="n">
         <v>43891</v>
       </c>
       <c r="B172" t="n">
@@ -6981,7 +6993,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="1" t="n">
+      <c r="A173" s="2" t="n">
         <v>43922</v>
       </c>
       <c r="B173" t="n">
@@ -7019,7 +7031,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="1" t="n">
+      <c r="A174" s="2" t="n">
         <v>43952</v>
       </c>
       <c r="B174" t="n">
@@ -7057,7 +7069,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="1" t="n">
+      <c r="A175" s="2" t="n">
         <v>43983</v>
       </c>
       <c r="B175" t="n">
@@ -7095,7 +7107,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="1" t="n">
+      <c r="A176" s="2" t="n">
         <v>44013</v>
       </c>
       <c r="B176" t="n">
@@ -7133,7 +7145,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="1" t="n">
+      <c r="A177" s="2" t="n">
         <v>44044</v>
       </c>
       <c r="B177" t="n">
@@ -7171,7 +7183,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="1" t="n">
+      <c r="A178" s="2" t="n">
         <v>44075</v>
       </c>
       <c r="B178" t="n">
@@ -7209,7 +7221,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="1" t="n">
+      <c r="A179" s="2" t="n">
         <v>44105</v>
       </c>
       <c r="B179" t="n">
@@ -7247,7 +7259,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="1" t="n">
+      <c r="A180" s="2" t="n">
         <v>44136</v>
       </c>
       <c r="B180" t="n">
@@ -7285,7 +7297,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="1" t="n">
+      <c r="A181" s="2" t="n">
         <v>44166</v>
       </c>
       <c r="B181" t="n">
@@ -7323,7 +7335,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="1" t="n">
+      <c r="A182" s="2" t="n">
         <v>44197</v>
       </c>
       <c r="B182" t="n">
@@ -7361,7 +7373,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="1" t="n">
+      <c r="A183" s="2" t="n">
         <v>44228</v>
       </c>
       <c r="B183" t="n">
@@ -7399,7 +7411,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="1" t="n">
+      <c r="A184" s="2" t="n">
         <v>44256</v>
       </c>
       <c r="B184" t="n">
@@ -7437,7 +7449,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="1" t="n">
+      <c r="A185" s="2" t="n">
         <v>44287</v>
       </c>
       <c r="B185" t="n">
@@ -7475,7 +7487,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="1" t="n">
+      <c r="A186" s="2" t="n">
         <v>44317</v>
       </c>
       <c r="B186" t="n">
@@ -7513,7 +7525,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="1" t="n">
+      <c r="A187" s="2" t="n">
         <v>44348</v>
       </c>
       <c r="B187" t="n">
@@ -7551,7 +7563,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="1" t="n">
+      <c r="A188" s="2" t="n">
         <v>44378</v>
       </c>
       <c r="B188" t="n">
@@ -7589,7 +7601,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="1" t="n">
+      <c r="A189" s="2" t="n">
         <v>44409</v>
       </c>
       <c r="B189" t="n">
@@ -7627,7 +7639,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="1" t="n">
+      <c r="A190" s="2" t="n">
         <v>44440</v>
       </c>
       <c r="B190" t="n">
@@ -7665,7 +7677,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="1" t="n">
+      <c r="A191" s="2" t="n">
         <v>44470</v>
       </c>
       <c r="B191" t="n">
@@ -7703,7 +7715,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="1" t="n">
+      <c r="A192" s="2" t="n">
         <v>44501</v>
       </c>
       <c r="B192" t="n">
@@ -7741,7 +7753,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="1" t="n">
+      <c r="A193" s="2" t="n">
         <v>44531</v>
       </c>
       <c r="B193" t="n">
@@ -7779,7 +7791,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="1" t="n">
+      <c r="A194" s="2" t="n">
         <v>44562</v>
       </c>
       <c r="B194" t="n">
@@ -7817,7 +7829,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="1" t="n">
+      <c r="A195" s="2" t="n">
         <v>44593</v>
       </c>
       <c r="B195" t="n">
@@ -7855,7 +7867,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="1" t="n">
+      <c r="A196" s="2" t="n">
         <v>44621</v>
       </c>
       <c r="B196" t="n">
@@ -7893,7 +7905,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="1" t="n">
+      <c r="A197" s="2" t="n">
         <v>44652</v>
       </c>
       <c r="B197" t="n">
@@ -7931,7 +7943,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="1" t="n">
+      <c r="A198" s="2" t="n">
         <v>44682</v>
       </c>
       <c r="B198" t="n">
@@ -7969,7 +7981,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="1" t="n">
+      <c r="A199" s="2" t="n">
         <v>44713</v>
       </c>
       <c r="B199" t="n">
@@ -8007,7 +8019,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="1" t="n">
+      <c r="A200" s="2" t="n">
         <v>44743</v>
       </c>
       <c r="B200" t="n">
@@ -8045,7 +8057,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="1" t="n">
+      <c r="A201" s="2" t="n">
         <v>44774</v>
       </c>
       <c r="B201" t="n">
@@ -8083,7 +8095,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="1" t="n">
+      <c r="A202" s="2" t="n">
         <v>44805</v>
       </c>
       <c r="B202" t="n">
@@ -8121,7 +8133,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="1" t="n">
+      <c r="A203" s="2" t="n">
         <v>44835</v>
       </c>
       <c r="B203" t="n">
@@ -8159,7 +8171,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="1" t="n">
+      <c r="A204" s="2" t="n">
         <v>44866</v>
       </c>
       <c r="B204" t="n">
@@ -8197,7 +8209,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="1" t="n">
+      <c r="A205" s="2" t="n">
         <v>44896</v>
       </c>
       <c r="B205" t="n">
@@ -8235,7 +8247,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="1" t="n">
+      <c r="A206" s="2" t="n">
         <v>44927</v>
       </c>
       <c r="B206" t="n">
@@ -8273,7 +8285,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="1" t="n">
+      <c r="A207" s="2" t="n">
         <v>44958</v>
       </c>
       <c r="B207" t="n">
@@ -8311,7 +8323,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="1" t="n">
+      <c r="A208" s="2" t="n">
         <v>44986</v>
       </c>
       <c r="B208" t="n">
@@ -8349,7 +8361,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="1" t="n">
+      <c r="A209" s="2" t="n">
         <v>45017</v>
       </c>
       <c r="B209" t="n">
@@ -8387,7 +8399,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="1" t="n">
+      <c r="A210" s="2" t="n">
         <v>45047</v>
       </c>
       <c r="B210" t="n">
@@ -8425,7 +8437,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="1" t="n">
+      <c r="A211" s="2" t="n">
         <v>45078</v>
       </c>
       <c r="B211" t="n">
@@ -8463,7 +8475,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="1" t="n">
+      <c r="A212" s="2" t="n">
         <v>45108</v>
       </c>
       <c r="B212" t="n">
@@ -8501,7 +8513,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="1" t="n">
+      <c r="A213" s="2" t="n">
         <v>45139</v>
       </c>
       <c r="B213" t="n">
@@ -8539,7 +8551,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="1" t="n">
+      <c r="A214" s="2" t="n">
         <v>45170</v>
       </c>
       <c r="B214" t="n">
@@ -8577,7 +8589,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="1" t="n">
+      <c r="A215" s="2" t="n">
         <v>45200</v>
       </c>
       <c r="B215" t="n">
@@ -8615,7 +8627,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="1" t="n">
+      <c r="A216" s="2" t="n">
         <v>45231</v>
       </c>
       <c r="B216" t="n">
@@ -8653,7 +8665,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="1" t="n">
+      <c r="A217" s="2" t="n">
         <v>45261</v>
       </c>
       <c r="B217" t="n">
@@ -8691,7 +8703,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="1" t="n">
+      <c r="A218" s="2" t="n">
         <v>45292</v>
       </c>
       <c r="B218" t="n">
@@ -8729,7 +8741,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="1" t="n">
+      <c r="A219" s="2" t="n">
         <v>45323</v>
       </c>
       <c r="B219" t="n">
@@ -8767,7 +8779,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="1" t="n">
+      <c r="A220" s="2" t="n">
         <v>45352</v>
       </c>
       <c r="B220" t="n">
@@ -8805,7 +8817,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="1" t="n">
+      <c r="A221" s="2" t="n">
         <v>45383</v>
       </c>
       <c r="B221" t="n">
@@ -8843,7 +8855,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="1" t="n">
+      <c r="A222" s="2" t="n">
         <v>45413</v>
       </c>
       <c r="B222" t="n">
@@ -8881,7 +8893,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="1" t="n">
+      <c r="A223" s="2" t="n">
         <v>45444</v>
       </c>
       <c r="B223" t="n">
@@ -8919,7 +8931,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="1" t="n">
+      <c r="A224" s="2" t="n">
         <v>45474</v>
       </c>
       <c r="B224" t="n">
@@ -8957,7 +8969,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="1" t="n">
+      <c r="A225" s="2" t="n">
         <v>45505</v>
       </c>
       <c r="B225" t="n">
@@ -8995,7 +9007,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="1" t="n">
+      <c r="A226" s="2" t="n">
         <v>45536</v>
       </c>
       <c r="B226" t="n">
@@ -9033,7 +9045,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="1" t="n">
+      <c r="A227" s="2" t="n">
         <v>45566</v>
       </c>
       <c r="B227" t="n">
@@ -9071,7 +9083,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="1" t="n">
+      <c r="A228" s="2" t="n">
         <v>45597</v>
       </c>
       <c r="B228" t="n">
@@ -9109,7 +9121,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="1" t="n">
+      <c r="A229" s="2" t="n">
         <v>45627</v>
       </c>
       <c r="B229" t="n">
@@ -9147,7 +9159,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="1" t="n">
+      <c r="A230" s="2" t="n">
         <v>45658</v>
       </c>
       <c r="B230" t="n">
@@ -9185,7 +9197,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="1" t="n">
+      <c r="A231" s="2" t="n">
         <v>45689</v>
       </c>
       <c r="B231" t="n">
@@ -9223,7 +9235,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="1" t="n">
+      <c r="A232" s="2" t="n">
         <v>45717</v>
       </c>
       <c r="B232" t="n">
@@ -9261,7 +9273,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="1" t="n">
+      <c r="A233" s="2" t="n">
         <v>45748</v>
       </c>
       <c r="B233" t="n">
@@ -9299,7 +9311,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="1" t="n">
+      <c r="A234" s="2" t="n">
         <v>45778</v>
       </c>
       <c r="B234" t="n">
@@ -9337,7 +9349,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="1" t="n">
+      <c r="A235" s="2" t="n">
         <v>45809</v>
       </c>
       <c r="B235" t="n">
@@ -9375,7 +9387,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="1" t="n">
+      <c r="A236" s="2" t="n">
         <v>45839</v>
       </c>
       <c r="B236" t="n">
@@ -9413,7 +9425,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="1" t="n">
+      <c r="A237" s="2" t="n">
         <v>45870</v>
       </c>
       <c r="B237" t="n">
@@ -9451,7 +9463,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="1" t="n">
+      <c r="A238" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="B238" t="n">
@@ -9489,7 +9501,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="1" t="n">
+      <c r="A239" s="2" t="n">
         <v>45931</v>
       </c>
       <c r="B239" t="n">
@@ -9527,7 +9539,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="1" t="n">
+      <c r="A240" s="2" t="n">
         <v>45962</v>
       </c>
       <c r="B240" t="n">
@@ -9565,7 +9577,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="1" t="n">
+      <c r="A241" s="2" t="n">
         <v>45992</v>
       </c>
       <c r="B241" t="n">
@@ -9603,7 +9615,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="1" t="n">
+      <c r="A242" s="2" t="n">
         <v>46023</v>
       </c>
       <c r="B242" t="n">
@@ -9641,7 +9653,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="1" t="n">
+      <c r="A243" s="2" t="n">
         <v>46054</v>
       </c>
       <c r="B243" t="n">
@@ -9679,7 +9691,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="1" t="n">
+      <c r="A244" s="2" t="n">
         <v>46082</v>
       </c>
       <c r="B244" t="n">
@@ -9717,7 +9729,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="1" t="n">
+      <c r="A245" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="B245" t="n">
@@ -9755,7 +9767,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="1" t="n">
+      <c r="A246" s="2" t="n">
         <v>46143</v>
       </c>
       <c r="B246" t="n">
@@ -9793,7 +9805,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="1" t="n">
+      <c r="A247" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="B247" t="n">
@@ -9828,6 +9840,44 @@
       </c>
       <c r="L247" t="n">
         <v>114163.5484753808</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B248" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C248" t="n">
+        <v>7</v>
+      </c>
+      <c r="D248" t="n">
+        <v>1412397.48453032</v>
+      </c>
+      <c r="E248" t="n">
+        <v>1234841.86735525</v>
+      </c>
+      <c r="F248" t="n">
+        <v>480251.57667159</v>
+      </c>
+      <c r="G248" t="n">
+        <v>754590.29068366</v>
+      </c>
+      <c r="H248" t="n">
+        <v>1790502.39061571</v>
+      </c>
+      <c r="I248" t="n">
+        <v>1463738.0229466</v>
+      </c>
+      <c r="J248" t="n">
+        <v>326764.36766911</v>
+      </c>
+      <c r="K248" t="n">
+        <v>-51340.53841628041</v>
+      </c>
+      <c r="L248" t="n">
+        <v>-378104.9060853904</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Otomatik veri güncelleme (27.08.2026 21:20 UTC)
</commit_message>
<xml_diff>
--- a/butce/butce.xlsx
+++ b/butce/butce.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,69 +421,69 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tarih</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>yil</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ay</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>gelir</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>vergi</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>dolaysiz_vergi</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>dolayli_vergi</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>gider</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>faiz_haric_gider</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>faiz_gideri</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>faiz_disi_denge</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>denge</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>38718</v>
       </c>
       <c r="B2" t="n">
@@ -533,7 +521,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>38749</v>
       </c>
       <c r="B3" t="n">
@@ -571,7 +559,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>38777</v>
       </c>
       <c r="B4" t="n">
@@ -609,7 +597,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>38808</v>
       </c>
       <c r="B5" t="n">
@@ -647,7 +635,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>38838</v>
       </c>
       <c r="B6" t="n">
@@ -685,7 +673,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>38869</v>
       </c>
       <c r="B7" t="n">
@@ -723,7 +711,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>38899</v>
       </c>
       <c r="B8" t="n">
@@ -761,7 +749,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>38930</v>
       </c>
       <c r="B9" t="n">
@@ -799,7 +787,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>38961</v>
       </c>
       <c r="B10" t="n">
@@ -837,7 +825,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>38991</v>
       </c>
       <c r="B11" t="n">
@@ -875,7 +863,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>39022</v>
       </c>
       <c r="B12" t="n">
@@ -913,7 +901,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>39052</v>
       </c>
       <c r="B13" t="n">
@@ -951,7 +939,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>39083</v>
       </c>
       <c r="B14" t="n">
@@ -989,7 +977,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>39114</v>
       </c>
       <c r="B15" t="n">
@@ -1027,7 +1015,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>39142</v>
       </c>
       <c r="B16" t="n">
@@ -1065,7 +1053,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>39173</v>
       </c>
       <c r="B17" t="n">
@@ -1103,7 +1091,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>39203</v>
       </c>
       <c r="B18" t="n">
@@ -1141,7 +1129,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>39234</v>
       </c>
       <c r="B19" t="n">
@@ -1179,7 +1167,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>39264</v>
       </c>
       <c r="B20" t="n">
@@ -1217,7 +1205,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>39295</v>
       </c>
       <c r="B21" t="n">
@@ -1255,7 +1243,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>39326</v>
       </c>
       <c r="B22" t="n">
@@ -1293,7 +1281,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>39356</v>
       </c>
       <c r="B23" t="n">
@@ -1331,7 +1319,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>39387</v>
       </c>
       <c r="B24" t="n">
@@ -1369,7 +1357,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>39417</v>
       </c>
       <c r="B25" t="n">
@@ -1407,7 +1395,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>39448</v>
       </c>
       <c r="B26" t="n">
@@ -1445,7 +1433,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="1" t="n">
         <v>39479</v>
       </c>
       <c r="B27" t="n">
@@ -1483,7 +1471,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>39508</v>
       </c>
       <c r="B28" t="n">
@@ -1521,7 +1509,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>39539</v>
       </c>
       <c r="B29" t="n">
@@ -1559,7 +1547,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>39569</v>
       </c>
       <c r="B30" t="n">
@@ -1597,7 +1585,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>39600</v>
       </c>
       <c r="B31" t="n">
@@ -1635,7 +1623,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>39630</v>
       </c>
       <c r="B32" t="n">
@@ -1673,7 +1661,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>39661</v>
       </c>
       <c r="B33" t="n">
@@ -1711,7 +1699,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>39692</v>
       </c>
       <c r="B34" t="n">
@@ -1749,7 +1737,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>39722</v>
       </c>
       <c r="B35" t="n">
@@ -1787,7 +1775,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>39753</v>
       </c>
       <c r="B36" t="n">
@@ -1825,7 +1813,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>39783</v>
       </c>
       <c r="B37" t="n">
@@ -1863,7 +1851,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>39814</v>
       </c>
       <c r="B38" t="n">
@@ -1901,7 +1889,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>39845</v>
       </c>
       <c r="B39" t="n">
@@ -1939,7 +1927,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>39873</v>
       </c>
       <c r="B40" t="n">
@@ -1977,7 +1965,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>39904</v>
       </c>
       <c r="B41" t="n">
@@ -2015,7 +2003,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>39934</v>
       </c>
       <c r="B42" t="n">
@@ -2053,7 +2041,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>39965</v>
       </c>
       <c r="B43" t="n">
@@ -2091,7 +2079,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>39995</v>
       </c>
       <c r="B44" t="n">
@@ -2129,7 +2117,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>40026</v>
       </c>
       <c r="B45" t="n">
@@ -2167,7 +2155,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>40057</v>
       </c>
       <c r="B46" t="n">
@@ -2205,7 +2193,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>40087</v>
       </c>
       <c r="B47" t="n">
@@ -2243,7 +2231,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>40118</v>
       </c>
       <c r="B48" t="n">
@@ -2281,7 +2269,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>40148</v>
       </c>
       <c r="B49" t="n">
@@ -2319,7 +2307,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>40179</v>
       </c>
       <c r="B50" t="n">
@@ -2357,7 +2345,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>40210</v>
       </c>
       <c r="B51" t="n">
@@ -2395,7 +2383,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>40238</v>
       </c>
       <c r="B52" t="n">
@@ -2433,7 +2421,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>40269</v>
       </c>
       <c r="B53" t="n">
@@ -2471,7 +2459,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>40299</v>
       </c>
       <c r="B54" t="n">
@@ -2509,7 +2497,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>40330</v>
       </c>
       <c r="B55" t="n">
@@ -2547,7 +2535,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>40360</v>
       </c>
       <c r="B56" t="n">
@@ -2585,7 +2573,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>40391</v>
       </c>
       <c r="B57" t="n">
@@ -2623,7 +2611,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>40422</v>
       </c>
       <c r="B58" t="n">
@@ -2661,7 +2649,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>40452</v>
       </c>
       <c r="B59" t="n">
@@ -2699,7 +2687,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>40483</v>
       </c>
       <c r="B60" t="n">
@@ -2737,7 +2725,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>40513</v>
       </c>
       <c r="B61" t="n">
@@ -2775,7 +2763,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>40544</v>
       </c>
       <c r="B62" t="n">
@@ -2813,7 +2801,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="1" t="n">
         <v>40575</v>
       </c>
       <c r="B63" t="n">
@@ -2851,7 +2839,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="1" t="n">
         <v>40603</v>
       </c>
       <c r="B64" t="n">
@@ -2889,7 +2877,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="1" t="n">
         <v>40634</v>
       </c>
       <c r="B65" t="n">
@@ -2927,7 +2915,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="1" t="n">
         <v>40664</v>
       </c>
       <c r="B66" t="n">
@@ -2965,7 +2953,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="1" t="n">
         <v>40695</v>
       </c>
       <c r="B67" t="n">
@@ -3003,7 +2991,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="1" t="n">
         <v>40725</v>
       </c>
       <c r="B68" t="n">
@@ -3041,7 +3029,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="1" t="n">
         <v>40756</v>
       </c>
       <c r="B69" t="n">
@@ -3079,7 +3067,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="1" t="n">
         <v>40787</v>
       </c>
       <c r="B70" t="n">
@@ -3117,7 +3105,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="1" t="n">
         <v>40817</v>
       </c>
       <c r="B71" t="n">
@@ -3155,7 +3143,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="1" t="n">
         <v>40848</v>
       </c>
       <c r="B72" t="n">
@@ -3193,7 +3181,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="1" t="n">
         <v>40878</v>
       </c>
       <c r="B73" t="n">
@@ -3231,7 +3219,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="1" t="n">
         <v>40909</v>
       </c>
       <c r="B74" t="n">
@@ -3269,7 +3257,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="1" t="n">
         <v>40940</v>
       </c>
       <c r="B75" t="n">
@@ -3307,7 +3295,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="1" t="n">
         <v>40969</v>
       </c>
       <c r="B76" t="n">
@@ -3345,7 +3333,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="1" t="n">
         <v>41000</v>
       </c>
       <c r="B77" t="n">
@@ -3383,7 +3371,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="1" t="n">
         <v>41030</v>
       </c>
       <c r="B78" t="n">
@@ -3421,7 +3409,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="1" t="n">
         <v>41061</v>
       </c>
       <c r="B79" t="n">
@@ -3459,7 +3447,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="1" t="n">
         <v>41091</v>
       </c>
       <c r="B80" t="n">
@@ -3497,7 +3485,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="1" t="n">
         <v>41122</v>
       </c>
       <c r="B81" t="n">
@@ -3535,7 +3523,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="1" t="n">
         <v>41153</v>
       </c>
       <c r="B82" t="n">
@@ -3573,7 +3561,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="1" t="n">
         <v>41183</v>
       </c>
       <c r="B83" t="n">
@@ -3611,7 +3599,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="1" t="n">
         <v>41214</v>
       </c>
       <c r="B84" t="n">
@@ -3649,7 +3637,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="1" t="n">
         <v>41244</v>
       </c>
       <c r="B85" t="n">
@@ -3687,7 +3675,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="1" t="n">
         <v>41275</v>
       </c>
       <c r="B86" t="n">
@@ -3725,7 +3713,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="1" t="n">
         <v>41306</v>
       </c>
       <c r="B87" t="n">
@@ -3763,7 +3751,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="1" t="n">
         <v>41334</v>
       </c>
       <c r="B88" t="n">
@@ -3801,7 +3789,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="1" t="n">
         <v>41365</v>
       </c>
       <c r="B89" t="n">
@@ -3839,7 +3827,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="1" t="n">
         <v>41395</v>
       </c>
       <c r="B90" t="n">
@@ -3877,7 +3865,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="1" t="n">
         <v>41426</v>
       </c>
       <c r="B91" t="n">
@@ -3915,7 +3903,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="1" t="n">
         <v>41456</v>
       </c>
       <c r="B92" t="n">
@@ -3953,7 +3941,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="1" t="n">
         <v>41487</v>
       </c>
       <c r="B93" t="n">
@@ -3991,7 +3979,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="1" t="n">
         <v>41518</v>
       </c>
       <c r="B94" t="n">
@@ -4029,7 +4017,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" s="1" t="n">
         <v>41548</v>
       </c>
       <c r="B95" t="n">
@@ -4067,7 +4055,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="1" t="n">
         <v>41579</v>
       </c>
       <c r="B96" t="n">
@@ -4105,7 +4093,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="1" t="n">
         <v>41609</v>
       </c>
       <c r="B97" t="n">
@@ -4143,7 +4131,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="1" t="n">
         <v>41640</v>
       </c>
       <c r="B98" t="n">
@@ -4181,7 +4169,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="1" t="n">
         <v>41671</v>
       </c>
       <c r="B99" t="n">
@@ -4219,7 +4207,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="1" t="n">
         <v>41699</v>
       </c>
       <c r="B100" t="n">
@@ -4257,7 +4245,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="1" t="n">
         <v>41730</v>
       </c>
       <c r="B101" t="n">
@@ -4295,7 +4283,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="1" t="n">
         <v>41760</v>
       </c>
       <c r="B102" t="n">
@@ -4333,7 +4321,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="1" t="n">
         <v>41791</v>
       </c>
       <c r="B103" t="n">
@@ -4371,7 +4359,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="1" t="n">
         <v>41821</v>
       </c>
       <c r="B104" t="n">
@@ -4409,7 +4397,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="1" t="n">
         <v>41852</v>
       </c>
       <c r="B105" t="n">
@@ -4447,7 +4435,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="1" t="n">
         <v>41883</v>
       </c>
       <c r="B106" t="n">
@@ -4485,7 +4473,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="1" t="n">
         <v>41913</v>
       </c>
       <c r="B107" t="n">
@@ -4523,7 +4511,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="1" t="n">
         <v>41944</v>
       </c>
       <c r="B108" t="n">
@@ -4561,7 +4549,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
+      <c r="A109" s="1" t="n">
         <v>41974</v>
       </c>
       <c r="B109" t="n">
@@ -4599,7 +4587,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
+      <c r="A110" s="1" t="n">
         <v>42005</v>
       </c>
       <c r="B110" t="n">
@@ -4637,7 +4625,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="1" t="n">
         <v>42036</v>
       </c>
       <c r="B111" t="n">
@@ -4675,7 +4663,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="1" t="n">
         <v>42064</v>
       </c>
       <c r="B112" t="n">
@@ -4713,7 +4701,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="1" t="n">
         <v>42095</v>
       </c>
       <c r="B113" t="n">
@@ -4751,7 +4739,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="1" t="n">
         <v>42125</v>
       </c>
       <c r="B114" t="n">
@@ -4789,7 +4777,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="1" t="n">
         <v>42156</v>
       </c>
       <c r="B115" t="n">
@@ -4827,7 +4815,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
+      <c r="A116" s="1" t="n">
         <v>42186</v>
       </c>
       <c r="B116" t="n">
@@ -4865,7 +4853,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
+      <c r="A117" s="1" t="n">
         <v>42217</v>
       </c>
       <c r="B117" t="n">
@@ -4903,7 +4891,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
+      <c r="A118" s="1" t="n">
         <v>42248</v>
       </c>
       <c r="B118" t="n">
@@ -4941,7 +4929,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
+      <c r="A119" s="1" t="n">
         <v>42278</v>
       </c>
       <c r="B119" t="n">
@@ -4979,7 +4967,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
+      <c r="A120" s="1" t="n">
         <v>42309</v>
       </c>
       <c r="B120" t="n">
@@ -5017,7 +5005,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
+      <c r="A121" s="1" t="n">
         <v>42339</v>
       </c>
       <c r="B121" t="n">
@@ -5055,7 +5043,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
+      <c r="A122" s="1" t="n">
         <v>42370</v>
       </c>
       <c r="B122" t="n">
@@ -5093,7 +5081,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
+      <c r="A123" s="1" t="n">
         <v>42401</v>
       </c>
       <c r="B123" t="n">
@@ -5131,7 +5119,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
+      <c r="A124" s="1" t="n">
         <v>42430</v>
       </c>
       <c r="B124" t="n">
@@ -5169,7 +5157,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
+      <c r="A125" s="1" t="n">
         <v>42461</v>
       </c>
       <c r="B125" t="n">
@@ -5207,7 +5195,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" s="1" t="n">
         <v>42491</v>
       </c>
       <c r="B126" t="n">
@@ -5245,7 +5233,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
+      <c r="A127" s="1" t="n">
         <v>42522</v>
       </c>
       <c r="B127" t="n">
@@ -5283,7 +5271,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
+      <c r="A128" s="1" t="n">
         <v>42552</v>
       </c>
       <c r="B128" t="n">
@@ -5321,7 +5309,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
+      <c r="A129" s="1" t="n">
         <v>42583</v>
       </c>
       <c r="B129" t="n">
@@ -5359,7 +5347,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
+      <c r="A130" s="1" t="n">
         <v>42614</v>
       </c>
       <c r="B130" t="n">
@@ -5397,7 +5385,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
+      <c r="A131" s="1" t="n">
         <v>42644</v>
       </c>
       <c r="B131" t="n">
@@ -5435,7 +5423,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" s="1" t="n">
         <v>42675</v>
       </c>
       <c r="B132" t="n">
@@ -5473,7 +5461,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" s="1" t="n">
         <v>42705</v>
       </c>
       <c r="B133" t="n">
@@ -5511,7 +5499,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
+      <c r="A134" s="1" t="n">
         <v>42736</v>
       </c>
       <c r="B134" t="n">
@@ -5549,7 +5537,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
+      <c r="A135" s="1" t="n">
         <v>42767</v>
       </c>
       <c r="B135" t="n">
@@ -5587,7 +5575,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="1" t="n">
         <v>42795</v>
       </c>
       <c r="B136" t="n">
@@ -5625,7 +5613,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
+      <c r="A137" s="1" t="n">
         <v>42826</v>
       </c>
       <c r="B137" t="n">
@@ -5663,7 +5651,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
+      <c r="A138" s="1" t="n">
         <v>42856</v>
       </c>
       <c r="B138" t="n">
@@ -5701,7 +5689,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
+      <c r="A139" s="1" t="n">
         <v>42887</v>
       </c>
       <c r="B139" t="n">
@@ -5739,7 +5727,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
+      <c r="A140" s="1" t="n">
         <v>42917</v>
       </c>
       <c r="B140" t="n">
@@ -5777,7 +5765,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
+      <c r="A141" s="1" t="n">
         <v>42948</v>
       </c>
       <c r="B141" t="n">
@@ -5815,7 +5803,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
+      <c r="A142" s="1" t="n">
         <v>42979</v>
       </c>
       <c r="B142" t="n">
@@ -5853,7 +5841,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
+      <c r="A143" s="1" t="n">
         <v>43009</v>
       </c>
       <c r="B143" t="n">
@@ -5891,7 +5879,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
+      <c r="A144" s="1" t="n">
         <v>43040</v>
       </c>
       <c r="B144" t="n">
@@ -5929,7 +5917,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
+      <c r="A145" s="1" t="n">
         <v>43070</v>
       </c>
       <c r="B145" t="n">
@@ -5967,7 +5955,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n">
+      <c r="A146" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="B146" t="n">
@@ -6005,7 +5993,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
+      <c r="A147" s="1" t="n">
         <v>43132</v>
       </c>
       <c r="B147" t="n">
@@ -6043,7 +6031,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
+      <c r="A148" s="1" t="n">
         <v>43160</v>
       </c>
       <c r="B148" t="n">
@@ -6081,7 +6069,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
+      <c r="A149" s="1" t="n">
         <v>43191</v>
       </c>
       <c r="B149" t="n">
@@ -6119,7 +6107,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
+      <c r="A150" s="1" t="n">
         <v>43221</v>
       </c>
       <c r="B150" t="n">
@@ -6157,7 +6145,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n">
+      <c r="A151" s="1" t="n">
         <v>43252</v>
       </c>
       <c r="B151" t="n">
@@ -6195,7 +6183,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n">
+      <c r="A152" s="1" t="n">
         <v>43282</v>
       </c>
       <c r="B152" t="n">
@@ -6233,7 +6221,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
+      <c r="A153" s="1" t="n">
         <v>43313</v>
       </c>
       <c r="B153" t="n">
@@ -6271,7 +6259,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
+      <c r="A154" s="1" t="n">
         <v>43344</v>
       </c>
       <c r="B154" t="n">
@@ -6309,7 +6297,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n">
+      <c r="A155" s="1" t="n">
         <v>43374</v>
       </c>
       <c r="B155" t="n">
@@ -6347,7 +6335,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
+      <c r="A156" s="1" t="n">
         <v>43405</v>
       </c>
       <c r="B156" t="n">
@@ -6385,7 +6373,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n">
+      <c r="A157" s="1" t="n">
         <v>43435</v>
       </c>
       <c r="B157" t="n">
@@ -6423,7 +6411,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n">
+      <c r="A158" s="1" t="n">
         <v>43466</v>
       </c>
       <c r="B158" t="n">
@@ -6461,7 +6449,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n">
+      <c r="A159" s="1" t="n">
         <v>43497</v>
       </c>
       <c r="B159" t="n">
@@ -6499,7 +6487,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
+      <c r="A160" s="1" t="n">
         <v>43525</v>
       </c>
       <c r="B160" t="n">
@@ -6537,7 +6525,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
+      <c r="A161" s="1" t="n">
         <v>43556</v>
       </c>
       <c r="B161" t="n">
@@ -6575,7 +6563,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
+      <c r="A162" s="1" t="n">
         <v>43586</v>
       </c>
       <c r="B162" t="n">
@@ -6613,7 +6601,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
+      <c r="A163" s="1" t="n">
         <v>43617</v>
       </c>
       <c r="B163" t="n">
@@ -6651,7 +6639,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
+      <c r="A164" s="1" t="n">
         <v>43647</v>
       </c>
       <c r="B164" t="n">
@@ -6689,7 +6677,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n">
+      <c r="A165" s="1" t="n">
         <v>43678</v>
       </c>
       <c r="B165" t="n">
@@ -6727,7 +6715,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n">
+      <c r="A166" s="1" t="n">
         <v>43709</v>
       </c>
       <c r="B166" t="n">
@@ -6765,7 +6753,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
+      <c r="A167" s="1" t="n">
         <v>43739</v>
       </c>
       <c r="B167" t="n">
@@ -6803,7 +6791,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
+      <c r="A168" s="1" t="n">
         <v>43770</v>
       </c>
       <c r="B168" t="n">
@@ -6841,7 +6829,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
+      <c r="A169" s="1" t="n">
         <v>43800</v>
       </c>
       <c r="B169" t="n">
@@ -6879,7 +6867,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n">
+      <c r="A170" s="1" t="n">
         <v>43831</v>
       </c>
       <c r="B170" t="n">
@@ -6917,7 +6905,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
+      <c r="A171" s="1" t="n">
         <v>43862</v>
       </c>
       <c r="B171" t="n">
@@ -6955,7 +6943,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n">
+      <c r="A172" s="1" t="n">
         <v>43891</v>
       </c>
       <c r="B172" t="n">
@@ -6993,7 +6981,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n">
+      <c r="A173" s="1" t="n">
         <v>43922</v>
       </c>
       <c r="B173" t="n">
@@ -7031,7 +7019,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
+      <c r="A174" s="1" t="n">
         <v>43952</v>
       </c>
       <c r="B174" t="n">
@@ -7069,7 +7057,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
+      <c r="A175" s="1" t="n">
         <v>43983</v>
       </c>
       <c r="B175" t="n">
@@ -7107,7 +7095,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
+      <c r="A176" s="1" t="n">
         <v>44013</v>
       </c>
       <c r="B176" t="n">
@@ -7145,7 +7133,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
+      <c r="A177" s="1" t="n">
         <v>44044</v>
       </c>
       <c r="B177" t="n">
@@ -7183,7 +7171,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
+      <c r="A178" s="1" t="n">
         <v>44075</v>
       </c>
       <c r="B178" t="n">
@@ -7221,7 +7209,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n">
+      <c r="A179" s="1" t="n">
         <v>44105</v>
       </c>
       <c r="B179" t="n">
@@ -7259,7 +7247,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n">
+      <c r="A180" s="1" t="n">
         <v>44136</v>
       </c>
       <c r="B180" t="n">
@@ -7297,7 +7285,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
+      <c r="A181" s="1" t="n">
         <v>44166</v>
       </c>
       <c r="B181" t="n">
@@ -7335,7 +7323,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
+      <c r="A182" s="1" t="n">
         <v>44197</v>
       </c>
       <c r="B182" t="n">
@@ -7373,7 +7361,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
+      <c r="A183" s="1" t="n">
         <v>44228</v>
       </c>
       <c r="B183" t="n">
@@ -7411,7 +7399,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n">
+      <c r="A184" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="B184" t="n">
@@ -7449,7 +7437,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n">
+      <c r="A185" s="1" t="n">
         <v>44287</v>
       </c>
       <c r="B185" t="n">
@@ -7487,7 +7475,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n">
+      <c r="A186" s="1" t="n">
         <v>44317</v>
       </c>
       <c r="B186" t="n">
@@ -7525,7 +7513,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n">
+      <c r="A187" s="1" t="n">
         <v>44348</v>
       </c>
       <c r="B187" t="n">
@@ -7563,7 +7551,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n">
+      <c r="A188" s="1" t="n">
         <v>44378</v>
       </c>
       <c r="B188" t="n">
@@ -7601,7 +7589,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n">
+      <c r="A189" s="1" t="n">
         <v>44409</v>
       </c>
       <c r="B189" t="n">
@@ -7639,7 +7627,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n">
+      <c r="A190" s="1" t="n">
         <v>44440</v>
       </c>
       <c r="B190" t="n">
@@ -7677,7 +7665,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="n">
+      <c r="A191" s="1" t="n">
         <v>44470</v>
       </c>
       <c r="B191" t="n">
@@ -7715,7 +7703,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n">
+      <c r="A192" s="1" t="n">
         <v>44501</v>
       </c>
       <c r="B192" t="n">
@@ -7753,7 +7741,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="n">
+      <c r="A193" s="1" t="n">
         <v>44531</v>
       </c>
       <c r="B193" t="n">
@@ -7791,7 +7779,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="n">
+      <c r="A194" s="1" t="n">
         <v>44562</v>
       </c>
       <c r="B194" t="n">
@@ -7829,7 +7817,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="n">
+      <c r="A195" s="1" t="n">
         <v>44593</v>
       </c>
       <c r="B195" t="n">
@@ -7867,7 +7855,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="n">
+      <c r="A196" s="1" t="n">
         <v>44621</v>
       </c>
       <c r="B196" t="n">
@@ -7905,7 +7893,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="n">
+      <c r="A197" s="1" t="n">
         <v>44652</v>
       </c>
       <c r="B197" t="n">
@@ -7943,7 +7931,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n">
+      <c r="A198" s="1" t="n">
         <v>44682</v>
       </c>
       <c r="B198" t="n">
@@ -7981,7 +7969,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="n">
+      <c r="A199" s="1" t="n">
         <v>44713</v>
       </c>
       <c r="B199" t="n">
@@ -8019,7 +8007,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n">
+      <c r="A200" s="1" t="n">
         <v>44743</v>
       </c>
       <c r="B200" t="n">
@@ -8057,7 +8045,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="n">
+      <c r="A201" s="1" t="n">
         <v>44774</v>
       </c>
       <c r="B201" t="n">
@@ -8095,7 +8083,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="n">
+      <c r="A202" s="1" t="n">
         <v>44805</v>
       </c>
       <c r="B202" t="n">
@@ -8133,7 +8121,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="n">
+      <c r="A203" s="1" t="n">
         <v>44835</v>
       </c>
       <c r="B203" t="n">
@@ -8171,7 +8159,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="n">
+      <c r="A204" s="1" t="n">
         <v>44866</v>
       </c>
       <c r="B204" t="n">
@@ -8209,7 +8197,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="n">
+      <c r="A205" s="1" t="n">
         <v>44896</v>
       </c>
       <c r="B205" t="n">
@@ -8247,7 +8235,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="n">
+      <c r="A206" s="1" t="n">
         <v>44927</v>
       </c>
       <c r="B206" t="n">
@@ -8285,7 +8273,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="n">
+      <c r="A207" s="1" t="n">
         <v>44958</v>
       </c>
       <c r="B207" t="n">
@@ -8323,7 +8311,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="n">
+      <c r="A208" s="1" t="n">
         <v>44986</v>
       </c>
       <c r="B208" t="n">
@@ -8361,7 +8349,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="n">
+      <c r="A209" s="1" t="n">
         <v>45017</v>
       </c>
       <c r="B209" t="n">
@@ -8399,7 +8387,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n">
+      <c r="A210" s="1" t="n">
         <v>45047</v>
       </c>
       <c r="B210" t="n">
@@ -8437,7 +8425,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="2" t="n">
+      <c r="A211" s="1" t="n">
         <v>45078</v>
       </c>
       <c r="B211" t="n">
@@ -8475,7 +8463,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="n">
+      <c r="A212" s="1" t="n">
         <v>45108</v>
       </c>
       <c r="B212" t="n">
@@ -8513,7 +8501,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="n">
+      <c r="A213" s="1" t="n">
         <v>45139</v>
       </c>
       <c r="B213" t="n">
@@ -8551,7 +8539,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="n">
+      <c r="A214" s="1" t="n">
         <v>45170</v>
       </c>
       <c r="B214" t="n">
@@ -8589,7 +8577,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="2" t="n">
+      <c r="A215" s="1" t="n">
         <v>45200</v>
       </c>
       <c r="B215" t="n">
@@ -8627,7 +8615,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="2" t="n">
+      <c r="A216" s="1" t="n">
         <v>45231</v>
       </c>
       <c r="B216" t="n">
@@ -8665,7 +8653,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="n">
+      <c r="A217" s="1" t="n">
         <v>45261</v>
       </c>
       <c r="B217" t="n">
@@ -8703,7 +8691,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="n">
+      <c r="A218" s="1" t="n">
         <v>45292</v>
       </c>
       <c r="B218" t="n">
@@ -8741,7 +8729,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="n">
+      <c r="A219" s="1" t="n">
         <v>45323</v>
       </c>
       <c r="B219" t="n">
@@ -8779,7 +8767,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="n">
+      <c r="A220" s="1" t="n">
         <v>45352</v>
       </c>
       <c r="B220" t="n">
@@ -8817,7 +8805,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="n">
+      <c r="A221" s="1" t="n">
         <v>45383</v>
       </c>
       <c r="B221" t="n">
@@ -8855,7 +8843,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="n">
+      <c r="A222" s="1" t="n">
         <v>45413</v>
       </c>
       <c r="B222" t="n">
@@ -8893,7 +8881,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="n">
+      <c r="A223" s="1" t="n">
         <v>45444</v>
       </c>
       <c r="B223" t="n">
@@ -8931,7 +8919,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="n">
+      <c r="A224" s="1" t="n">
         <v>45474</v>
       </c>
       <c r="B224" t="n">
@@ -8969,7 +8957,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="n">
+      <c r="A225" s="1" t="n">
         <v>45505</v>
       </c>
       <c r="B225" t="n">
@@ -9007,7 +8995,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="n">
+      <c r="A226" s="1" t="n">
         <v>45536</v>
       </c>
       <c r="B226" t="n">
@@ -9045,7 +9033,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="n">
+      <c r="A227" s="1" t="n">
         <v>45566</v>
       </c>
       <c r="B227" t="n">
@@ -9083,7 +9071,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="n">
+      <c r="A228" s="1" t="n">
         <v>45597</v>
       </c>
       <c r="B228" t="n">
@@ -9121,7 +9109,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="n">
+      <c r="A229" s="1" t="n">
         <v>45627</v>
       </c>
       <c r="B229" t="n">
@@ -9159,7 +9147,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="n">
+      <c r="A230" s="1" t="n">
         <v>45658</v>
       </c>
       <c r="B230" t="n">
@@ -9197,7 +9185,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="n">
+      <c r="A231" s="1" t="n">
         <v>45689</v>
       </c>
       <c r="B231" t="n">
@@ -9235,7 +9223,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="n">
+      <c r="A232" s="1" t="n">
         <v>45717</v>
       </c>
       <c r="B232" t="n">
@@ -9273,7 +9261,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="n">
+      <c r="A233" s="1" t="n">
         <v>45748</v>
       </c>
       <c r="B233" t="n">
@@ -9311,7 +9299,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="n">
+      <c r="A234" s="1" t="n">
         <v>45778</v>
       </c>
       <c r="B234" t="n">
@@ -9349,7 +9337,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="n">
+      <c r="A235" s="1" t="n">
         <v>45809</v>
       </c>
       <c r="B235" t="n">
@@ -9387,7 +9375,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="2" t="n">
+      <c r="A236" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="B236" t="n">
@@ -9425,7 +9413,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="2" t="n">
+      <c r="A237" s="1" t="n">
         <v>45870</v>
       </c>
       <c r="B237" t="n">
@@ -9463,7 +9451,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="2" t="n">
+      <c r="A238" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="B238" t="n">
@@ -9501,7 +9489,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="2" t="n">
+      <c r="A239" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="B239" t="n">
@@ -9539,7 +9527,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="2" t="n">
+      <c r="A240" s="1" t="n">
         <v>45962</v>
       </c>
       <c r="B240" t="n">
@@ -9577,7 +9565,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="2" t="n">
+      <c r="A241" s="1" t="n">
         <v>45992</v>
       </c>
       <c r="B241" t="n">
@@ -9615,7 +9603,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="2" t="n">
+      <c r="A242" s="1" t="n">
         <v>46023</v>
       </c>
       <c r="B242" t="n">
@@ -9653,7 +9641,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="n">
+      <c r="A243" s="1" t="n">
         <v>46054</v>
       </c>
       <c r="B243" t="n">
@@ -9691,7 +9679,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="2" t="n">
+      <c r="A244" s="1" t="n">
         <v>46082</v>
       </c>
       <c r="B244" t="n">
@@ -9729,7 +9717,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="2" t="n">
+      <c r="A245" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="B245" t="n">
@@ -9767,7 +9755,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="2" t="n">
+      <c r="A246" s="1" t="n">
         <v>46143</v>
       </c>
       <c r="B246" t="n">
@@ -9805,7 +9793,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="2" t="n">
+      <c r="A247" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="B247" t="n">
@@ -9843,7 +9831,7 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="2" t="n">
+      <c r="A248" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="B248" t="n">

</xml_diff>

<commit_message>
Toplu veri güncelleme (yerel, 28.08.2026 13:53)
</commit_message>
<xml_diff>
--- a/butce/butce.xlsx
+++ b/butce/butce.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,69 +433,69 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>tarih</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>yil</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ay</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>gelir</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>vergi</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>dolaysiz_vergi</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>dolayli_vergi</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>gider</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>faiz_haric_gider</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>faiz_gideri</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>faiz_disi_denge</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>denge</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>38718</v>
       </c>
       <c r="B2" t="n">
@@ -521,7 +533,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>38749</v>
       </c>
       <c r="B3" t="n">
@@ -559,7 +571,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>38777</v>
       </c>
       <c r="B4" t="n">
@@ -597,7 +609,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>38808</v>
       </c>
       <c r="B5" t="n">
@@ -635,7 +647,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>38838</v>
       </c>
       <c r="B6" t="n">
@@ -673,7 +685,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>38869</v>
       </c>
       <c r="B7" t="n">
@@ -711,7 +723,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>38899</v>
       </c>
       <c r="B8" t="n">
@@ -749,7 +761,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>38930</v>
       </c>
       <c r="B9" t="n">
@@ -787,7 +799,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>38961</v>
       </c>
       <c r="B10" t="n">
@@ -825,7 +837,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>38991</v>
       </c>
       <c r="B11" t="n">
@@ -863,7 +875,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>39022</v>
       </c>
       <c r="B12" t="n">
@@ -901,7 +913,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>39052</v>
       </c>
       <c r="B13" t="n">
@@ -939,7 +951,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>39083</v>
       </c>
       <c r="B14" t="n">
@@ -977,7 +989,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>39114</v>
       </c>
       <c r="B15" t="n">
@@ -1015,7 +1027,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>39142</v>
       </c>
       <c r="B16" t="n">
@@ -1053,7 +1065,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>39173</v>
       </c>
       <c r="B17" t="n">
@@ -1091,7 +1103,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>39203</v>
       </c>
       <c r="B18" t="n">
@@ -1129,7 +1141,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>39234</v>
       </c>
       <c r="B19" t="n">
@@ -1167,7 +1179,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>39264</v>
       </c>
       <c r="B20" t="n">
@@ -1205,7 +1217,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>39295</v>
       </c>
       <c r="B21" t="n">
@@ -1243,7 +1255,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>39326</v>
       </c>
       <c r="B22" t="n">
@@ -1281,7 +1293,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>39356</v>
       </c>
       <c r="B23" t="n">
@@ -1319,7 +1331,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>39387</v>
       </c>
       <c r="B24" t="n">
@@ -1357,7 +1369,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>39417</v>
       </c>
       <c r="B25" t="n">
@@ -1395,7 +1407,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>39448</v>
       </c>
       <c r="B26" t="n">
@@ -1433,7 +1445,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>39479</v>
       </c>
       <c r="B27" t="n">
@@ -1471,7 +1483,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>39508</v>
       </c>
       <c r="B28" t="n">
@@ -1509,7 +1521,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>39539</v>
       </c>
       <c r="B29" t="n">
@@ -1547,7 +1559,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>39569</v>
       </c>
       <c r="B30" t="n">
@@ -1585,7 +1597,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>39600</v>
       </c>
       <c r="B31" t="n">
@@ -1623,7 +1635,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>39630</v>
       </c>
       <c r="B32" t="n">
@@ -1661,7 +1673,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>39661</v>
       </c>
       <c r="B33" t="n">
@@ -1699,7 +1711,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>39692</v>
       </c>
       <c r="B34" t="n">
@@ -1737,7 +1749,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>39722</v>
       </c>
       <c r="B35" t="n">
@@ -1775,7 +1787,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>39753</v>
       </c>
       <c r="B36" t="n">
@@ -1813,7 +1825,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>39783</v>
       </c>
       <c r="B37" t="n">
@@ -1851,7 +1863,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>39814</v>
       </c>
       <c r="B38" t="n">
@@ -1889,7 +1901,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>39845</v>
       </c>
       <c r="B39" t="n">
@@ -1927,7 +1939,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>39873</v>
       </c>
       <c r="B40" t="n">
@@ -1965,7 +1977,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>39904</v>
       </c>
       <c r="B41" t="n">
@@ -2003,7 +2015,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>39934</v>
       </c>
       <c r="B42" t="n">
@@ -2041,7 +2053,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>39965</v>
       </c>
       <c r="B43" t="n">
@@ -2079,7 +2091,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>39995</v>
       </c>
       <c r="B44" t="n">
@@ -2117,7 +2129,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>40026</v>
       </c>
       <c r="B45" t="n">
@@ -2155,7 +2167,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>40057</v>
       </c>
       <c r="B46" t="n">
@@ -2193,7 +2205,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>40087</v>
       </c>
       <c r="B47" t="n">
@@ -2231,7 +2243,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>40118</v>
       </c>
       <c r="B48" t="n">
@@ -2269,7 +2281,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>40148</v>
       </c>
       <c r="B49" t="n">
@@ -2307,7 +2319,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>40179</v>
       </c>
       <c r="B50" t="n">
@@ -2345,7 +2357,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>40210</v>
       </c>
       <c r="B51" t="n">
@@ -2383,7 +2395,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>40238</v>
       </c>
       <c r="B52" t="n">
@@ -2421,7 +2433,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>40269</v>
       </c>
       <c r="B53" t="n">
@@ -2459,7 +2471,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>40299</v>
       </c>
       <c r="B54" t="n">
@@ -2497,7 +2509,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>40330</v>
       </c>
       <c r="B55" t="n">
@@ -2535,7 +2547,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>40360</v>
       </c>
       <c r="B56" t="n">
@@ -2573,7 +2585,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>40391</v>
       </c>
       <c r="B57" t="n">
@@ -2611,7 +2623,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>40422</v>
       </c>
       <c r="B58" t="n">
@@ -2649,7 +2661,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>40452</v>
       </c>
       <c r="B59" t="n">
@@ -2687,7 +2699,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>40483</v>
       </c>
       <c r="B60" t="n">
@@ -2725,7 +2737,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>40513</v>
       </c>
       <c r="B61" t="n">
@@ -2763,7 +2775,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>40544</v>
       </c>
       <c r="B62" t="n">
@@ -2801,7 +2813,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" s="2" t="n">
         <v>40575</v>
       </c>
       <c r="B63" t="n">
@@ -2839,7 +2851,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" s="2" t="n">
         <v>40603</v>
       </c>
       <c r="B64" t="n">
@@ -2877,7 +2889,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" s="2" t="n">
         <v>40634</v>
       </c>
       <c r="B65" t="n">
@@ -2915,7 +2927,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="2" t="n">
         <v>40664</v>
       </c>
       <c r="B66" t="n">
@@ -2953,7 +2965,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="2" t="n">
         <v>40695</v>
       </c>
       <c r="B67" t="n">
@@ -2991,7 +3003,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="2" t="n">
         <v>40725</v>
       </c>
       <c r="B68" t="n">
@@ -3029,7 +3041,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="2" t="n">
         <v>40756</v>
       </c>
       <c r="B69" t="n">
@@ -3067,7 +3079,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="2" t="n">
         <v>40787</v>
       </c>
       <c r="B70" t="n">
@@ -3105,7 +3117,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="2" t="n">
         <v>40817</v>
       </c>
       <c r="B71" t="n">
@@ -3143,7 +3155,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" s="2" t="n">
         <v>40848</v>
       </c>
       <c r="B72" t="n">
@@ -3181,7 +3193,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="2" t="n">
         <v>40878</v>
       </c>
       <c r="B73" t="n">
@@ -3219,7 +3231,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="2" t="n">
         <v>40909</v>
       </c>
       <c r="B74" t="n">
@@ -3257,7 +3269,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="2" t="n">
         <v>40940</v>
       </c>
       <c r="B75" t="n">
@@ -3295,7 +3307,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="2" t="n">
         <v>40969</v>
       </c>
       <c r="B76" t="n">
@@ -3333,7 +3345,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="2" t="n">
         <v>41000</v>
       </c>
       <c r="B77" t="n">
@@ -3371,7 +3383,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="2" t="n">
         <v>41030</v>
       </c>
       <c r="B78" t="n">
@@ -3409,7 +3421,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="2" t="n">
         <v>41061</v>
       </c>
       <c r="B79" t="n">
@@ -3447,7 +3459,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="2" t="n">
         <v>41091</v>
       </c>
       <c r="B80" t="n">
@@ -3485,7 +3497,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" s="2" t="n">
         <v>41122</v>
       </c>
       <c r="B81" t="n">
@@ -3523,7 +3535,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" s="2" t="n">
         <v>41153</v>
       </c>
       <c r="B82" t="n">
@@ -3561,7 +3573,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="2" t="n">
         <v>41183</v>
       </c>
       <c r="B83" t="n">
@@ -3599,7 +3611,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="2" t="n">
         <v>41214</v>
       </c>
       <c r="B84" t="n">
@@ -3637,7 +3649,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" s="2" t="n">
         <v>41244</v>
       </c>
       <c r="B85" t="n">
@@ -3675,7 +3687,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" s="2" t="n">
         <v>41275</v>
       </c>
       <c r="B86" t="n">
@@ -3713,7 +3725,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="2" t="n">
         <v>41306</v>
       </c>
       <c r="B87" t="n">
@@ -3751,7 +3763,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="2" t="n">
         <v>41334</v>
       </c>
       <c r="B88" t="n">
@@ -3789,7 +3801,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="2" t="n">
         <v>41365</v>
       </c>
       <c r="B89" t="n">
@@ -3827,7 +3839,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="2" t="n">
         <v>41395</v>
       </c>
       <c r="B90" t="n">
@@ -3865,7 +3877,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="2" t="n">
         <v>41426</v>
       </c>
       <c r="B91" t="n">
@@ -3903,7 +3915,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="2" t="n">
         <v>41456</v>
       </c>
       <c r="B92" t="n">
@@ -3941,7 +3953,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" s="2" t="n">
         <v>41487</v>
       </c>
       <c r="B93" t="n">
@@ -3979,7 +3991,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" s="2" t="n">
         <v>41518</v>
       </c>
       <c r="B94" t="n">
@@ -4017,7 +4029,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" s="2" t="n">
         <v>41548</v>
       </c>
       <c r="B95" t="n">
@@ -4055,7 +4067,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" s="2" t="n">
         <v>41579</v>
       </c>
       <c r="B96" t="n">
@@ -4093,7 +4105,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" s="2" t="n">
         <v>41609</v>
       </c>
       <c r="B97" t="n">
@@ -4131,7 +4143,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" s="2" t="n">
         <v>41640</v>
       </c>
       <c r="B98" t="n">
@@ -4169,7 +4181,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" s="2" t="n">
         <v>41671</v>
       </c>
       <c r="B99" t="n">
@@ -4207,7 +4219,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" s="2" t="n">
         <v>41699</v>
       </c>
       <c r="B100" t="n">
@@ -4245,7 +4257,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" s="2" t="n">
         <v>41730</v>
       </c>
       <c r="B101" t="n">
@@ -4283,7 +4295,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" s="2" t="n">
         <v>41760</v>
       </c>
       <c r="B102" t="n">
@@ -4321,7 +4333,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" s="2" t="n">
         <v>41791</v>
       </c>
       <c r="B103" t="n">
@@ -4359,7 +4371,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" s="2" t="n">
         <v>41821</v>
       </c>
       <c r="B104" t="n">
@@ -4397,7 +4409,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" s="2" t="n">
         <v>41852</v>
       </c>
       <c r="B105" t="n">
@@ -4435,7 +4447,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" s="2" t="n">
         <v>41883</v>
       </c>
       <c r="B106" t="n">
@@ -4473,7 +4485,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" s="2" t="n">
         <v>41913</v>
       </c>
       <c r="B107" t="n">
@@ -4511,7 +4523,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" s="2" t="n">
         <v>41944</v>
       </c>
       <c r="B108" t="n">
@@ -4549,7 +4561,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" s="2" t="n">
         <v>41974</v>
       </c>
       <c r="B109" t="n">
@@ -4587,7 +4599,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" s="2" t="n">
         <v>42005</v>
       </c>
       <c r="B110" t="n">
@@ -4625,7 +4637,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" s="2" t="n">
         <v>42036</v>
       </c>
       <c r="B111" t="n">
@@ -4663,7 +4675,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" s="2" t="n">
         <v>42064</v>
       </c>
       <c r="B112" t="n">
@@ -4701,7 +4713,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" s="2" t="n">
         <v>42095</v>
       </c>
       <c r="B113" t="n">
@@ -4739,7 +4751,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" s="2" t="n">
         <v>42125</v>
       </c>
       <c r="B114" t="n">
@@ -4777,7 +4789,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" s="2" t="n">
         <v>42156</v>
       </c>
       <c r="B115" t="n">
@@ -4815,7 +4827,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" s="2" t="n">
         <v>42186</v>
       </c>
       <c r="B116" t="n">
@@ -4853,7 +4865,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" s="2" t="n">
         <v>42217</v>
       </c>
       <c r="B117" t="n">
@@ -4891,7 +4903,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" s="2" t="n">
         <v>42248</v>
       </c>
       <c r="B118" t="n">
@@ -4929,7 +4941,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" s="2" t="n">
         <v>42278</v>
       </c>
       <c r="B119" t="n">
@@ -4967,7 +4979,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" s="2" t="n">
         <v>42309</v>
       </c>
       <c r="B120" t="n">
@@ -5005,7 +5017,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" s="2" t="n">
         <v>42339</v>
       </c>
       <c r="B121" t="n">
@@ -5043,7 +5055,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" s="2" t="n">
         <v>42370</v>
       </c>
       <c r="B122" t="n">
@@ -5081,7 +5093,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" s="2" t="n">
         <v>42401</v>
       </c>
       <c r="B123" t="n">
@@ -5119,7 +5131,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" s="2" t="n">
         <v>42430</v>
       </c>
       <c r="B124" t="n">
@@ -5157,7 +5169,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" s="2" t="n">
         <v>42461</v>
       </c>
       <c r="B125" t="n">
@@ -5195,7 +5207,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" s="2" t="n">
         <v>42491</v>
       </c>
       <c r="B126" t="n">
@@ -5233,7 +5245,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" s="2" t="n">
         <v>42522</v>
       </c>
       <c r="B127" t="n">
@@ -5271,7 +5283,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" s="2" t="n">
         <v>42552</v>
       </c>
       <c r="B128" t="n">
@@ -5309,7 +5321,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" s="2" t="n">
         <v>42583</v>
       </c>
       <c r="B129" t="n">
@@ -5347,7 +5359,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
+      <c r="A130" s="2" t="n">
         <v>42614</v>
       </c>
       <c r="B130" t="n">
@@ -5385,7 +5397,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
+      <c r="A131" s="2" t="n">
         <v>42644</v>
       </c>
       <c r="B131" t="n">
@@ -5423,7 +5435,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
+      <c r="A132" s="2" t="n">
         <v>42675</v>
       </c>
       <c r="B132" t="n">
@@ -5461,7 +5473,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
+      <c r="A133" s="2" t="n">
         <v>42705</v>
       </c>
       <c r="B133" t="n">
@@ -5499,7 +5511,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
+      <c r="A134" s="2" t="n">
         <v>42736</v>
       </c>
       <c r="B134" t="n">
@@ -5537,7 +5549,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
+      <c r="A135" s="2" t="n">
         <v>42767</v>
       </c>
       <c r="B135" t="n">
@@ -5575,7 +5587,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
+      <c r="A136" s="2" t="n">
         <v>42795</v>
       </c>
       <c r="B136" t="n">
@@ -5613,7 +5625,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
+      <c r="A137" s="2" t="n">
         <v>42826</v>
       </c>
       <c r="B137" t="n">
@@ -5651,7 +5663,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
+      <c r="A138" s="2" t="n">
         <v>42856</v>
       </c>
       <c r="B138" t="n">
@@ -5689,7 +5701,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="n">
+      <c r="A139" s="2" t="n">
         <v>42887</v>
       </c>
       <c r="B139" t="n">
@@ -5727,7 +5739,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="n">
+      <c r="A140" s="2" t="n">
         <v>42917</v>
       </c>
       <c r="B140" t="n">
@@ -5765,7 +5777,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="n">
+      <c r="A141" s="2" t="n">
         <v>42948</v>
       </c>
       <c r="B141" t="n">
@@ -5803,7 +5815,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="n">
+      <c r="A142" s="2" t="n">
         <v>42979</v>
       </c>
       <c r="B142" t="n">
@@ -5841,7 +5853,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="n">
+      <c r="A143" s="2" t="n">
         <v>43009</v>
       </c>
       <c r="B143" t="n">
@@ -5879,7 +5891,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="n">
+      <c r="A144" s="2" t="n">
         <v>43040</v>
       </c>
       <c r="B144" t="n">
@@ -5917,7 +5929,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="n">
+      <c r="A145" s="2" t="n">
         <v>43070</v>
       </c>
       <c r="B145" t="n">
@@ -5955,7 +5967,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="1" t="n">
+      <c r="A146" s="2" t="n">
         <v>43101</v>
       </c>
       <c r="B146" t="n">
@@ -5993,7 +6005,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="1" t="n">
+      <c r="A147" s="2" t="n">
         <v>43132</v>
       </c>
       <c r="B147" t="n">
@@ -6031,7 +6043,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="1" t="n">
+      <c r="A148" s="2" t="n">
         <v>43160</v>
       </c>
       <c r="B148" t="n">
@@ -6069,7 +6081,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="1" t="n">
+      <c r="A149" s="2" t="n">
         <v>43191</v>
       </c>
       <c r="B149" t="n">
@@ -6107,7 +6119,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="1" t="n">
+      <c r="A150" s="2" t="n">
         <v>43221</v>
       </c>
       <c r="B150" t="n">
@@ -6145,7 +6157,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="1" t="n">
+      <c r="A151" s="2" t="n">
         <v>43252</v>
       </c>
       <c r="B151" t="n">
@@ -6183,7 +6195,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="1" t="n">
+      <c r="A152" s="2" t="n">
         <v>43282</v>
       </c>
       <c r="B152" t="n">
@@ -6221,7 +6233,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="1" t="n">
+      <c r="A153" s="2" t="n">
         <v>43313</v>
       </c>
       <c r="B153" t="n">
@@ -6259,7 +6271,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="1" t="n">
+      <c r="A154" s="2" t="n">
         <v>43344</v>
       </c>
       <c r="B154" t="n">
@@ -6297,7 +6309,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="1" t="n">
+      <c r="A155" s="2" t="n">
         <v>43374</v>
       </c>
       <c r="B155" t="n">
@@ -6335,7 +6347,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="1" t="n">
+      <c r="A156" s="2" t="n">
         <v>43405</v>
       </c>
       <c r="B156" t="n">
@@ -6373,7 +6385,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="1" t="n">
+      <c r="A157" s="2" t="n">
         <v>43435</v>
       </c>
       <c r="B157" t="n">
@@ -6411,7 +6423,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="1" t="n">
+      <c r="A158" s="2" t="n">
         <v>43466</v>
       </c>
       <c r="B158" t="n">
@@ -6449,7 +6461,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="1" t="n">
+      <c r="A159" s="2" t="n">
         <v>43497</v>
       </c>
       <c r="B159" t="n">
@@ -6487,7 +6499,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="1" t="n">
+      <c r="A160" s="2" t="n">
         <v>43525</v>
       </c>
       <c r="B160" t="n">
@@ -6525,7 +6537,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="1" t="n">
+      <c r="A161" s="2" t="n">
         <v>43556</v>
       </c>
       <c r="B161" t="n">
@@ -6563,7 +6575,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="1" t="n">
+      <c r="A162" s="2" t="n">
         <v>43586</v>
       </c>
       <c r="B162" t="n">
@@ -6601,7 +6613,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="1" t="n">
+      <c r="A163" s="2" t="n">
         <v>43617</v>
       </c>
       <c r="B163" t="n">
@@ -6639,7 +6651,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="1" t="n">
+      <c r="A164" s="2" t="n">
         <v>43647</v>
       </c>
       <c r="B164" t="n">
@@ -6677,7 +6689,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="1" t="n">
+      <c r="A165" s="2" t="n">
         <v>43678</v>
       </c>
       <c r="B165" t="n">
@@ -6715,7 +6727,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="1" t="n">
+      <c r="A166" s="2" t="n">
         <v>43709</v>
       </c>
       <c r="B166" t="n">
@@ -6753,7 +6765,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="1" t="n">
+      <c r="A167" s="2" t="n">
         <v>43739</v>
       </c>
       <c r="B167" t="n">
@@ -6791,7 +6803,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="1" t="n">
+      <c r="A168" s="2" t="n">
         <v>43770</v>
       </c>
       <c r="B168" t="n">
@@ -6829,7 +6841,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="1" t="n">
+      <c r="A169" s="2" t="n">
         <v>43800</v>
       </c>
       <c r="B169" t="n">
@@ -6867,7 +6879,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="1" t="n">
+      <c r="A170" s="2" t="n">
         <v>43831</v>
       </c>
       <c r="B170" t="n">
@@ -6905,7 +6917,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="1" t="n">
+      <c r="A171" s="2" t="n">
         <v>43862</v>
       </c>
       <c r="B171" t="n">
@@ -6943,7 +6955,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="1" t="n">
+      <c r="A172" s="2" t="n">
         <v>43891</v>
       </c>
       <c r="B172" t="n">
@@ -6981,7 +6993,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="1" t="n">
+      <c r="A173" s="2" t="n">
         <v>43922</v>
       </c>
       <c r="B173" t="n">
@@ -7019,7 +7031,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="1" t="n">
+      <c r="A174" s="2" t="n">
         <v>43952</v>
       </c>
       <c r="B174" t="n">
@@ -7057,7 +7069,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="1" t="n">
+      <c r="A175" s="2" t="n">
         <v>43983</v>
       </c>
       <c r="B175" t="n">
@@ -7095,7 +7107,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="1" t="n">
+      <c r="A176" s="2" t="n">
         <v>44013</v>
       </c>
       <c r="B176" t="n">
@@ -7133,7 +7145,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="1" t="n">
+      <c r="A177" s="2" t="n">
         <v>44044</v>
       </c>
       <c r="B177" t="n">
@@ -7171,7 +7183,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="1" t="n">
+      <c r="A178" s="2" t="n">
         <v>44075</v>
       </c>
       <c r="B178" t="n">
@@ -7209,7 +7221,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="1" t="n">
+      <c r="A179" s="2" t="n">
         <v>44105</v>
       </c>
       <c r="B179" t="n">
@@ -7247,7 +7259,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="1" t="n">
+      <c r="A180" s="2" t="n">
         <v>44136</v>
       </c>
       <c r="B180" t="n">
@@ -7285,7 +7297,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="1" t="n">
+      <c r="A181" s="2" t="n">
         <v>44166</v>
       </c>
       <c r="B181" t="n">
@@ -7323,7 +7335,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="1" t="n">
+      <c r="A182" s="2" t="n">
         <v>44197</v>
       </c>
       <c r="B182" t="n">
@@ -7361,7 +7373,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="1" t="n">
+      <c r="A183" s="2" t="n">
         <v>44228</v>
       </c>
       <c r="B183" t="n">
@@ -7399,7 +7411,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="1" t="n">
+      <c r="A184" s="2" t="n">
         <v>44256</v>
       </c>
       <c r="B184" t="n">
@@ -7437,7 +7449,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="1" t="n">
+      <c r="A185" s="2" t="n">
         <v>44287</v>
       </c>
       <c r="B185" t="n">
@@ -7475,7 +7487,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="1" t="n">
+      <c r="A186" s="2" t="n">
         <v>44317</v>
       </c>
       <c r="B186" t="n">
@@ -7513,7 +7525,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="1" t="n">
+      <c r="A187" s="2" t="n">
         <v>44348</v>
       </c>
       <c r="B187" t="n">
@@ -7551,7 +7563,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="1" t="n">
+      <c r="A188" s="2" t="n">
         <v>44378</v>
       </c>
       <c r="B188" t="n">
@@ -7589,7 +7601,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="1" t="n">
+      <c r="A189" s="2" t="n">
         <v>44409</v>
       </c>
       <c r="B189" t="n">
@@ -7627,7 +7639,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="1" t="n">
+      <c r="A190" s="2" t="n">
         <v>44440</v>
       </c>
       <c r="B190" t="n">
@@ -7665,7 +7677,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="1" t="n">
+      <c r="A191" s="2" t="n">
         <v>44470</v>
       </c>
       <c r="B191" t="n">
@@ -7703,7 +7715,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="1" t="n">
+      <c r="A192" s="2" t="n">
         <v>44501</v>
       </c>
       <c r="B192" t="n">
@@ -7741,7 +7753,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="1" t="n">
+      <c r="A193" s="2" t="n">
         <v>44531</v>
       </c>
       <c r="B193" t="n">
@@ -7779,7 +7791,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="1" t="n">
+      <c r="A194" s="2" t="n">
         <v>44562</v>
       </c>
       <c r="B194" t="n">
@@ -7817,7 +7829,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="1" t="n">
+      <c r="A195" s="2" t="n">
         <v>44593</v>
       </c>
       <c r="B195" t="n">
@@ -7855,7 +7867,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="1" t="n">
+      <c r="A196" s="2" t="n">
         <v>44621</v>
       </c>
       <c r="B196" t="n">
@@ -7893,7 +7905,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="1" t="n">
+      <c r="A197" s="2" t="n">
         <v>44652</v>
       </c>
       <c r="B197" t="n">
@@ -7931,7 +7943,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="1" t="n">
+      <c r="A198" s="2" t="n">
         <v>44682</v>
       </c>
       <c r="B198" t="n">
@@ -7969,7 +7981,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="1" t="n">
+      <c r="A199" s="2" t="n">
         <v>44713</v>
       </c>
       <c r="B199" t="n">
@@ -8007,7 +8019,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="1" t="n">
+      <c r="A200" s="2" t="n">
         <v>44743</v>
       </c>
       <c r="B200" t="n">
@@ -8045,7 +8057,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="1" t="n">
+      <c r="A201" s="2" t="n">
         <v>44774</v>
       </c>
       <c r="B201" t="n">
@@ -8083,7 +8095,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="1" t="n">
+      <c r="A202" s="2" t="n">
         <v>44805</v>
       </c>
       <c r="B202" t="n">
@@ -8121,7 +8133,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="1" t="n">
+      <c r="A203" s="2" t="n">
         <v>44835</v>
       </c>
       <c r="B203" t="n">
@@ -8159,7 +8171,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="1" t="n">
+      <c r="A204" s="2" t="n">
         <v>44866</v>
       </c>
       <c r="B204" t="n">
@@ -8197,7 +8209,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="1" t="n">
+      <c r="A205" s="2" t="n">
         <v>44896</v>
       </c>
       <c r="B205" t="n">
@@ -8235,7 +8247,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="1" t="n">
+      <c r="A206" s="2" t="n">
         <v>44927</v>
       </c>
       <c r="B206" t="n">
@@ -8273,7 +8285,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="1" t="n">
+      <c r="A207" s="2" t="n">
         <v>44958</v>
       </c>
       <c r="B207" t="n">
@@ -8311,7 +8323,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="1" t="n">
+      <c r="A208" s="2" t="n">
         <v>44986</v>
       </c>
       <c r="B208" t="n">
@@ -8349,7 +8361,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="1" t="n">
+      <c r="A209" s="2" t="n">
         <v>45017</v>
       </c>
       <c r="B209" t="n">
@@ -8387,7 +8399,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="1" t="n">
+      <c r="A210" s="2" t="n">
         <v>45047</v>
       </c>
       <c r="B210" t="n">
@@ -8425,7 +8437,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="1" t="n">
+      <c r="A211" s="2" t="n">
         <v>45078</v>
       </c>
       <c r="B211" t="n">
@@ -8463,7 +8475,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="1" t="n">
+      <c r="A212" s="2" t="n">
         <v>45108</v>
       </c>
       <c r="B212" t="n">
@@ -8501,7 +8513,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="1" t="n">
+      <c r="A213" s="2" t="n">
         <v>45139</v>
       </c>
       <c r="B213" t="n">
@@ -8539,7 +8551,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="1" t="n">
+      <c r="A214" s="2" t="n">
         <v>45170</v>
       </c>
       <c r="B214" t="n">
@@ -8577,7 +8589,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="1" t="n">
+      <c r="A215" s="2" t="n">
         <v>45200</v>
       </c>
       <c r="B215" t="n">
@@ -8615,7 +8627,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="1" t="n">
+      <c r="A216" s="2" t="n">
         <v>45231</v>
       </c>
       <c r="B216" t="n">
@@ -8653,7 +8665,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="1" t="n">
+      <c r="A217" s="2" t="n">
         <v>45261</v>
       </c>
       <c r="B217" t="n">
@@ -8691,7 +8703,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="1" t="n">
+      <c r="A218" s="2" t="n">
         <v>45292</v>
       </c>
       <c r="B218" t="n">
@@ -8729,7 +8741,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="1" t="n">
+      <c r="A219" s="2" t="n">
         <v>45323</v>
       </c>
       <c r="B219" t="n">
@@ -8767,7 +8779,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="1" t="n">
+      <c r="A220" s="2" t="n">
         <v>45352</v>
       </c>
       <c r="B220" t="n">
@@ -8805,7 +8817,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="1" t="n">
+      <c r="A221" s="2" t="n">
         <v>45383</v>
       </c>
       <c r="B221" t="n">
@@ -8843,7 +8855,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="1" t="n">
+      <c r="A222" s="2" t="n">
         <v>45413</v>
       </c>
       <c r="B222" t="n">
@@ -8881,7 +8893,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="1" t="n">
+      <c r="A223" s="2" t="n">
         <v>45444</v>
       </c>
       <c r="B223" t="n">
@@ -8919,7 +8931,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="1" t="n">
+      <c r="A224" s="2" t="n">
         <v>45474</v>
       </c>
       <c r="B224" t="n">
@@ -8957,7 +8969,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="1" t="n">
+      <c r="A225" s="2" t="n">
         <v>45505</v>
       </c>
       <c r="B225" t="n">
@@ -8995,7 +9007,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="1" t="n">
+      <c r="A226" s="2" t="n">
         <v>45536</v>
       </c>
       <c r="B226" t="n">
@@ -9033,7 +9045,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="1" t="n">
+      <c r="A227" s="2" t="n">
         <v>45566</v>
       </c>
       <c r="B227" t="n">
@@ -9071,7 +9083,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="1" t="n">
+      <c r="A228" s="2" t="n">
         <v>45597</v>
       </c>
       <c r="B228" t="n">
@@ -9109,7 +9121,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="1" t="n">
+      <c r="A229" s="2" t="n">
         <v>45627</v>
       </c>
       <c r="B229" t="n">
@@ -9147,7 +9159,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="1" t="n">
+      <c r="A230" s="2" t="n">
         <v>45658</v>
       </c>
       <c r="B230" t="n">
@@ -9185,7 +9197,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="1" t="n">
+      <c r="A231" s="2" t="n">
         <v>45689</v>
       </c>
       <c r="B231" t="n">
@@ -9223,7 +9235,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="1" t="n">
+      <c r="A232" s="2" t="n">
         <v>45717</v>
       </c>
       <c r="B232" t="n">
@@ -9261,7 +9273,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="1" t="n">
+      <c r="A233" s="2" t="n">
         <v>45748</v>
       </c>
       <c r="B233" t="n">
@@ -9299,7 +9311,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="1" t="n">
+      <c r="A234" s="2" t="n">
         <v>45778</v>
       </c>
       <c r="B234" t="n">
@@ -9337,7 +9349,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="1" t="n">
+      <c r="A235" s="2" t="n">
         <v>45809</v>
       </c>
       <c r="B235" t="n">
@@ -9375,7 +9387,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="1" t="n">
+      <c r="A236" s="2" t="n">
         <v>45839</v>
       </c>
       <c r="B236" t="n">
@@ -9413,7 +9425,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="1" t="n">
+      <c r="A237" s="2" t="n">
         <v>45870</v>
       </c>
       <c r="B237" t="n">
@@ -9451,7 +9463,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="1" t="n">
+      <c r="A238" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="B238" t="n">
@@ -9489,7 +9501,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="1" t="n">
+      <c r="A239" s="2" t="n">
         <v>45931</v>
       </c>
       <c r="B239" t="n">
@@ -9527,7 +9539,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="1" t="n">
+      <c r="A240" s="2" t="n">
         <v>45962</v>
       </c>
       <c r="B240" t="n">
@@ -9565,7 +9577,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="1" t="n">
+      <c r="A241" s="2" t="n">
         <v>45992</v>
       </c>
       <c r="B241" t="n">
@@ -9603,7 +9615,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="1" t="n">
+      <c r="A242" s="2" t="n">
         <v>46023</v>
       </c>
       <c r="B242" t="n">
@@ -9641,7 +9653,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="1" t="n">
+      <c r="A243" s="2" t="n">
         <v>46054</v>
       </c>
       <c r="B243" t="n">
@@ -9679,7 +9691,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="1" t="n">
+      <c r="A244" s="2" t="n">
         <v>46082</v>
       </c>
       <c r="B244" t="n">
@@ -9717,7 +9729,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="1" t="n">
+      <c r="A245" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="B245" t="n">
@@ -9755,7 +9767,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="1" t="n">
+      <c r="A246" s="2" t="n">
         <v>46143</v>
       </c>
       <c r="B246" t="n">
@@ -9793,7 +9805,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="1" t="n">
+      <c r="A247" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="B247" t="n">
@@ -9831,7 +9843,7 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="1" t="n">
+      <c r="A248" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="B248" t="n">

</xml_diff>

<commit_message>
Otomatik veri güncelleme (28.08.2026 21:33 UTC)
</commit_message>
<xml_diff>
--- a/butce/butce.xlsx
+++ b/butce/butce.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Aylik" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,69 +421,69 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tarih</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>yil</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ay</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>gelir</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>vergi</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>dolaysiz_vergi</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>dolayli_vergi</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>gider</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>faiz_haric_gider</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>faiz_gideri</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>faiz_disi_denge</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>denge</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>38718</v>
       </c>
       <c r="B2" t="n">
@@ -533,7 +521,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>38749</v>
       </c>
       <c r="B3" t="n">
@@ -571,7 +559,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>38777</v>
       </c>
       <c r="B4" t="n">
@@ -609,7 +597,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>38808</v>
       </c>
       <c r="B5" t="n">
@@ -647,7 +635,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>38838</v>
       </c>
       <c r="B6" t="n">
@@ -685,7 +673,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>38869</v>
       </c>
       <c r="B7" t="n">
@@ -723,7 +711,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>38899</v>
       </c>
       <c r="B8" t="n">
@@ -761,7 +749,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>38930</v>
       </c>
       <c r="B9" t="n">
@@ -799,7 +787,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>38961</v>
       </c>
       <c r="B10" t="n">
@@ -837,7 +825,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>38991</v>
       </c>
       <c r="B11" t="n">
@@ -875,7 +863,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>39022</v>
       </c>
       <c r="B12" t="n">
@@ -913,7 +901,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>39052</v>
       </c>
       <c r="B13" t="n">
@@ -951,7 +939,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>39083</v>
       </c>
       <c r="B14" t="n">
@@ -989,7 +977,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>39114</v>
       </c>
       <c r="B15" t="n">
@@ -1027,7 +1015,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>39142</v>
       </c>
       <c r="B16" t="n">
@@ -1065,7 +1053,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>39173</v>
       </c>
       <c r="B17" t="n">
@@ -1103,7 +1091,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>39203</v>
       </c>
       <c r="B18" t="n">
@@ -1141,7 +1129,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>39234</v>
       </c>
       <c r="B19" t="n">
@@ -1179,7 +1167,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>39264</v>
       </c>
       <c r="B20" t="n">
@@ -1217,7 +1205,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>39295</v>
       </c>
       <c r="B21" t="n">
@@ -1255,7 +1243,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>39326</v>
       </c>
       <c r="B22" t="n">
@@ -1293,7 +1281,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>39356</v>
       </c>
       <c r="B23" t="n">
@@ -1331,7 +1319,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>39387</v>
       </c>
       <c r="B24" t="n">
@@ -1369,7 +1357,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>39417</v>
       </c>
       <c r="B25" t="n">
@@ -1407,7 +1395,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>39448</v>
       </c>
       <c r="B26" t="n">
@@ -1445,7 +1433,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="1" t="n">
         <v>39479</v>
       </c>
       <c r="B27" t="n">
@@ -1483,7 +1471,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>39508</v>
       </c>
       <c r="B28" t="n">
@@ -1521,7 +1509,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>39539</v>
       </c>
       <c r="B29" t="n">
@@ -1559,7 +1547,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>39569</v>
       </c>
       <c r="B30" t="n">
@@ -1597,7 +1585,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>39600</v>
       </c>
       <c r="B31" t="n">
@@ -1635,7 +1623,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>39630</v>
       </c>
       <c r="B32" t="n">
@@ -1673,7 +1661,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>39661</v>
       </c>
       <c r="B33" t="n">
@@ -1711,7 +1699,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>39692</v>
       </c>
       <c r="B34" t="n">
@@ -1749,7 +1737,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>39722</v>
       </c>
       <c r="B35" t="n">
@@ -1787,7 +1775,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>39753</v>
       </c>
       <c r="B36" t="n">
@@ -1825,7 +1813,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>39783</v>
       </c>
       <c r="B37" t="n">
@@ -1863,7 +1851,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>39814</v>
       </c>
       <c r="B38" t="n">
@@ -1901,7 +1889,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>39845</v>
       </c>
       <c r="B39" t="n">
@@ -1939,7 +1927,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>39873</v>
       </c>
       <c r="B40" t="n">
@@ -1977,7 +1965,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>39904</v>
       </c>
       <c r="B41" t="n">
@@ -2015,7 +2003,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>39934</v>
       </c>
       <c r="B42" t="n">
@@ -2053,7 +2041,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>39965</v>
       </c>
       <c r="B43" t="n">
@@ -2091,7 +2079,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>39995</v>
       </c>
       <c r="B44" t="n">
@@ -2129,7 +2117,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>40026</v>
       </c>
       <c r="B45" t="n">
@@ -2167,7 +2155,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>40057</v>
       </c>
       <c r="B46" t="n">
@@ -2205,7 +2193,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>40087</v>
       </c>
       <c r="B47" t="n">
@@ -2243,7 +2231,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>40118</v>
       </c>
       <c r="B48" t="n">
@@ -2281,7 +2269,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>40148</v>
       </c>
       <c r="B49" t="n">
@@ -2319,7 +2307,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>40179</v>
       </c>
       <c r="B50" t="n">
@@ -2357,7 +2345,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>40210</v>
       </c>
       <c r="B51" t="n">
@@ -2395,7 +2383,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>40238</v>
       </c>
       <c r="B52" t="n">
@@ -2433,7 +2421,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>40269</v>
       </c>
       <c r="B53" t="n">
@@ -2471,7 +2459,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>40299</v>
       </c>
       <c r="B54" t="n">
@@ -2509,7 +2497,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>40330</v>
       </c>
       <c r="B55" t="n">
@@ -2547,7 +2535,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>40360</v>
       </c>
       <c r="B56" t="n">
@@ -2585,7 +2573,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>40391</v>
       </c>
       <c r="B57" t="n">
@@ -2623,7 +2611,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>40422</v>
       </c>
       <c r="B58" t="n">
@@ -2661,7 +2649,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>40452</v>
       </c>
       <c r="B59" t="n">
@@ -2699,7 +2687,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>40483</v>
       </c>
       <c r="B60" t="n">
@@ -2737,7 +2725,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>40513</v>
       </c>
       <c r="B61" t="n">
@@ -2775,7 +2763,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>40544</v>
       </c>
       <c r="B62" t="n">
@@ -2813,7 +2801,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="1" t="n">
         <v>40575</v>
       </c>
       <c r="B63" t="n">
@@ -2851,7 +2839,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="1" t="n">
         <v>40603</v>
       </c>
       <c r="B64" t="n">
@@ -2889,7 +2877,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="1" t="n">
         <v>40634</v>
       </c>
       <c r="B65" t="n">
@@ -2927,7 +2915,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="1" t="n">
         <v>40664</v>
       </c>
       <c r="B66" t="n">
@@ -2965,7 +2953,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="1" t="n">
         <v>40695</v>
       </c>
       <c r="B67" t="n">
@@ -3003,7 +2991,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="1" t="n">
         <v>40725</v>
       </c>
       <c r="B68" t="n">
@@ -3041,7 +3029,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="1" t="n">
         <v>40756</v>
       </c>
       <c r="B69" t="n">
@@ -3079,7 +3067,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="1" t="n">
         <v>40787</v>
       </c>
       <c r="B70" t="n">
@@ -3117,7 +3105,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="1" t="n">
         <v>40817</v>
       </c>
       <c r="B71" t="n">
@@ -3155,7 +3143,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="1" t="n">
         <v>40848</v>
       </c>
       <c r="B72" t="n">
@@ -3193,7 +3181,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="1" t="n">
         <v>40878</v>
       </c>
       <c r="B73" t="n">
@@ -3231,7 +3219,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="1" t="n">
         <v>40909</v>
       </c>
       <c r="B74" t="n">
@@ -3269,7 +3257,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="1" t="n">
         <v>40940</v>
       </c>
       <c r="B75" t="n">
@@ -3307,7 +3295,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="1" t="n">
         <v>40969</v>
       </c>
       <c r="B76" t="n">
@@ -3345,7 +3333,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="1" t="n">
         <v>41000</v>
       </c>
       <c r="B77" t="n">
@@ -3383,7 +3371,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="1" t="n">
         <v>41030</v>
       </c>
       <c r="B78" t="n">
@@ -3421,7 +3409,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="1" t="n">
         <v>41061</v>
       </c>
       <c r="B79" t="n">
@@ -3459,7 +3447,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="1" t="n">
         <v>41091</v>
       </c>
       <c r="B80" t="n">
@@ -3497,7 +3485,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="1" t="n">
         <v>41122</v>
       </c>
       <c r="B81" t="n">
@@ -3535,7 +3523,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="1" t="n">
         <v>41153</v>
       </c>
       <c r="B82" t="n">
@@ -3573,7 +3561,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="1" t="n">
         <v>41183</v>
       </c>
       <c r="B83" t="n">
@@ -3611,7 +3599,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="1" t="n">
         <v>41214</v>
       </c>
       <c r="B84" t="n">
@@ -3649,7 +3637,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="1" t="n">
         <v>41244</v>
       </c>
       <c r="B85" t="n">
@@ -3687,7 +3675,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="1" t="n">
         <v>41275</v>
       </c>
       <c r="B86" t="n">
@@ -3725,7 +3713,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="1" t="n">
         <v>41306</v>
       </c>
       <c r="B87" t="n">
@@ -3763,7 +3751,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="1" t="n">
         <v>41334</v>
       </c>
       <c r="B88" t="n">
@@ -3801,7 +3789,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="1" t="n">
         <v>41365</v>
       </c>
       <c r="B89" t="n">
@@ -3839,7 +3827,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="1" t="n">
         <v>41395</v>
       </c>
       <c r="B90" t="n">
@@ -3877,7 +3865,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="1" t="n">
         <v>41426</v>
       </c>
       <c r="B91" t="n">
@@ -3915,7 +3903,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="1" t="n">
         <v>41456</v>
       </c>
       <c r="B92" t="n">
@@ -3953,7 +3941,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="1" t="n">
         <v>41487</v>
       </c>
       <c r="B93" t="n">
@@ -3991,7 +3979,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="1" t="n">
         <v>41518</v>
       </c>
       <c r="B94" t="n">
@@ -4029,7 +4017,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" s="1" t="n">
         <v>41548</v>
       </c>
       <c r="B95" t="n">
@@ -4067,7 +4055,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="1" t="n">
         <v>41579</v>
       </c>
       <c r="B96" t="n">
@@ -4105,7 +4093,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="1" t="n">
         <v>41609</v>
       </c>
       <c r="B97" t="n">
@@ -4143,7 +4131,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="1" t="n">
         <v>41640</v>
       </c>
       <c r="B98" t="n">
@@ -4181,7 +4169,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="1" t="n">
         <v>41671</v>
       </c>
       <c r="B99" t="n">
@@ -4219,7 +4207,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="1" t="n">
         <v>41699</v>
       </c>
       <c r="B100" t="n">
@@ -4257,7 +4245,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="1" t="n">
         <v>41730</v>
       </c>
       <c r="B101" t="n">
@@ -4295,7 +4283,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="1" t="n">
         <v>41760</v>
       </c>
       <c r="B102" t="n">
@@ -4333,7 +4321,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="1" t="n">
         <v>41791</v>
       </c>
       <c r="B103" t="n">
@@ -4371,7 +4359,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="1" t="n">
         <v>41821</v>
       </c>
       <c r="B104" t="n">
@@ -4409,7 +4397,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="1" t="n">
         <v>41852</v>
       </c>
       <c r="B105" t="n">
@@ -4447,7 +4435,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="1" t="n">
         <v>41883</v>
       </c>
       <c r="B106" t="n">
@@ -4485,7 +4473,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="1" t="n">
         <v>41913</v>
       </c>
       <c r="B107" t="n">
@@ -4523,7 +4511,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="1" t="n">
         <v>41944</v>
       </c>
       <c r="B108" t="n">
@@ -4561,7 +4549,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
+      <c r="A109" s="1" t="n">
         <v>41974</v>
       </c>
       <c r="B109" t="n">
@@ -4599,7 +4587,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
+      <c r="A110" s="1" t="n">
         <v>42005</v>
       </c>
       <c r="B110" t="n">
@@ -4637,7 +4625,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="1" t="n">
         <v>42036</v>
       </c>
       <c r="B111" t="n">
@@ -4675,7 +4663,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="1" t="n">
         <v>42064</v>
       </c>
       <c r="B112" t="n">
@@ -4713,7 +4701,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="1" t="n">
         <v>42095</v>
       </c>
       <c r="B113" t="n">
@@ -4751,7 +4739,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="1" t="n">
         <v>42125</v>
       </c>
       <c r="B114" t="n">
@@ -4789,7 +4777,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="1" t="n">
         <v>42156</v>
       </c>
       <c r="B115" t="n">
@@ -4827,7 +4815,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
+      <c r="A116" s="1" t="n">
         <v>42186</v>
       </c>
       <c r="B116" t="n">
@@ -4865,7 +4853,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
+      <c r="A117" s="1" t="n">
         <v>42217</v>
       </c>
       <c r="B117" t="n">
@@ -4903,7 +4891,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
+      <c r="A118" s="1" t="n">
         <v>42248</v>
       </c>
       <c r="B118" t="n">
@@ -4941,7 +4929,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
+      <c r="A119" s="1" t="n">
         <v>42278</v>
       </c>
       <c r="B119" t="n">
@@ -4979,7 +4967,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
+      <c r="A120" s="1" t="n">
         <v>42309</v>
       </c>
       <c r="B120" t="n">
@@ -5017,7 +5005,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
+      <c r="A121" s="1" t="n">
         <v>42339</v>
       </c>
       <c r="B121" t="n">
@@ -5055,7 +5043,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
+      <c r="A122" s="1" t="n">
         <v>42370</v>
       </c>
       <c r="B122" t="n">
@@ -5093,7 +5081,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
+      <c r="A123" s="1" t="n">
         <v>42401</v>
       </c>
       <c r="B123" t="n">
@@ -5131,7 +5119,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
+      <c r="A124" s="1" t="n">
         <v>42430</v>
       </c>
       <c r="B124" t="n">
@@ -5169,7 +5157,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
+      <c r="A125" s="1" t="n">
         <v>42461</v>
       </c>
       <c r="B125" t="n">
@@ -5207,7 +5195,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" s="1" t="n">
         <v>42491</v>
       </c>
       <c r="B126" t="n">
@@ -5245,7 +5233,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
+      <c r="A127" s="1" t="n">
         <v>42522</v>
       </c>
       <c r="B127" t="n">
@@ -5283,7 +5271,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
+      <c r="A128" s="1" t="n">
         <v>42552</v>
       </c>
       <c r="B128" t="n">
@@ -5321,7 +5309,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
+      <c r="A129" s="1" t="n">
         <v>42583</v>
       </c>
       <c r="B129" t="n">
@@ -5359,7 +5347,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
+      <c r="A130" s="1" t="n">
         <v>42614</v>
       </c>
       <c r="B130" t="n">
@@ -5397,7 +5385,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
+      <c r="A131" s="1" t="n">
         <v>42644</v>
       </c>
       <c r="B131" t="n">
@@ -5435,7 +5423,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" s="1" t="n">
         <v>42675</v>
       </c>
       <c r="B132" t="n">
@@ -5473,7 +5461,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" s="1" t="n">
         <v>42705</v>
       </c>
       <c r="B133" t="n">
@@ -5511,7 +5499,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
+      <c r="A134" s="1" t="n">
         <v>42736</v>
       </c>
       <c r="B134" t="n">
@@ -5549,7 +5537,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
+      <c r="A135" s="1" t="n">
         <v>42767</v>
       </c>
       <c r="B135" t="n">
@@ -5587,7 +5575,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="1" t="n">
         <v>42795</v>
       </c>
       <c r="B136" t="n">
@@ -5625,7 +5613,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
+      <c r="A137" s="1" t="n">
         <v>42826</v>
       </c>
       <c r="B137" t="n">
@@ -5663,7 +5651,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
+      <c r="A138" s="1" t="n">
         <v>42856</v>
       </c>
       <c r="B138" t="n">
@@ -5701,7 +5689,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
+      <c r="A139" s="1" t="n">
         <v>42887</v>
       </c>
       <c r="B139" t="n">
@@ -5739,7 +5727,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
+      <c r="A140" s="1" t="n">
         <v>42917</v>
       </c>
       <c r="B140" t="n">
@@ -5777,7 +5765,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
+      <c r="A141" s="1" t="n">
         <v>42948</v>
       </c>
       <c r="B141" t="n">
@@ -5815,7 +5803,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
+      <c r="A142" s="1" t="n">
         <v>42979</v>
       </c>
       <c r="B142" t="n">
@@ -5853,7 +5841,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
+      <c r="A143" s="1" t="n">
         <v>43009</v>
       </c>
       <c r="B143" t="n">
@@ -5891,7 +5879,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
+      <c r="A144" s="1" t="n">
         <v>43040</v>
       </c>
       <c r="B144" t="n">
@@ -5929,7 +5917,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
+      <c r="A145" s="1" t="n">
         <v>43070</v>
       </c>
       <c r="B145" t="n">
@@ -5967,7 +5955,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n">
+      <c r="A146" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="B146" t="n">
@@ -6005,7 +5993,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
+      <c r="A147" s="1" t="n">
         <v>43132</v>
       </c>
       <c r="B147" t="n">
@@ -6043,7 +6031,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
+      <c r="A148" s="1" t="n">
         <v>43160</v>
       </c>
       <c r="B148" t="n">
@@ -6081,7 +6069,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
+      <c r="A149" s="1" t="n">
         <v>43191</v>
       </c>
       <c r="B149" t="n">
@@ -6119,7 +6107,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
+      <c r="A150" s="1" t="n">
         <v>43221</v>
       </c>
       <c r="B150" t="n">
@@ -6157,7 +6145,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n">
+      <c r="A151" s="1" t="n">
         <v>43252</v>
       </c>
       <c r="B151" t="n">
@@ -6195,7 +6183,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n">
+      <c r="A152" s="1" t="n">
         <v>43282</v>
       </c>
       <c r="B152" t="n">
@@ -6233,7 +6221,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
+      <c r="A153" s="1" t="n">
         <v>43313</v>
       </c>
       <c r="B153" t="n">
@@ -6271,7 +6259,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
+      <c r="A154" s="1" t="n">
         <v>43344</v>
       </c>
       <c r="B154" t="n">
@@ -6309,7 +6297,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n">
+      <c r="A155" s="1" t="n">
         <v>43374</v>
       </c>
       <c r="B155" t="n">
@@ -6347,7 +6335,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
+      <c r="A156" s="1" t="n">
         <v>43405</v>
       </c>
       <c r="B156" t="n">
@@ -6385,7 +6373,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n">
+      <c r="A157" s="1" t="n">
         <v>43435</v>
       </c>
       <c r="B157" t="n">
@@ -6423,7 +6411,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n">
+      <c r="A158" s="1" t="n">
         <v>43466</v>
       </c>
       <c r="B158" t="n">
@@ -6461,7 +6449,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n">
+      <c r="A159" s="1" t="n">
         <v>43497</v>
       </c>
       <c r="B159" t="n">
@@ -6499,7 +6487,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
+      <c r="A160" s="1" t="n">
         <v>43525</v>
       </c>
       <c r="B160" t="n">
@@ -6537,7 +6525,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
+      <c r="A161" s="1" t="n">
         <v>43556</v>
       </c>
       <c r="B161" t="n">
@@ -6575,7 +6563,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
+      <c r="A162" s="1" t="n">
         <v>43586</v>
       </c>
       <c r="B162" t="n">
@@ -6613,7 +6601,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
+      <c r="A163" s="1" t="n">
         <v>43617</v>
       </c>
       <c r="B163" t="n">
@@ -6651,7 +6639,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
+      <c r="A164" s="1" t="n">
         <v>43647</v>
       </c>
       <c r="B164" t="n">
@@ -6689,7 +6677,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n">
+      <c r="A165" s="1" t="n">
         <v>43678</v>
       </c>
       <c r="B165" t="n">
@@ -6727,7 +6715,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n">
+      <c r="A166" s="1" t="n">
         <v>43709</v>
       </c>
       <c r="B166" t="n">
@@ -6765,7 +6753,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
+      <c r="A167" s="1" t="n">
         <v>43739</v>
       </c>
       <c r="B167" t="n">
@@ -6803,7 +6791,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
+      <c r="A168" s="1" t="n">
         <v>43770</v>
       </c>
       <c r="B168" t="n">
@@ -6841,7 +6829,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
+      <c r="A169" s="1" t="n">
         <v>43800</v>
       </c>
       <c r="B169" t="n">
@@ -6879,7 +6867,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n">
+      <c r="A170" s="1" t="n">
         <v>43831</v>
       </c>
       <c r="B170" t="n">
@@ -6917,7 +6905,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
+      <c r="A171" s="1" t="n">
         <v>43862</v>
       </c>
       <c r="B171" t="n">
@@ -6955,7 +6943,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n">
+      <c r="A172" s="1" t="n">
         <v>43891</v>
       </c>
       <c r="B172" t="n">
@@ -6993,7 +6981,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n">
+      <c r="A173" s="1" t="n">
         <v>43922</v>
       </c>
       <c r="B173" t="n">
@@ -7031,7 +7019,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
+      <c r="A174" s="1" t="n">
         <v>43952</v>
       </c>
       <c r="B174" t="n">
@@ -7069,7 +7057,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
+      <c r="A175" s="1" t="n">
         <v>43983</v>
       </c>
       <c r="B175" t="n">
@@ -7107,7 +7095,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
+      <c r="A176" s="1" t="n">
         <v>44013</v>
       </c>
       <c r="B176" t="n">
@@ -7145,7 +7133,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
+      <c r="A177" s="1" t="n">
         <v>44044</v>
       </c>
       <c r="B177" t="n">
@@ -7183,7 +7171,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
+      <c r="A178" s="1" t="n">
         <v>44075</v>
       </c>
       <c r="B178" t="n">
@@ -7221,7 +7209,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n">
+      <c r="A179" s="1" t="n">
         <v>44105</v>
       </c>
       <c r="B179" t="n">
@@ -7259,7 +7247,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n">
+      <c r="A180" s="1" t="n">
         <v>44136</v>
       </c>
       <c r="B180" t="n">
@@ -7297,7 +7285,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
+      <c r="A181" s="1" t="n">
         <v>44166</v>
       </c>
       <c r="B181" t="n">
@@ -7335,7 +7323,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
+      <c r="A182" s="1" t="n">
         <v>44197</v>
       </c>
       <c r="B182" t="n">
@@ -7373,7 +7361,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
+      <c r="A183" s="1" t="n">
         <v>44228</v>
       </c>
       <c r="B183" t="n">
@@ -7411,7 +7399,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n">
+      <c r="A184" s="1" t="n">
         <v>44256</v>
       </c>
       <c r="B184" t="n">
@@ -7449,7 +7437,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n">
+      <c r="A185" s="1" t="n">
         <v>44287</v>
       </c>
       <c r="B185" t="n">
@@ -7487,7 +7475,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n">
+      <c r="A186" s="1" t="n">
         <v>44317</v>
       </c>
       <c r="B186" t="n">
@@ -7525,7 +7513,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n">
+      <c r="A187" s="1" t="n">
         <v>44348</v>
       </c>
       <c r="B187" t="n">
@@ -7563,7 +7551,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n">
+      <c r="A188" s="1" t="n">
         <v>44378</v>
       </c>
       <c r="B188" t="n">
@@ -7601,7 +7589,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n">
+      <c r="A189" s="1" t="n">
         <v>44409</v>
       </c>
       <c r="B189" t="n">
@@ -7639,7 +7627,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n">
+      <c r="A190" s="1" t="n">
         <v>44440</v>
       </c>
       <c r="B190" t="n">
@@ -7677,7 +7665,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="n">
+      <c r="A191" s="1" t="n">
         <v>44470</v>
       </c>
       <c r="B191" t="n">
@@ -7715,7 +7703,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n">
+      <c r="A192" s="1" t="n">
         <v>44501</v>
       </c>
       <c r="B192" t="n">
@@ -7753,7 +7741,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="n">
+      <c r="A193" s="1" t="n">
         <v>44531</v>
       </c>
       <c r="B193" t="n">
@@ -7791,7 +7779,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="n">
+      <c r="A194" s="1" t="n">
         <v>44562</v>
       </c>
       <c r="B194" t="n">
@@ -7829,7 +7817,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="n">
+      <c r="A195" s="1" t="n">
         <v>44593</v>
       </c>
       <c r="B195" t="n">
@@ -7867,7 +7855,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="n">
+      <c r="A196" s="1" t="n">
         <v>44621</v>
       </c>
       <c r="B196" t="n">
@@ -7905,7 +7893,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="n">
+      <c r="A197" s="1" t="n">
         <v>44652</v>
       </c>
       <c r="B197" t="n">
@@ -7943,7 +7931,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n">
+      <c r="A198" s="1" t="n">
         <v>44682</v>
       </c>
       <c r="B198" t="n">
@@ -7981,7 +7969,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="n">
+      <c r="A199" s="1" t="n">
         <v>44713</v>
       </c>
       <c r="B199" t="n">
@@ -8019,7 +8007,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n">
+      <c r="A200" s="1" t="n">
         <v>44743</v>
       </c>
       <c r="B200" t="n">
@@ -8057,7 +8045,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="n">
+      <c r="A201" s="1" t="n">
         <v>44774</v>
       </c>
       <c r="B201" t="n">
@@ -8095,7 +8083,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="n">
+      <c r="A202" s="1" t="n">
         <v>44805</v>
       </c>
       <c r="B202" t="n">
@@ -8133,7 +8121,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="n">
+      <c r="A203" s="1" t="n">
         <v>44835</v>
       </c>
       <c r="B203" t="n">
@@ -8171,7 +8159,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="n">
+      <c r="A204" s="1" t="n">
         <v>44866</v>
       </c>
       <c r="B204" t="n">
@@ -8209,7 +8197,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="n">
+      <c r="A205" s="1" t="n">
         <v>44896</v>
       </c>
       <c r="B205" t="n">
@@ -8247,7 +8235,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="n">
+      <c r="A206" s="1" t="n">
         <v>44927</v>
       </c>
       <c r="B206" t="n">
@@ -8285,7 +8273,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="n">
+      <c r="A207" s="1" t="n">
         <v>44958</v>
       </c>
       <c r="B207" t="n">
@@ -8323,7 +8311,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="n">
+      <c r="A208" s="1" t="n">
         <v>44986</v>
       </c>
       <c r="B208" t="n">
@@ -8361,7 +8349,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="n">
+      <c r="A209" s="1" t="n">
         <v>45017</v>
       </c>
       <c r="B209" t="n">
@@ -8399,7 +8387,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n">
+      <c r="A210" s="1" t="n">
         <v>45047</v>
       </c>
       <c r="B210" t="n">
@@ -8437,7 +8425,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="2" t="n">
+      <c r="A211" s="1" t="n">
         <v>45078</v>
       </c>
       <c r="B211" t="n">
@@ -8475,7 +8463,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="n">
+      <c r="A212" s="1" t="n">
         <v>45108</v>
       </c>
       <c r="B212" t="n">
@@ -8513,7 +8501,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="n">
+      <c r="A213" s="1" t="n">
         <v>45139</v>
       </c>
       <c r="B213" t="n">
@@ -8551,7 +8539,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="n">
+      <c r="A214" s="1" t="n">
         <v>45170</v>
       </c>
       <c r="B214" t="n">
@@ -8589,7 +8577,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="2" t="n">
+      <c r="A215" s="1" t="n">
         <v>45200</v>
       </c>
       <c r="B215" t="n">
@@ -8627,7 +8615,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="2" t="n">
+      <c r="A216" s="1" t="n">
         <v>45231</v>
       </c>
       <c r="B216" t="n">
@@ -8665,7 +8653,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="n">
+      <c r="A217" s="1" t="n">
         <v>45261</v>
       </c>
       <c r="B217" t="n">
@@ -8703,7 +8691,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="n">
+      <c r="A218" s="1" t="n">
         <v>45292</v>
       </c>
       <c r="B218" t="n">
@@ -8741,7 +8729,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="n">
+      <c r="A219" s="1" t="n">
         <v>45323</v>
       </c>
       <c r="B219" t="n">
@@ -8779,7 +8767,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="n">
+      <c r="A220" s="1" t="n">
         <v>45352</v>
       </c>
       <c r="B220" t="n">
@@ -8817,7 +8805,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="n">
+      <c r="A221" s="1" t="n">
         <v>45383</v>
       </c>
       <c r="B221" t="n">
@@ -8855,7 +8843,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="n">
+      <c r="A222" s="1" t="n">
         <v>45413</v>
       </c>
       <c r="B222" t="n">
@@ -8893,7 +8881,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="n">
+      <c r="A223" s="1" t="n">
         <v>45444</v>
       </c>
       <c r="B223" t="n">
@@ -8931,7 +8919,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="n">
+      <c r="A224" s="1" t="n">
         <v>45474</v>
       </c>
       <c r="B224" t="n">
@@ -8969,7 +8957,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="n">
+      <c r="A225" s="1" t="n">
         <v>45505</v>
       </c>
       <c r="B225" t="n">
@@ -9007,7 +8995,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="n">
+      <c r="A226" s="1" t="n">
         <v>45536</v>
       </c>
       <c r="B226" t="n">
@@ -9045,7 +9033,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="n">
+      <c r="A227" s="1" t="n">
         <v>45566</v>
       </c>
       <c r="B227" t="n">
@@ -9083,7 +9071,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="n">
+      <c r="A228" s="1" t="n">
         <v>45597</v>
       </c>
       <c r="B228" t="n">
@@ -9121,7 +9109,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="n">
+      <c r="A229" s="1" t="n">
         <v>45627</v>
       </c>
       <c r="B229" t="n">
@@ -9159,7 +9147,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="n">
+      <c r="A230" s="1" t="n">
         <v>45658</v>
       </c>
       <c r="B230" t="n">
@@ -9197,7 +9185,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="n">
+      <c r="A231" s="1" t="n">
         <v>45689</v>
       </c>
       <c r="B231" t="n">
@@ -9235,7 +9223,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="n">
+      <c r="A232" s="1" t="n">
         <v>45717</v>
       </c>
       <c r="B232" t="n">
@@ -9273,7 +9261,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="n">
+      <c r="A233" s="1" t="n">
         <v>45748</v>
       </c>
       <c r="B233" t="n">
@@ -9311,7 +9299,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="n">
+      <c r="A234" s="1" t="n">
         <v>45778</v>
       </c>
       <c r="B234" t="n">
@@ -9349,7 +9337,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="n">
+      <c r="A235" s="1" t="n">
         <v>45809</v>
       </c>
       <c r="B235" t="n">
@@ -9387,7 +9375,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="2" t="n">
+      <c r="A236" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="B236" t="n">
@@ -9425,7 +9413,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="2" t="n">
+      <c r="A237" s="1" t="n">
         <v>45870</v>
       </c>
       <c r="B237" t="n">
@@ -9463,7 +9451,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="2" t="n">
+      <c r="A238" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="B238" t="n">
@@ -9501,7 +9489,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="2" t="n">
+      <c r="A239" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="B239" t="n">
@@ -9539,7 +9527,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="2" t="n">
+      <c r="A240" s="1" t="n">
         <v>45962</v>
       </c>
       <c r="B240" t="n">
@@ -9577,7 +9565,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="2" t="n">
+      <c r="A241" s="1" t="n">
         <v>45992</v>
       </c>
       <c r="B241" t="n">
@@ -9615,7 +9603,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="2" t="n">
+      <c r="A242" s="1" t="n">
         <v>46023</v>
       </c>
       <c r="B242" t="n">
@@ -9653,7 +9641,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="n">
+      <c r="A243" s="1" t="n">
         <v>46054</v>
       </c>
       <c r="B243" t="n">
@@ -9691,7 +9679,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="2" t="n">
+      <c r="A244" s="1" t="n">
         <v>46082</v>
       </c>
       <c r="B244" t="n">
@@ -9729,7 +9717,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="2" t="n">
+      <c r="A245" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="B245" t="n">
@@ -9767,7 +9755,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="2" t="n">
+      <c r="A246" s="1" t="n">
         <v>46143</v>
       </c>
       <c r="B246" t="n">
@@ -9805,7 +9793,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="2" t="n">
+      <c r="A247" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="B247" t="n">
@@ -9843,7 +9831,7 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="2" t="n">
+      <c r="A248" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="B248" t="n">

</xml_diff>